<commit_message>
Ensemble experiment: 5 seeds of band_g_mix, averaged (1.06g) vs single seed 0 (1.12g); seed variance dominates
</commit_message>
<xml_diff>
--- a/results/LSTM_ABS_RESULTS.xlsx
+++ b/results/LSTM_ABS_RESULTS.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -508,22 +508,22 @@
         <v>60</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3" t="n">
-        <v>1.149</v>
+        <v>1.14</v>
       </c>
       <c r="E3" t="n">
-        <v>1.1286</v>
+        <v>1.1067</v>
       </c>
       <c r="F3" t="n">
         <v>1.16</v>
       </c>
       <c r="G3" t="n">
-        <v>31.8734</v>
+        <v>32.1309</v>
       </c>
       <c r="H3" t="n">
-        <v>2.6</v>
+        <v>2.85</v>
       </c>
     </row>
     <row r="4">
@@ -613,7 +613,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>band_g_dyn</t>
+          <t>ens_band_g_mix5</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -623,25 +623,25 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>1.0636</v>
+        <v>1.0637</v>
       </c>
       <c r="E7" t="n">
-        <v>1.0628</v>
+        <v>1.0538</v>
       </c>
       <c r="F7" t="n">
-        <v>1.0644</v>
+        <v>1.0736</v>
       </c>
       <c r="G7" t="n">
-        <v>34.4297</v>
+        <v>34.428</v>
       </c>
       <c r="H7" t="n">
-        <v>4.15</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>band_gy_dyn</t>
+          <t>band_g_dyn</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -651,25 +651,25 @@
         <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>1.0506</v>
+        <v>1.0636</v>
       </c>
       <c r="E8" t="n">
-        <v>1.0459</v>
+        <v>1.0628</v>
       </c>
       <c r="F8" t="n">
-        <v>1.0554</v>
+        <v>1.0644</v>
       </c>
       <c r="G8" t="n">
-        <v>34.8533</v>
+        <v>34.4297</v>
       </c>
       <c r="H8" t="n">
-        <v>2.6</v>
+        <v>4.15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>avg_g_window_hg</t>
+          <t>band_gy_dyn</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -679,53 +679,53 @@
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>1.0301</v>
+        <v>1.0506</v>
       </c>
       <c r="E9" t="n">
-        <v>1.0294</v>
+        <v>1.0459</v>
       </c>
       <c r="F9" t="n">
-        <v>1.0308</v>
+        <v>1.0554</v>
       </c>
       <c r="G9" t="n">
-        <v>35.5482</v>
+        <v>34.8533</v>
       </c>
       <c r="H9" t="n">
-        <v>2.55</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>band_g_mix_s1</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>60</v>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>1.0292</v>
+        <v>1.0432</v>
       </c>
       <c r="E10" t="n">
-        <v>1.0039</v>
+        <v>1.0376</v>
       </c>
       <c r="F10" t="n">
-        <v>1.066</v>
+        <v>1.0488</v>
       </c>
       <c r="G10" t="n">
-        <v>35.6013</v>
+        <v>35.1022</v>
       </c>
       <c r="H10" t="n">
-        <v>0.8</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>avg_g_window_stock</t>
+          <t>avg_g_window_hg</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -735,299 +735,299 @@
         <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>1.029</v>
+        <v>1.0301</v>
       </c>
       <c r="E11" t="n">
-        <v>1.026</v>
+        <v>1.0294</v>
       </c>
       <c r="F11" t="n">
-        <v>1.0319</v>
+        <v>1.0308</v>
       </c>
       <c r="G11" t="n">
-        <v>35.5875</v>
-      </c>
-      <c r="H11" t="inlineStr"/>
+        <v>35.5482</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2.55</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>baseline_hg</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>60</v>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>1.0162</v>
+        <v>1.0292</v>
       </c>
       <c r="E12" t="n">
-        <v>1.0147</v>
+        <v>1.0039</v>
       </c>
       <c r="F12" t="n">
-        <v>1.0177</v>
+        <v>1.066</v>
       </c>
       <c r="G12" t="n">
-        <v>36.0347</v>
+        <v>35.6013</v>
       </c>
       <c r="H12" t="n">
-        <v>3</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>baseline FORCE_CMD=1.0</t>
+          <t>avg_g_window_stock</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>60</v>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>1.0017</v>
+        <v>1.029</v>
       </c>
       <c r="E13" t="n">
-        <v>1.0017</v>
+        <v>1.026</v>
       </c>
       <c r="F13" t="n">
-        <v>1.0017</v>
+        <v>1.0319</v>
       </c>
       <c r="G13" t="n">
-        <v>36.5572</v>
-      </c>
-      <c r="H13" t="n">
-        <v>3.5</v>
-      </c>
+        <v>35.5875</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>baseline_stocknorpm</t>
+          <t>baseline_hg</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>60</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.0162</v>
       </c>
       <c r="E14" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.0147</v>
       </c>
       <c r="F14" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.0177</v>
       </c>
       <c r="G14" t="n">
-        <v>37.0845</v>
+        <v>36.0347</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>baseline_stock</t>
+          <t>baseline FORCE_CMD=1.0</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>60</v>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8937</v>
+        <v>1.0017</v>
       </c>
       <c r="E15" t="n">
-        <v>0.8933</v>
+        <v>1.0017</v>
       </c>
       <c r="F15" t="n">
-        <v>0.8942</v>
+        <v>1.0017</v>
       </c>
       <c r="G15" t="n">
-        <v>40.9724</v>
+        <v>36.5572</v>
       </c>
       <c r="H15" t="n">
-        <v>3.5667</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>curation_hg</t>
+          <t>baseline_stocknorpm</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>60</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>0.8874</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="E16" t="n">
-        <v>0.8813</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="F16" t="n">
-        <v>0.8935</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>41.266</v>
-      </c>
-      <c r="H16" t="inlineStr"/>
+        <v>37.0845</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs2</t>
+          <t>baseline_stock</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>60</v>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>0.8228</v>
+        <v>0.8937</v>
       </c>
       <c r="E17" t="n">
-        <v>0.8045</v>
+        <v>0.8933</v>
       </c>
       <c r="F17" t="n">
-        <v>0.8411</v>
+        <v>0.8942</v>
       </c>
       <c r="G17" t="n">
-        <v>44.527</v>
+        <v>40.9724</v>
       </c>
       <c r="H17" t="n">
-        <v>1.9</v>
+        <v>3.5667</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>baseline_stock16</t>
+          <t>curation_hg</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>60</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>0.7467</v>
+        <v>0.8874</v>
       </c>
       <c r="E18" t="n">
-        <v>0.7467</v>
+        <v>0.8813</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7467</v>
+        <v>0.8935</v>
       </c>
       <c r="G18" t="n">
-        <v>49.0416</v>
+        <v>41.266</v>
       </c>
       <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>baseline_dynstocknoabs2</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>60</v>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>0.4106</v>
+        <v>0.8228</v>
       </c>
       <c r="E19" t="n">
-        <v>0.2278</v>
+        <v>0.8045</v>
       </c>
       <c r="F19" t="n">
-        <v>0.7759</v>
+        <v>0.8411</v>
       </c>
       <c r="G19" t="n">
-        <v>122.7889</v>
+        <v>44.527</v>
       </c>
       <c r="H19" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>baseline_dynnoimu</t>
+          <t>baseline_stock16</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>60</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>0.3672</v>
+        <v>0.7467</v>
       </c>
       <c r="E20" t="n">
-        <v>0.3661</v>
+        <v>0.7467</v>
       </c>
       <c r="F20" t="n">
-        <v>0.3683</v>
+        <v>0.7467</v>
       </c>
       <c r="G20" t="n">
-        <v>99.72539999999999</v>
-      </c>
-      <c r="H20" t="n">
-        <v>4.6</v>
-      </c>
+        <v>49.0416</v>
+      </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>baseline_dynstock2</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>60</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>0.2488</v>
+        <v>0.4106</v>
       </c>
       <c r="E21" t="n">
-        <v>0.2481</v>
+        <v>0.2278</v>
       </c>
       <c r="F21" t="n">
-        <v>0.2496</v>
+        <v>0.7759</v>
       </c>
       <c r="G21" t="n">
-        <v>147.1485</v>
+        <v>122.7889</v>
       </c>
       <c r="H21" t="n">
-        <v>2.8</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>baseline_dynnoimu</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1037,51 +1037,53 @@
         <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>0.2302</v>
+        <v>0.3672</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2295</v>
+        <v>0.3661</v>
       </c>
       <c r="F22" t="n">
-        <v>0.2309</v>
+        <v>0.3683</v>
       </c>
       <c r="G22" t="n">
-        <v>159.0684</v>
-      </c>
-      <c r="H22" t="inlineStr"/>
+        <v>99.72539999999999</v>
+      </c>
+      <c r="H22" t="n">
+        <v>4.6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>avg_g_window</t>
+          <t>baseline_dynstock2</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>60</v>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>0.2283</v>
+        <v>0.2488</v>
       </c>
       <c r="E23" t="n">
-        <v>0.2276</v>
+        <v>0.2481</v>
       </c>
       <c r="F23" t="n">
-        <v>0.2291</v>
+        <v>0.2496</v>
       </c>
       <c r="G23" t="n">
-        <v>160.3908</v>
+        <v>147.1485</v>
       </c>
       <c r="H23" t="n">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>peak_g</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1091,49 +1093,51 @@
         <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>0.2258</v>
+        <v>0.2302</v>
       </c>
       <c r="E24" t="n">
-        <v>0.2252</v>
+        <v>0.2295</v>
       </c>
       <c r="F24" t="n">
-        <v>0.2263</v>
+        <v>0.2309</v>
       </c>
       <c r="G24" t="n">
-        <v>162.2099</v>
+        <v>159.0684</v>
       </c>
       <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>peak_g_norpm</t>
+          <t>avg_g_window</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>60</v>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D25" t="n">
-        <v>0.2245</v>
+        <v>0.2283</v>
       </c>
       <c r="E25" t="n">
-        <v>0.2238</v>
+        <v>0.2276</v>
       </c>
       <c r="F25" t="n">
-        <v>0.2252</v>
+        <v>0.2291</v>
       </c>
       <c r="G25" t="n">
-        <v>163.1152</v>
-      </c>
-      <c r="H25" t="inlineStr"/>
+        <v>160.3908</v>
+      </c>
+      <c r="H25" t="n">
+        <v>3.2</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>baseline_dynstock</t>
+          <t>yaw_intent</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1143,25 +1147,23 @@
         <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>0.2241</v>
+        <v>0.2258</v>
       </c>
       <c r="E26" t="n">
-        <v>0.2235</v>
+        <v>0.2252</v>
       </c>
       <c r="F26" t="n">
-        <v>0.2247</v>
+        <v>0.2263</v>
       </c>
       <c r="G26" t="n">
-        <v>163.3969</v>
-      </c>
-      <c r="H26" t="n">
-        <v>3.05</v>
-      </c>
+        <v>162.2099</v>
+      </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs</t>
+          <t>peak_g_norpm</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1171,79 +1173,79 @@
         <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>0.1982</v>
+        <v>0.2245</v>
       </c>
       <c r="E27" t="n">
-        <v>0.198</v>
+        <v>0.2238</v>
       </c>
       <c r="F27" t="n">
-        <v>0.1985</v>
+        <v>0.2252</v>
       </c>
       <c r="G27" t="n">
-        <v>184.7105</v>
-      </c>
-      <c r="H27" t="n">
-        <v>3.75</v>
-      </c>
+        <v>163.1152</v>
+      </c>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>avg_g_window_hg</t>
+          <t>baseline_dynstock</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" t="n">
-        <v>1.0148</v>
+        <v>0.2241</v>
       </c>
       <c r="E28" t="n">
-        <v>1.0148</v>
+        <v>0.2235</v>
       </c>
       <c r="F28" t="n">
-        <v>1.0148</v>
+        <v>0.2247</v>
       </c>
       <c r="G28" t="n">
-        <v>64.18680000000001</v>
+        <v>163.3969</v>
       </c>
       <c r="H28" t="n">
-        <v>3.8</v>
+        <v>3.05</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>baseline_dynstocknoabs</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C29" t="n">
         <v>2</v>
       </c>
       <c r="D29" t="n">
-        <v>1.011</v>
+        <v>0.1982</v>
       </c>
       <c r="E29" t="n">
-        <v>1.0062</v>
+        <v>0.198</v>
       </c>
       <c r="F29" t="n">
-        <v>1.0158</v>
+        <v>0.1985</v>
       </c>
       <c r="G29" t="n">
-        <v>50.3918</v>
-      </c>
-      <c r="H29" t="inlineStr"/>
+        <v>184.7105</v>
+      </c>
+      <c r="H29" t="n">
+        <v>3.75</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>avg_g_window_hg</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1253,101 +1255,103 @@
         <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>0.9869</v>
+        <v>1.0148</v>
       </c>
       <c r="E30" t="n">
-        <v>0.9869</v>
+        <v>1.0148</v>
       </c>
       <c r="F30" t="n">
-        <v>0.9869</v>
+        <v>1.0148</v>
       </c>
       <c r="G30" t="n">
-        <v>66.0052</v>
-      </c>
-      <c r="H30" t="inlineStr"/>
+        <v>64.18680000000001</v>
+      </c>
+      <c r="H30" t="n">
+        <v>3.8</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>combined</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>80</v>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" t="n">
-        <v>0.2276</v>
+        <v>1.011</v>
       </c>
       <c r="E31" t="n">
-        <v>0.2276</v>
+        <v>1.0062</v>
       </c>
       <c r="F31" t="n">
-        <v>0.2276</v>
+        <v>1.0158</v>
       </c>
       <c r="G31" t="n">
-        <v>160.9226</v>
+        <v>50.3918</v>
       </c>
       <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>80</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D32" t="n">
-        <v>0.2159</v>
+        <v>0.9869</v>
       </c>
       <c r="E32" t="n">
-        <v>0.2156</v>
+        <v>0.9869</v>
       </c>
       <c r="F32" t="n">
-        <v>0.2162</v>
+        <v>0.9869</v>
       </c>
       <c r="G32" t="n">
-        <v>301.7328</v>
+        <v>66.0052</v>
       </c>
       <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>combined</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>80</v>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>0.1782</v>
+        <v>0.2276</v>
       </c>
       <c r="E33" t="n">
-        <v>0.1779</v>
+        <v>0.2276</v>
       </c>
       <c r="F33" t="n">
-        <v>0.1784</v>
+        <v>0.2276</v>
       </c>
       <c r="G33" t="n">
-        <v>365.637</v>
+        <v>160.9226</v>
       </c>
       <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>avg_g_window</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1357,23 +1361,23 @@
         <v>2</v>
       </c>
       <c r="D34" t="n">
-        <v>0.1778</v>
+        <v>0.2159</v>
       </c>
       <c r="E34" t="n">
-        <v>0.1776</v>
+        <v>0.2156</v>
       </c>
       <c r="F34" t="n">
-        <v>0.178</v>
+        <v>0.2162</v>
       </c>
       <c r="G34" t="n">
-        <v>366.3356</v>
+        <v>301.7328</v>
       </c>
       <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>peak_g</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1383,18 +1387,70 @@
         <v>2</v>
       </c>
       <c r="D35" t="n">
+        <v>0.1782</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.1779</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.1784</v>
+      </c>
+      <c r="G35" t="n">
+        <v>365.637</v>
+      </c>
+      <c r="H35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>avg_g_window</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>80</v>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.1778</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.1776</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="G36" t="n">
+        <v>366.3356</v>
+      </c>
+      <c r="H36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>yaw_intent</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>80</v>
+      </c>
+      <c r="C37" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" t="n">
         <v>0.1766</v>
       </c>
-      <c r="E35" t="n">
+      <c r="E37" t="n">
         <v>0.1766</v>
       </c>
-      <c r="F35" t="n">
+      <c r="F37" t="n">
         <v>0.1766</v>
       </c>
-      <c r="G35" t="n">
+      <c r="G37" t="n">
         <v>368.9042</v>
       </c>
-      <c r="H35" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1407,7 +1463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4120,36 +4176,316 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
+          <t>ctrl_v2</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>band_g_mix</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>60</v>
+      </c>
+      <c r="E76" t="n">
+        <v>1.1546</v>
+      </c>
+      <c r="F76" t="n">
+        <v>31.7152</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>1788400580-0001</t>
+        </is>
+      </c>
+      <c r="H76" t="n">
+        <v>31.72</v>
+      </c>
+      <c r="I76" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="J76" t="n">
+        <v>2.29</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>band_g_mix</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>60</v>
+      </c>
+      <c r="E77" t="n">
+        <v>1.1316</v>
+      </c>
+      <c r="F77" t="n">
+        <v>32.361</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>1788400999-0003</t>
+        </is>
+      </c>
+      <c r="H77" t="n">
+        <v>32.36</v>
+      </c>
+      <c r="I77" t="n">
+        <v>4</v>
+      </c>
+      <c r="J77" t="n">
+        <v>2.33</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>band_g_mix</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>60</v>
+      </c>
+      <c r="E78" t="n">
+        <v>1.1067</v>
+      </c>
+      <c r="F78" t="n">
+        <v>33.0891</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>1788401032-0004</t>
+        </is>
+      </c>
+      <c r="H78" t="n">
+        <v>33.09</v>
+      </c>
+      <c r="I78" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J78" t="n">
+        <v>2.37</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>band_g_mix_s1</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>60</v>
+      </c>
+      <c r="E79" t="n">
+        <v>1.0488</v>
+      </c>
+      <c r="F79" t="n">
+        <v>34.9145</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>1788401068-0005</t>
+        </is>
+      </c>
+      <c r="H79" t="n">
+        <v>34.91</v>
+      </c>
+      <c r="I79" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J79" t="n">
+        <v>2.48</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>band_g_mix_s1</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>60</v>
+      </c>
+      <c r="E80" t="n">
+        <v>1.0376</v>
+      </c>
+      <c r="F80" t="n">
+        <v>35.29</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>1788401101-0006</t>
+        </is>
+      </c>
+      <c r="H80" t="n">
+        <v>35.29</v>
+      </c>
+      <c r="I80" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J80" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
           <t>restructure</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>baseline_dyn</t>
         </is>
       </c>
-      <c r="D76" t="n">
-        <v>60</v>
-      </c>
-      <c r="E76" t="n">
+      <c r="D81" t="n">
+        <v>60</v>
+      </c>
+      <c r="E81" t="n">
         <v>1.1085</v>
       </c>
-      <c r="F76" t="n">
+      <c r="F81" t="n">
         <v>33.0351</v>
       </c>
-      <c r="G76" t="inlineStr">
+      <c r="G81" t="inlineStr">
         <is>
           <t>1788399311-0002</t>
         </is>
       </c>
-      <c r="H76" t="n">
+      <c r="H81" t="n">
         <v>33.04</v>
       </c>
-      <c r="I76" t="n">
+      <c r="I81" t="n">
         <v>4.8</v>
       </c>
-      <c r="J76" t="n">
+      <c r="J81" t="n">
         <v>2.4</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>ens_band_g_mix5</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>60</v>
+      </c>
+      <c r="E82" t="n">
+        <v>1.0736</v>
+      </c>
+      <c r="F82" t="n">
+        <v>34.1079</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>1788400929-0001</t>
+        </is>
+      </c>
+      <c r="H82" t="n">
+        <v>34.11</v>
+      </c>
+      <c r="I82" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J82" t="n">
+        <v>2.44</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>ens_band_g_mix5</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>60</v>
+      </c>
+      <c r="E83" t="n">
+        <v>1.0538</v>
+      </c>
+      <c r="F83" t="n">
+        <v>34.7482</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>1788400962-0002</t>
+        </is>
+      </c>
+      <c r="H83" t="n">
+        <v>34.75</v>
+      </c>
+      <c r="I83" t="n">
+        <v>2</v>
+      </c>
+      <c r="J83" t="n">
+        <v>2.48</v>
       </c>
     </row>
   </sheetData>
@@ -4163,22 +4499,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
     <col width="48" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -4274,7 +4610,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
@@ -4298,7 +4634,7 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
@@ -4322,7 +4658,7 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
@@ -4346,7 +4682,7 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
@@ -4370,134 +4706,294 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>band_gy_dyn</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
+          <t>band_g_mix_s1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:54:00</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
-        </is>
-      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>[0.14226, 0.15404, 0.16814, 0.16762]</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>band_gy_mix</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
+          <t>band_g_mix_s2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:55:36</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>[0.15115, 0.15324, 0.16928, 0.16978]</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>baseline</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
+          <t>band_g_mix_s3</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:57:18</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
-        </is>
-      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>[0.15575, 0.16054, 0.1713, 0.17144]</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+          <t>band_g_mix_s4</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:58:55</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
-        </is>
-      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>[0.14723, 0.15025, 0.16854, 0.16772]</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>baseline_dynnoimu</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+          <t>band_g_mix_s5</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-09-02T19:00:42</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>5</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>[0.14491, 0.15532, 0.16904, 0.16805]</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>baseline_dynstock2</t>
+          <t>band_gy_dyn</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -4514,14 +5010,14 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>baseline_dynstock</t>
+          <t>band_gy_mix</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -4538,14 +5034,14 @@
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs2</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -4562,14 +5058,14 @@
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs</t>
+          <t>baseline_dyn</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -4586,14 +5082,14 @@
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>baseline_hg</t>
+          <t>baseline_dynnoimu</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -4610,14 +5106,14 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>baseline_norpm</t>
+          <t>baseline_dynstock2</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -4634,14 +5130,14 @@
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>baseline_stock16</t>
+          <t>baseline_dynstock</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -4658,14 +5154,14 @@
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>baseline_dynstocknoabs2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -4682,14 +5178,14 @@
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>baseline_stock</t>
+          <t>baseline_dynstocknoabs</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -4706,14 +5202,14 @@
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>baseline_stocknorpm</t>
+          <t>baseline_hg</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -4730,14 +5226,14 @@
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>combined</t>
+          <t>baseline_norpm</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -4754,14 +5250,14 @@
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>baseline_stock16</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -4778,14 +5274,14 @@
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>curation_hg</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -4802,14 +5298,14 @@
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>baseline_stock</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -4826,14 +5322,14 @@
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>peak_g_norpm</t>
+          <t>baseline_stocknorpm</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -4850,14 +5346,14 @@
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>combined</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -4874,7 +5370,127 @@
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/LSTM_ABS_HANDOFF.md</t>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>curation</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>curation_hg</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>peak_g</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>peak_g_norpm</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>yaw_intent</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Band-width/overlap sweep on seed 0: 1 to 20 mph, 1 to 3 windows per speed
</commit_message>
<xml_diff>
--- a/results/LSTM_ABS_RESULTS.xlsx
+++ b/results/LSTM_ABS_RESULTS.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -585,35 +585,35 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>band_g_mix_b1o1</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>60</v>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>1.0671</v>
+        <v>1.1018</v>
       </c>
       <c r="E6" t="n">
-        <v>1.0582</v>
+        <v>1.0902</v>
       </c>
       <c r="F6" t="n">
-        <v>1.0716</v>
+        <v>1.1133</v>
       </c>
       <c r="G6" t="n">
-        <v>34.3171</v>
+        <v>33.2398</v>
       </c>
       <c r="H6" t="n">
-        <v>2.3667</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ens_band_g_mix5</t>
+          <t>band_g_mix_b2p5o2</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -623,53 +623,53 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>1.0637</v>
+        <v>1.0884</v>
       </c>
       <c r="E7" t="n">
-        <v>1.0538</v>
+        <v>1.0823</v>
       </c>
       <c r="F7" t="n">
-        <v>1.0736</v>
+        <v>1.0944</v>
       </c>
       <c r="G7" t="n">
-        <v>34.428</v>
+        <v>33.6464</v>
       </c>
       <c r="H7" t="n">
-        <v>2.2</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>band_g_dyn</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>60</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>1.0636</v>
+        <v>1.0671</v>
       </c>
       <c r="E8" t="n">
-        <v>1.0628</v>
+        <v>1.0582</v>
       </c>
       <c r="F8" t="n">
-        <v>1.0644</v>
+        <v>1.0716</v>
       </c>
       <c r="G8" t="n">
-        <v>34.4297</v>
+        <v>34.3171</v>
       </c>
       <c r="H8" t="n">
-        <v>4.15</v>
+        <v>2.3667</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>band_gy_dyn</t>
+          <t>ens_band_g_mix5</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -679,25 +679,25 @@
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>1.0506</v>
+        <v>1.0637</v>
       </c>
       <c r="E9" t="n">
-        <v>1.0459</v>
+        <v>1.0538</v>
       </c>
       <c r="F9" t="n">
-        <v>1.0554</v>
+        <v>1.0736</v>
       </c>
       <c r="G9" t="n">
-        <v>34.8533</v>
+        <v>34.428</v>
       </c>
       <c r="H9" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_dyn</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -707,25 +707,25 @@
         <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>1.0432</v>
+        <v>1.0636</v>
       </c>
       <c r="E10" t="n">
-        <v>1.0376</v>
+        <v>1.0628</v>
       </c>
       <c r="F10" t="n">
-        <v>1.0488</v>
+        <v>1.0644</v>
       </c>
       <c r="G10" t="n">
-        <v>35.1022</v>
+        <v>34.4297</v>
       </c>
       <c r="H10" t="n">
-        <v>2.9</v>
+        <v>4.15</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>avg_g_window_hg</t>
+          <t>band_g_mix_b7p5o3</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -735,53 +735,53 @@
         <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>1.0301</v>
+        <v>1.061</v>
       </c>
       <c r="E11" t="n">
-        <v>1.0294</v>
+        <v>1.048</v>
       </c>
       <c r="F11" t="n">
-        <v>1.0308</v>
+        <v>1.0741</v>
       </c>
       <c r="G11" t="n">
-        <v>35.5482</v>
+        <v>34.5166</v>
       </c>
       <c r="H11" t="n">
-        <v>2.55</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>band_g_mix_b10o1</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>60</v>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>1.0292</v>
+        <v>1.0608</v>
       </c>
       <c r="E12" t="n">
-        <v>1.0039</v>
+        <v>1.0578</v>
       </c>
       <c r="F12" t="n">
-        <v>1.066</v>
+        <v>1.0639</v>
       </c>
       <c r="G12" t="n">
-        <v>35.6013</v>
+        <v>34.5166</v>
       </c>
       <c r="H12" t="n">
-        <v>0.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>avg_g_window_stock</t>
+          <t>band_g_mix_b5o2</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -791,23 +791,25 @@
         <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>1.029</v>
+        <v>1.0579</v>
       </c>
       <c r="E13" t="n">
-        <v>1.026</v>
+        <v>1.0546</v>
       </c>
       <c r="F13" t="n">
-        <v>1.0319</v>
+        <v>1.0612</v>
       </c>
       <c r="G13" t="n">
-        <v>35.5875</v>
-      </c>
-      <c r="H13" t="inlineStr"/>
+        <v>34.6135</v>
+      </c>
+      <c r="H13" t="n">
+        <v>4.05</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>baseline_hg</t>
+          <t>band_gy_dyn</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -817,81 +819,81 @@
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>1.0162</v>
+        <v>1.0506</v>
       </c>
       <c r="E14" t="n">
-        <v>1.0147</v>
+        <v>1.0459</v>
       </c>
       <c r="F14" t="n">
-        <v>1.0177</v>
+        <v>1.0554</v>
       </c>
       <c r="G14" t="n">
-        <v>36.0347</v>
+        <v>34.8533</v>
       </c>
       <c r="H14" t="n">
-        <v>3</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>baseline FORCE_CMD=1.0</t>
+          <t>band_g_mix_s1</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>60</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>1.0017</v>
+        <v>1.0432</v>
       </c>
       <c r="E15" t="n">
-        <v>1.0017</v>
+        <v>1.0376</v>
       </c>
       <c r="F15" t="n">
-        <v>1.0017</v>
+        <v>1.0488</v>
       </c>
       <c r="G15" t="n">
-        <v>36.5572</v>
+        <v>35.1022</v>
       </c>
       <c r="H15" t="n">
-        <v>3.5</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>baseline_stocknorpm</t>
+          <t>avg_g_window_hg</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>60</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.0301</v>
       </c>
       <c r="E16" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.0294</v>
       </c>
       <c r="F16" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.0308</v>
       </c>
       <c r="G16" t="n">
-        <v>37.0845</v>
+        <v>35.5482</v>
       </c>
       <c r="H16" t="n">
-        <v>1</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>baseline_stock</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -901,25 +903,25 @@
         <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>0.8937</v>
+        <v>1.0292</v>
       </c>
       <c r="E17" t="n">
-        <v>0.8933</v>
+        <v>1.0039</v>
       </c>
       <c r="F17" t="n">
-        <v>0.8942</v>
+        <v>1.066</v>
       </c>
       <c r="G17" t="n">
-        <v>40.9724</v>
+        <v>35.6013</v>
       </c>
       <c r="H17" t="n">
-        <v>3.5667</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>curation_hg</t>
+          <t>avg_g_window_stock</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -929,23 +931,23 @@
         <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>0.8874</v>
+        <v>1.029</v>
       </c>
       <c r="E18" t="n">
-        <v>0.8813</v>
+        <v>1.026</v>
       </c>
       <c r="F18" t="n">
-        <v>0.8935</v>
+        <v>1.0319</v>
       </c>
       <c r="G18" t="n">
-        <v>41.266</v>
+        <v>35.5875</v>
       </c>
       <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs2</t>
+          <t>baseline_hg</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -955,25 +957,25 @@
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>0.8228</v>
+        <v>1.0162</v>
       </c>
       <c r="E19" t="n">
-        <v>0.8045</v>
+        <v>1.0147</v>
       </c>
       <c r="F19" t="n">
-        <v>0.8411</v>
+        <v>1.0177</v>
       </c>
       <c r="G19" t="n">
-        <v>44.527</v>
+        <v>36.0347</v>
       </c>
       <c r="H19" t="n">
-        <v>1.9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>baseline_stock16</t>
+          <t>baseline FORCE_CMD=1.0</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -983,79 +985,81 @@
         <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>0.7467</v>
+        <v>1.0017</v>
       </c>
       <c r="E20" t="n">
-        <v>0.7467</v>
+        <v>1.0017</v>
       </c>
       <c r="F20" t="n">
-        <v>0.7467</v>
+        <v>1.0017</v>
       </c>
       <c r="G20" t="n">
-        <v>49.0416</v>
-      </c>
-      <c r="H20" t="inlineStr"/>
+        <v>36.5572</v>
+      </c>
+      <c r="H20" t="n">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>baseline_stocknorpm</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>60</v>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>0.4106</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="E21" t="n">
-        <v>0.2278</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="F21" t="n">
-        <v>0.7759</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="G21" t="n">
-        <v>122.7889</v>
+        <v>37.0845</v>
       </c>
       <c r="H21" t="n">
-        <v>2.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>baseline_dynnoimu</t>
+          <t>baseline_stock</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>60</v>
       </c>
       <c r="C22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>0.3672</v>
+        <v>0.8937</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3661</v>
+        <v>0.8933</v>
       </c>
       <c r="F22" t="n">
-        <v>0.3683</v>
+        <v>0.8942</v>
       </c>
       <c r="G22" t="n">
-        <v>99.72539999999999</v>
+        <v>40.9724</v>
       </c>
       <c r="H22" t="n">
-        <v>4.6</v>
+        <v>3.5667</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>baseline_dynstock2</t>
+          <t>curation_hg</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1065,25 +1069,23 @@
         <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>0.2488</v>
+        <v>0.8874</v>
       </c>
       <c r="E23" t="n">
-        <v>0.2481</v>
+        <v>0.8813</v>
       </c>
       <c r="F23" t="n">
-        <v>0.2496</v>
+        <v>0.8935</v>
       </c>
       <c r="G23" t="n">
-        <v>147.1485</v>
-      </c>
-      <c r="H23" t="n">
-        <v>2.8</v>
-      </c>
+        <v>41.266</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>baseline_dynstocknoabs2</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1093,51 +1095,51 @@
         <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>0.2302</v>
+        <v>0.8228</v>
       </c>
       <c r="E24" t="n">
-        <v>0.2295</v>
+        <v>0.8045</v>
       </c>
       <c r="F24" t="n">
-        <v>0.2309</v>
+        <v>0.8411</v>
       </c>
       <c r="G24" t="n">
-        <v>159.0684</v>
-      </c>
-      <c r="H24" t="inlineStr"/>
+        <v>44.527</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1.9</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>avg_g_window</t>
+          <t>baseline_stock16</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>60</v>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>0.2283</v>
+        <v>0.7467</v>
       </c>
       <c r="E25" t="n">
-        <v>0.2276</v>
+        <v>0.7467</v>
       </c>
       <c r="F25" t="n">
-        <v>0.2291</v>
+        <v>0.7467</v>
       </c>
       <c r="G25" t="n">
-        <v>160.3908</v>
-      </c>
-      <c r="H25" t="n">
-        <v>3.2</v>
-      </c>
+        <v>49.0416</v>
+      </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>band_g_mix_b20o1</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1147,49 +1149,53 @@
         <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>0.2258</v>
+        <v>0.7231</v>
       </c>
       <c r="E26" t="n">
-        <v>0.2252</v>
+        <v>0.4061</v>
       </c>
       <c r="F26" t="n">
-        <v>0.2263</v>
+        <v>1.0401</v>
       </c>
       <c r="G26" t="n">
-        <v>162.2099</v>
-      </c>
-      <c r="H26" t="inlineStr"/>
+        <v>62.6864</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1.95</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>peak_g_norpm</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>60</v>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>0.2245</v>
+        <v>0.4106</v>
       </c>
       <c r="E27" t="n">
-        <v>0.2238</v>
+        <v>0.2278</v>
       </c>
       <c r="F27" t="n">
-        <v>0.2252</v>
+        <v>0.7759</v>
       </c>
       <c r="G27" t="n">
-        <v>163.1152</v>
-      </c>
-      <c r="H27" t="inlineStr"/>
+        <v>122.7889</v>
+      </c>
+      <c r="H27" t="n">
+        <v>2.1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>baseline_dynstock</t>
+          <t>baseline_dynnoimu</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1199,25 +1205,25 @@
         <v>2</v>
       </c>
       <c r="D28" t="n">
-        <v>0.2241</v>
+        <v>0.3672</v>
       </c>
       <c r="E28" t="n">
-        <v>0.2235</v>
+        <v>0.3661</v>
       </c>
       <c r="F28" t="n">
-        <v>0.2247</v>
+        <v>0.3683</v>
       </c>
       <c r="G28" t="n">
-        <v>163.3969</v>
+        <v>99.72539999999999</v>
       </c>
       <c r="H28" t="n">
-        <v>3.05</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs</t>
+          <t>baseline_dynstock2</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1227,209 +1233,215 @@
         <v>2</v>
       </c>
       <c r="D29" t="n">
-        <v>0.1982</v>
+        <v>0.2488</v>
       </c>
       <c r="E29" t="n">
-        <v>0.198</v>
+        <v>0.2481</v>
       </c>
       <c r="F29" t="n">
-        <v>0.1985</v>
+        <v>0.2496</v>
       </c>
       <c r="G29" t="n">
-        <v>184.7105</v>
+        <v>147.1485</v>
       </c>
       <c r="H29" t="n">
-        <v>3.75</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>avg_g_window_hg</t>
+          <t>peak_g</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>1.0148</v>
+        <v>0.2302</v>
       </c>
       <c r="E30" t="n">
-        <v>1.0148</v>
+        <v>0.2295</v>
       </c>
       <c r="F30" t="n">
-        <v>1.0148</v>
+        <v>0.2309</v>
       </c>
       <c r="G30" t="n">
-        <v>64.18680000000001</v>
-      </c>
-      <c r="H30" t="n">
-        <v>3.8</v>
-      </c>
+        <v>159.0684</v>
+      </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>avg_g_window</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>1.011</v>
+        <v>0.2283</v>
       </c>
       <c r="E31" t="n">
-        <v>1.0062</v>
+        <v>0.2276</v>
       </c>
       <c r="F31" t="n">
-        <v>1.0158</v>
+        <v>0.2291</v>
       </c>
       <c r="G31" t="n">
-        <v>50.3918</v>
-      </c>
-      <c r="H31" t="inlineStr"/>
+        <v>160.3908</v>
+      </c>
+      <c r="H31" t="n">
+        <v>3.2</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>yaw_intent</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
-        <v>0.9869</v>
+        <v>0.2258</v>
       </c>
       <c r="E32" t="n">
-        <v>0.9869</v>
+        <v>0.2252</v>
       </c>
       <c r="F32" t="n">
-        <v>0.9869</v>
+        <v>0.2263</v>
       </c>
       <c r="G32" t="n">
-        <v>66.0052</v>
+        <v>162.2099</v>
       </c>
       <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>combined</t>
+          <t>peak_g_norpm</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D33" t="n">
-        <v>0.2276</v>
+        <v>0.2245</v>
       </c>
       <c r="E33" t="n">
-        <v>0.2276</v>
+        <v>0.2238</v>
       </c>
       <c r="F33" t="n">
-        <v>0.2276</v>
+        <v>0.2252</v>
       </c>
       <c r="G33" t="n">
-        <v>160.9226</v>
+        <v>163.1152</v>
       </c>
       <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>baseline_dynstock</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C34" t="n">
         <v>2</v>
       </c>
       <c r="D34" t="n">
-        <v>0.2159</v>
+        <v>0.2241</v>
       </c>
       <c r="E34" t="n">
-        <v>0.2156</v>
+        <v>0.2235</v>
       </c>
       <c r="F34" t="n">
-        <v>0.2162</v>
+        <v>0.2247</v>
       </c>
       <c r="G34" t="n">
-        <v>301.7328</v>
-      </c>
-      <c r="H34" t="inlineStr"/>
+        <v>163.3969</v>
+      </c>
+      <c r="H34" t="n">
+        <v>3.05</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>baseline_dynstocknoabs</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C35" t="n">
         <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>0.1782</v>
+        <v>0.1982</v>
       </c>
       <c r="E35" t="n">
-        <v>0.1779</v>
+        <v>0.198</v>
       </c>
       <c r="F35" t="n">
-        <v>0.1784</v>
+        <v>0.1985</v>
       </c>
       <c r="G35" t="n">
-        <v>365.637</v>
-      </c>
-      <c r="H35" t="inlineStr"/>
+        <v>184.7105</v>
+      </c>
+      <c r="H35" t="n">
+        <v>3.75</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>avg_g_window</t>
+          <t>avg_g_window_hg</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>80</v>
       </c>
       <c r="C36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>0.1778</v>
+        <v>1.0148</v>
       </c>
       <c r="E36" t="n">
-        <v>0.1776</v>
+        <v>1.0148</v>
       </c>
       <c r="F36" t="n">
-        <v>0.178</v>
+        <v>1.0148</v>
       </c>
       <c r="G36" t="n">
-        <v>366.3356</v>
-      </c>
-      <c r="H36" t="inlineStr"/>
+        <v>64.18680000000001</v>
+      </c>
+      <c r="H36" t="n">
+        <v>3.8</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1439,18 +1451,174 @@
         <v>2</v>
       </c>
       <c r="D37" t="n">
+        <v>1.011</v>
+      </c>
+      <c r="E37" t="n">
+        <v>1.0062</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1.0158</v>
+      </c>
+      <c r="G37" t="n">
+        <v>50.3918</v>
+      </c>
+      <c r="H37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>baseline_stock800</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>80</v>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.9869</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.9869</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.9869</v>
+      </c>
+      <c r="G38" t="n">
+        <v>66.0052</v>
+      </c>
+      <c r="H38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>combined</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>80</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.2276</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.2276</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.2276</v>
+      </c>
+      <c r="G39" t="n">
+        <v>160.9226</v>
+      </c>
+      <c r="H39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>80</v>
+      </c>
+      <c r="C40" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.2159</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.2156</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.2162</v>
+      </c>
+      <c r="G40" t="n">
+        <v>301.7328</v>
+      </c>
+      <c r="H40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>peak_g</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>80</v>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.1782</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.1779</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.1784</v>
+      </c>
+      <c r="G41" t="n">
+        <v>365.637</v>
+      </c>
+      <c r="H41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>avg_g_window</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>80</v>
+      </c>
+      <c r="C42" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.1778</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.1776</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="G42" t="n">
+        <v>366.3356</v>
+      </c>
+      <c r="H42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>yaw_intent</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>80</v>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="n">
         <v>0.1766</v>
       </c>
-      <c r="E37" t="n">
+      <c r="E43" t="n">
         <v>0.1766</v>
       </c>
-      <c r="F37" t="n">
+      <c r="F43" t="n">
         <v>0.1766</v>
       </c>
-      <c r="G37" t="n">
+      <c r="G43" t="n">
         <v>368.9042</v>
       </c>
-      <c r="H37" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1463,7 +1631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4296,36 +4464,36 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ensemble</t>
+          <t>bandsweep</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_b10o1</t>
         </is>
       </c>
       <c r="D79" t="n">
         <v>60</v>
       </c>
       <c r="E79" t="n">
-        <v>1.0488</v>
+        <v>1.0639</v>
       </c>
       <c r="F79" t="n">
-        <v>34.9145</v>
+        <v>34.4174</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>1788401068-0005</t>
+          <t>1788404082-0009</t>
         </is>
       </c>
       <c r="H79" t="n">
-        <v>34.91</v>
+        <v>34.42</v>
       </c>
       <c r="I79" t="n">
-        <v>3.5</v>
+        <v>2.8</v>
       </c>
       <c r="J79" t="n">
-        <v>2.48</v>
+        <v>2.47</v>
       </c>
     </row>
     <row r="80">
@@ -4336,36 +4504,36 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ensemble</t>
+          <t>bandsweep</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_b10o1</t>
         </is>
       </c>
       <c r="D80" t="n">
         <v>60</v>
       </c>
       <c r="E80" t="n">
-        <v>1.0376</v>
+        <v>1.0578</v>
       </c>
       <c r="F80" t="n">
-        <v>35.29</v>
+        <v>34.6159</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>1788401101-0006</t>
+          <t>1788404114-0010</t>
         </is>
       </c>
       <c r="H80" t="n">
-        <v>35.29</v>
+        <v>34.62</v>
       </c>
       <c r="I80" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="J80" t="n">
-        <v>2.5</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="81">
@@ -4376,36 +4544,36 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>restructure</t>
+          <t>bandsweep</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
+          <t>band_g_mix_b1o1</t>
         </is>
       </c>
       <c r="D81" t="n">
         <v>60</v>
       </c>
       <c r="E81" t="n">
-        <v>1.1085</v>
+        <v>1.0902</v>
       </c>
       <c r="F81" t="n">
-        <v>33.0351</v>
+        <v>33.5875</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>1788399311-0002</t>
+          <t>1788403804-0001</t>
         </is>
       </c>
       <c r="H81" t="n">
-        <v>33.04</v>
+        <v>33.59</v>
       </c>
       <c r="I81" t="n">
-        <v>4.8</v>
+        <v>1.6</v>
       </c>
       <c r="J81" t="n">
-        <v>2.4</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="82">
@@ -4416,36 +4584,36 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ensemble</t>
+          <t>bandsweep</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ens_band_g_mix5</t>
+          <t>band_g_mix_b1o1</t>
         </is>
       </c>
       <c r="D82" t="n">
         <v>60</v>
       </c>
       <c r="E82" t="n">
-        <v>1.0736</v>
+        <v>1.1133</v>
       </c>
       <c r="F82" t="n">
-        <v>34.1079</v>
+        <v>32.8921</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>1788400929-0001</t>
+          <t>1788403836-0002</t>
         </is>
       </c>
       <c r="H82" t="n">
-        <v>34.11</v>
+        <v>32.89</v>
       </c>
       <c r="I82" t="n">
-        <v>2.4</v>
+        <v>1.4</v>
       </c>
       <c r="J82" t="n">
-        <v>2.44</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="83">
@@ -4456,35 +4624,515 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
+          <t>bandsweep</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>band_g_mix_b20o1</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>60</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0.4061</v>
+      </c>
+      <c r="F83" t="n">
+        <v>90.16759999999999</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>1788404151-0011</t>
+        </is>
+      </c>
+      <c r="H83" t="n">
+        <v>90.17</v>
+      </c>
+      <c r="I83" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J83" t="n">
+        <v>5.28</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>bandsweep</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>band_g_mix_b20o1</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>60</v>
+      </c>
+      <c r="E84" t="n">
+        <v>1.0401</v>
+      </c>
+      <c r="F84" t="n">
+        <v>35.2051</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>1788404187-0012</t>
+        </is>
+      </c>
+      <c r="H84" t="n">
+        <v>35.21</v>
+      </c>
+      <c r="I84" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="J84" t="n">
+        <v>2.55</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>bandsweep</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>band_g_mix_b2p5o2</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>60</v>
+      </c>
+      <c r="E85" t="n">
+        <v>1.0823</v>
+      </c>
+      <c r="F85" t="n">
+        <v>33.8327</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>1788403874-0003</t>
+        </is>
+      </c>
+      <c r="H85" t="n">
+        <v>33.83</v>
+      </c>
+      <c r="I85" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J85" t="n">
+        <v>2.47</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>bandsweep</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>band_g_mix_b2p5o2</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>60</v>
+      </c>
+      <c r="E86" t="n">
+        <v>1.0944</v>
+      </c>
+      <c r="F86" t="n">
+        <v>33.4601</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>1788403907-0004</t>
+        </is>
+      </c>
+      <c r="H86" t="n">
+        <v>33.46</v>
+      </c>
+      <c r="I86" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J86" t="n">
+        <v>2.45</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>bandsweep</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>band_g_mix_b5o2</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>60</v>
+      </c>
+      <c r="E87" t="n">
+        <v>1.0612</v>
+      </c>
+      <c r="F87" t="n">
+        <v>34.5049</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>1788403944-0005</t>
+        </is>
+      </c>
+      <c r="H87" t="n">
+        <v>34.51</v>
+      </c>
+      <c r="I87" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J87" t="n">
+        <v>2.48</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>bandsweep</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>band_g_mix_b5o2</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>60</v>
+      </c>
+      <c r="E88" t="n">
+        <v>1.0546</v>
+      </c>
+      <c r="F88" t="n">
+        <v>34.7221</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>1788403976-0006</t>
+        </is>
+      </c>
+      <c r="H88" t="n">
+        <v>34.72</v>
+      </c>
+      <c r="I88" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="J88" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>bandsweep</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>band_g_mix_b7p5o3</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>60</v>
+      </c>
+      <c r="E89" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="F89" t="n">
+        <v>34.9402</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>1788404012-0007</t>
+        </is>
+      </c>
+      <c r="H89" t="n">
+        <v>34.94</v>
+      </c>
+      <c r="I89" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J89" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>bandsweep</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>band_g_mix_b7p5o3</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>60</v>
+      </c>
+      <c r="E90" t="n">
+        <v>1.0741</v>
+      </c>
+      <c r="F90" t="n">
+        <v>34.0931</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>1788404045-0008</t>
+        </is>
+      </c>
+      <c r="H90" t="n">
+        <v>34.09</v>
+      </c>
+      <c r="I90" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J90" t="n">
+        <v>2.41</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
           <t>ensemble</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>band_g_mix_s1</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>60</v>
+      </c>
+      <c r="E91" t="n">
+        <v>1.0488</v>
+      </c>
+      <c r="F91" t="n">
+        <v>34.9145</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>1788401068-0005</t>
+        </is>
+      </c>
+      <c r="H91" t="n">
+        <v>34.91</v>
+      </c>
+      <c r="I91" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J91" t="n">
+        <v>2.48</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>band_g_mix_s1</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>60</v>
+      </c>
+      <c r="E92" t="n">
+        <v>1.0376</v>
+      </c>
+      <c r="F92" t="n">
+        <v>35.29</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>1788401101-0006</t>
+        </is>
+      </c>
+      <c r="H92" t="n">
+        <v>35.29</v>
+      </c>
+      <c r="I92" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J92" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>restructure</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>baseline_dyn</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>60</v>
+      </c>
+      <c r="E93" t="n">
+        <v>1.1085</v>
+      </c>
+      <c r="F93" t="n">
+        <v>33.0351</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>1788399311-0002</t>
+        </is>
+      </c>
+      <c r="H93" t="n">
+        <v>33.04</v>
+      </c>
+      <c r="I93" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="J93" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
         <is>
           <t>ens_band_g_mix5</t>
         </is>
       </c>
-      <c r="D83" t="n">
-        <v>60</v>
-      </c>
-      <c r="E83" t="n">
+      <c r="D94" t="n">
+        <v>60</v>
+      </c>
+      <c r="E94" t="n">
+        <v>1.0736</v>
+      </c>
+      <c r="F94" t="n">
+        <v>34.1079</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>1788400929-0001</t>
+        </is>
+      </c>
+      <c r="H94" t="n">
+        <v>34.11</v>
+      </c>
+      <c r="I94" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J94" t="n">
+        <v>2.44</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>ens_band_g_mix5</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>60</v>
+      </c>
+      <c r="E95" t="n">
         <v>1.0538</v>
       </c>
-      <c r="F83" t="n">
+      <c r="F95" t="n">
         <v>34.7482</v>
       </c>
-      <c r="G83" t="inlineStr">
+      <c r="G95" t="inlineStr">
         <is>
           <t>1788400962-0002</t>
         </is>
       </c>
-      <c r="H83" t="n">
+      <c r="H95" t="n">
         <v>34.75</v>
       </c>
-      <c r="I83" t="n">
+      <c r="I95" t="n">
         <v>2</v>
       </c>
-      <c r="J83" t="n">
+      <c r="J95" t="n">
         <v>2.48</v>
       </c>
     </row>
@@ -4499,7 +5147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -4713,7 +5361,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_b10o1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4723,7 +5371,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-02T18:54:00</t>
+          <t>2026-09-02T19:47:35</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -4751,7 +5399,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K7" t="n">
         <v>1</v>
@@ -4761,7 +5409,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>[0.14226, 0.15404, 0.16814, 0.16762]</t>
+          <t>[0.14416, 0.15257, 0.16969, 0.16911]</t>
         </is>
       </c>
       <c r="N7" t="inlineStr"/>
@@ -4769,7 +5417,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>band_g_mix_s2</t>
+          <t>band_g_mix_b1o1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4779,7 +5427,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-09-02T18:55:36</t>
+          <t>2026-09-02T19:41:08</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -4807,7 +5455,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K8" t="n">
         <v>1</v>
@@ -4817,7 +5465,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>[0.15115, 0.15324, 0.16928, 0.16978]</t>
+          <t>[0.15124, 0.15757, 0.16939, 0.16889]</t>
         </is>
       </c>
       <c r="N8" t="inlineStr"/>
@@ -4825,7 +5473,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>band_g_mix_s3</t>
+          <t>band_g_mix_b20o1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4835,7 +5483,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-02T18:57:18</t>
+          <t>2026-09-02T19:48:58</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -4863,7 +5511,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="K9" t="n">
         <v>1</v>
@@ -4873,7 +5521,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>[0.15575, 0.16054, 0.1713, 0.17144]</t>
+          <t>[0.14187, 0.15222, 0.16616, 0.16821]</t>
         </is>
       </c>
       <c r="N9" t="inlineStr"/>
@@ -4881,7 +5529,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>band_g_mix_s4</t>
+          <t>band_g_mix_b2p5o2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4891,7 +5539,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-09-02T18:58:55</t>
+          <t>2026-09-02T19:43:04</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -4919,17 +5567,17 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L10" t="n">
         <v>2289</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>[0.14723, 0.15025, 0.16854, 0.16772]</t>
+          <t>[0.14979, 0.15205, 0.16831, 0.16794]</t>
         </is>
       </c>
       <c r="N10" t="inlineStr"/>
@@ -4937,7 +5585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>band_g_mix_s5</t>
+          <t>band_g_mix_b5o2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4947,7 +5595,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-02T19:00:42</t>
+          <t>2026-09-02T19:44:39</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -4978,14 +5626,14 @@
         <v>5</v>
       </c>
       <c r="K11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L11" t="n">
         <v>2289</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>[0.14491, 0.15532, 0.16904, 0.16805]</t>
+          <t>[0.14764, 0.15345, 0.16899, 0.16945]</t>
         </is>
       </c>
       <c r="N11" t="inlineStr"/>
@@ -4993,151 +5641,343 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>band_gy_dyn</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
+          <t>band_g_mix_b7p5o3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-09-02T19:46:11</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="K12" t="n">
+        <v>3</v>
+      </c>
+      <c r="L12" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>[0.14858, 0.15176, 0.1686, 0.16846]</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>band_gy_mix</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
+          <t>band_g_mix_s1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:54:00</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>5</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>[0.14226, 0.15404, 0.16814, 0.16762]</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>baseline</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
+          <t>band_g_mix_s2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:55:36</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>5</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>[0.15115, 0.15324, 0.16928, 0.16978]</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+          <t>band_g_mix_s3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:57:18</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>5</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>[0.15575, 0.16054, 0.1713, 0.17144]</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>baseline_dynnoimu</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
+          <t>band_g_mix_s4</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:58:55</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>5</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>[0.14723, 0.15025, 0.16854, 0.16772]</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>baseline_dynstock2</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
+          <t>band_g_mix_s5</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-09-02T19:00:42</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>5</v>
+      </c>
+      <c r="K17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>[0.14491, 0.15532, 0.16904, 0.16805]</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>baseline_dynstock</t>
+          <t>band_gy_dyn</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -5161,7 +6001,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs2</t>
+          <t>band_gy_mix</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -5185,7 +6025,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -5209,7 +6049,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>baseline_hg</t>
+          <t>baseline_dyn</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -5233,7 +6073,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>baseline_norpm</t>
+          <t>baseline_dynnoimu</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -5257,7 +6097,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>baseline_stock16</t>
+          <t>baseline_dynstock2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -5281,7 +6121,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>baseline_dynstock</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -5305,7 +6145,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>baseline_stock</t>
+          <t>baseline_dynstocknoabs2</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -5329,7 +6169,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>baseline_stocknorpm</t>
+          <t>baseline_dynstocknoabs</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -5353,7 +6193,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>combined</t>
+          <t>baseline_hg</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -5377,7 +6217,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>baseline_norpm</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -5401,7 +6241,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>curation_hg</t>
+          <t>baseline_stock16</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -5425,7 +6265,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -5449,7 +6289,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>peak_g_norpm</t>
+          <t>baseline_stock</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -5473,7 +6313,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>baseline_stocknorpm</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -5494,6 +6334,150 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>combined</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>curation</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>curation_hg</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>peak_g</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>peak_g_norpm</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>yaw_intent</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Paired seed test: 1 mph vs 5 mph bands, 3 seeds each; harness attaches to a running game and retries brake_done reads
</commit_message>
<xml_diff>
--- a/results/LSTM_ABS_RESULTS.xlsx
+++ b/results/LSTM_ABS_RESULTS.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -501,91 +501,91 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>band_g_mix</t>
+          <t>band_g_mix_b1o1_s2</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>60</v>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>1.14</v>
+        <v>1.1473</v>
       </c>
       <c r="E3" t="n">
-        <v>1.1067</v>
+        <v>1.1391</v>
       </c>
       <c r="F3" t="n">
-        <v>1.16</v>
+        <v>1.1556</v>
       </c>
       <c r="G3" t="n">
-        <v>32.1309</v>
+        <v>31.9164</v>
       </c>
       <c r="H3" t="n">
-        <v>2.85</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
+          <t>band_g_mix</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>60</v>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>1.1232</v>
+        <v>1.14</v>
       </c>
       <c r="E4" t="n">
-        <v>1.1085</v>
+        <v>1.1067</v>
       </c>
       <c r="F4" t="n">
-        <v>1.1351</v>
+        <v>1.16</v>
       </c>
       <c r="G4" t="n">
-        <v>32.6046</v>
+        <v>32.1309</v>
       </c>
       <c r="H4" t="n">
-        <v>4.7</v>
+        <v>2.85</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>band_gy_mix</t>
+          <t>baseline_dyn</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>60</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D5" t="n">
-        <v>1.1219</v>
+        <v>1.1232</v>
       </c>
       <c r="E5" t="n">
-        <v>1.1198</v>
+        <v>1.1085</v>
       </c>
       <c r="F5" t="n">
-        <v>1.124</v>
+        <v>1.1351</v>
       </c>
       <c r="G5" t="n">
-        <v>32.6393</v>
+        <v>32.6046</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1</t>
+          <t>band_gy_mix</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -595,25 +595,25 @@
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>1.1018</v>
+        <v>1.1219</v>
       </c>
       <c r="E6" t="n">
-        <v>1.0902</v>
+        <v>1.1198</v>
       </c>
       <c r="F6" t="n">
-        <v>1.1133</v>
+        <v>1.124</v>
       </c>
       <c r="G6" t="n">
-        <v>33.2398</v>
+        <v>32.6393</v>
       </c>
       <c r="H6" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>band_g_mix_b2p5o2</t>
+          <t>band_g_mix_b1o1</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -623,53 +623,53 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>1.0884</v>
+        <v>1.1018</v>
       </c>
       <c r="E7" t="n">
-        <v>1.0823</v>
+        <v>1.0902</v>
       </c>
       <c r="F7" t="n">
-        <v>1.0944</v>
+        <v>1.1133</v>
       </c>
       <c r="G7" t="n">
-        <v>33.6464</v>
+        <v>33.2398</v>
       </c>
       <c r="H7" t="n">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>band_g_mix_s2</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>60</v>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>1.0671</v>
+        <v>1.092</v>
       </c>
       <c r="E8" t="n">
-        <v>1.0582</v>
+        <v>1.0916</v>
       </c>
       <c r="F8" t="n">
-        <v>1.0716</v>
+        <v>1.0923</v>
       </c>
       <c r="G8" t="n">
-        <v>34.3171</v>
+        <v>33.534</v>
       </c>
       <c r="H8" t="n">
-        <v>2.3667</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ens_band_g_mix5</t>
+          <t>band_g_mix_b2p5o2</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -679,25 +679,25 @@
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>1.0637</v>
+        <v>1.0884</v>
       </c>
       <c r="E9" t="n">
-        <v>1.0538</v>
+        <v>1.0823</v>
       </c>
       <c r="F9" t="n">
-        <v>1.0736</v>
+        <v>1.0944</v>
       </c>
       <c r="G9" t="n">
-        <v>34.428</v>
+        <v>33.6464</v>
       </c>
       <c r="H9" t="n">
-        <v>2.2</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>band_g_dyn</t>
+          <t>band_g_mix_b1o1_s1</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -707,53 +707,53 @@
         <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>1.0636</v>
+        <v>1.0703</v>
       </c>
       <c r="E10" t="n">
-        <v>1.0628</v>
+        <v>1.0684</v>
       </c>
       <c r="F10" t="n">
-        <v>1.0644</v>
+        <v>1.0722</v>
       </c>
       <c r="G10" t="n">
-        <v>34.4297</v>
+        <v>34.2125</v>
       </c>
       <c r="H10" t="n">
-        <v>4.15</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>band_g_mix_b7p5o3</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>60</v>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>1.061</v>
+        <v>1.0671</v>
       </c>
       <c r="E11" t="n">
-        <v>1.048</v>
+        <v>1.0582</v>
       </c>
       <c r="F11" t="n">
-        <v>1.0741</v>
+        <v>1.0716</v>
       </c>
       <c r="G11" t="n">
-        <v>34.5166</v>
+        <v>34.3171</v>
       </c>
       <c r="H11" t="n">
-        <v>1.45</v>
+        <v>2.3667</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>band_g_mix_b10o1</t>
+          <t>ens_band_g_mix5</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -763,25 +763,25 @@
         <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>1.0608</v>
+        <v>1.0637</v>
       </c>
       <c r="E12" t="n">
-        <v>1.0578</v>
+        <v>1.0538</v>
       </c>
       <c r="F12" t="n">
-        <v>1.0639</v>
+        <v>1.0736</v>
       </c>
       <c r="G12" t="n">
-        <v>34.5166</v>
+        <v>34.428</v>
       </c>
       <c r="H12" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>band_g_mix_b5o2</t>
+          <t>band_g_dyn</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -791,25 +791,25 @@
         <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>1.0579</v>
+        <v>1.0636</v>
       </c>
       <c r="E13" t="n">
-        <v>1.0546</v>
+        <v>1.0628</v>
       </c>
       <c r="F13" t="n">
-        <v>1.0612</v>
+        <v>1.0644</v>
       </c>
       <c r="G13" t="n">
-        <v>34.6135</v>
+        <v>34.4297</v>
       </c>
       <c r="H13" t="n">
-        <v>4.05</v>
+        <v>4.15</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>band_gy_dyn</t>
+          <t>band_g_mix_b7p5o3</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -819,25 +819,25 @@
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>1.0506</v>
+        <v>1.061</v>
       </c>
       <c r="E14" t="n">
-        <v>1.0459</v>
+        <v>1.048</v>
       </c>
       <c r="F14" t="n">
-        <v>1.0554</v>
+        <v>1.0741</v>
       </c>
       <c r="G14" t="n">
-        <v>34.8533</v>
+        <v>34.5166</v>
       </c>
       <c r="H14" t="n">
-        <v>2.6</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_b10o1</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -847,25 +847,25 @@
         <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>1.0432</v>
+        <v>1.0608</v>
       </c>
       <c r="E15" t="n">
-        <v>1.0376</v>
+        <v>1.0578</v>
       </c>
       <c r="F15" t="n">
-        <v>1.0488</v>
+        <v>1.0639</v>
       </c>
       <c r="G15" t="n">
-        <v>35.1022</v>
+        <v>34.5166</v>
       </c>
       <c r="H15" t="n">
-        <v>2.9</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>avg_g_window_hg</t>
+          <t>band_g_mix_b5o2</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -875,53 +875,53 @@
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>1.0301</v>
+        <v>1.0579</v>
       </c>
       <c r="E16" t="n">
-        <v>1.0294</v>
+        <v>1.0546</v>
       </c>
       <c r="F16" t="n">
-        <v>1.0308</v>
+        <v>1.0612</v>
       </c>
       <c r="G16" t="n">
-        <v>35.5482</v>
+        <v>34.6135</v>
       </c>
       <c r="H16" t="n">
-        <v>2.55</v>
+        <v>4.05</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>band_g_mix_s3</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>60</v>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>1.0292</v>
+        <v>1.0553</v>
       </c>
       <c r="E17" t="n">
-        <v>1.0039</v>
+        <v>1.0346</v>
       </c>
       <c r="F17" t="n">
-        <v>1.066</v>
+        <v>1.076</v>
       </c>
       <c r="G17" t="n">
-        <v>35.6013</v>
+        <v>34.7125</v>
       </c>
       <c r="H17" t="n">
-        <v>0.8</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>avg_g_window_stock</t>
+          <t>band_gy_dyn</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -931,23 +931,25 @@
         <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>1.029</v>
+        <v>1.0506</v>
       </c>
       <c r="E18" t="n">
-        <v>1.026</v>
+        <v>1.0459</v>
       </c>
       <c r="F18" t="n">
-        <v>1.0319</v>
+        <v>1.0554</v>
       </c>
       <c r="G18" t="n">
-        <v>35.5875</v>
-      </c>
-      <c r="H18" t="inlineStr"/>
+        <v>34.8533</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2.6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>baseline_hg</t>
+          <t>band_g_mix_s1</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -957,135 +959,135 @@
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>1.0162</v>
+        <v>1.0432</v>
       </c>
       <c r="E19" t="n">
-        <v>1.0147</v>
+        <v>1.0376</v>
       </c>
       <c r="F19" t="n">
-        <v>1.0177</v>
+        <v>1.0488</v>
       </c>
       <c r="G19" t="n">
-        <v>36.0347</v>
+        <v>35.1022</v>
       </c>
       <c r="H19" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>baseline FORCE_CMD=1.0</t>
+          <t>avg_g_window_hg</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>60</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>1.0017</v>
+        <v>1.0301</v>
       </c>
       <c r="E20" t="n">
-        <v>1.0017</v>
+        <v>1.0294</v>
       </c>
       <c r="F20" t="n">
-        <v>1.0017</v>
+        <v>1.0308</v>
       </c>
       <c r="G20" t="n">
-        <v>36.5572</v>
+        <v>35.5482</v>
       </c>
       <c r="H20" t="n">
-        <v>3.5</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>baseline_stocknorpm</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>60</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.0292</v>
       </c>
       <c r="E21" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.0039</v>
       </c>
       <c r="F21" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.066</v>
       </c>
       <c r="G21" t="n">
-        <v>37.0845</v>
+        <v>35.6013</v>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>baseline_stock</t>
+          <t>avg_g_window_stock</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>60</v>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>0.8937</v>
+        <v>1.029</v>
       </c>
       <c r="E22" t="n">
-        <v>0.8933</v>
+        <v>1.026</v>
       </c>
       <c r="F22" t="n">
-        <v>0.8942</v>
+        <v>1.0319</v>
       </c>
       <c r="G22" t="n">
-        <v>40.9724</v>
-      </c>
-      <c r="H22" t="n">
-        <v>3.5667</v>
-      </c>
+        <v>35.5875</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>curation_hg</t>
+          <t>band_g_mix_b1o1_s3</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>60</v>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>0.8874</v>
+        <v>1.0233</v>
       </c>
       <c r="E23" t="n">
-        <v>0.8813</v>
+        <v>1.0165</v>
       </c>
       <c r="F23" t="n">
-        <v>0.8935</v>
+        <v>1.0395</v>
       </c>
       <c r="G23" t="n">
-        <v>41.266</v>
-      </c>
-      <c r="H23" t="inlineStr"/>
+        <v>35.7888</v>
+      </c>
+      <c r="H23" t="n">
+        <v>3.2</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs2</t>
+          <t>baseline_hg</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1095,25 +1097,25 @@
         <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>0.8228</v>
+        <v>1.0162</v>
       </c>
       <c r="E24" t="n">
-        <v>0.8045</v>
+        <v>1.0147</v>
       </c>
       <c r="F24" t="n">
-        <v>0.8411</v>
+        <v>1.0177</v>
       </c>
       <c r="G24" t="n">
-        <v>44.527</v>
+        <v>36.0347</v>
       </c>
       <c r="H24" t="n">
-        <v>1.9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>baseline_stock16</t>
+          <t>baseline FORCE_CMD=1.0</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1123,51 +1125,53 @@
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>0.7467</v>
+        <v>1.0017</v>
       </c>
       <c r="E25" t="n">
-        <v>0.7467</v>
+        <v>1.0017</v>
       </c>
       <c r="F25" t="n">
-        <v>0.7467</v>
+        <v>1.0017</v>
       </c>
       <c r="G25" t="n">
-        <v>49.0416</v>
-      </c>
-      <c r="H25" t="inlineStr"/>
+        <v>36.5572</v>
+      </c>
+      <c r="H25" t="n">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>band_g_mix_b20o1</t>
+          <t>baseline_stocknorpm</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>60</v>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>0.7231</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="E26" t="n">
-        <v>0.4061</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="F26" t="n">
-        <v>1.0401</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="G26" t="n">
-        <v>62.6864</v>
+        <v>37.0845</v>
       </c>
       <c r="H26" t="n">
-        <v>1.95</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>baseline_stock</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1177,25 +1181,25 @@
         <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>0.4106</v>
+        <v>0.8937</v>
       </c>
       <c r="E27" t="n">
-        <v>0.2278</v>
+        <v>0.8933</v>
       </c>
       <c r="F27" t="n">
-        <v>0.7759</v>
+        <v>0.8942</v>
       </c>
       <c r="G27" t="n">
-        <v>122.7889</v>
+        <v>40.9724</v>
       </c>
       <c r="H27" t="n">
-        <v>2.1</v>
+        <v>3.5667</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>baseline_dynnoimu</t>
+          <t>curation_hg</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1205,25 +1209,23 @@
         <v>2</v>
       </c>
       <c r="D28" t="n">
-        <v>0.3672</v>
+        <v>0.8874</v>
       </c>
       <c r="E28" t="n">
-        <v>0.3661</v>
+        <v>0.8813</v>
       </c>
       <c r="F28" t="n">
-        <v>0.3683</v>
+        <v>0.8935</v>
       </c>
       <c r="G28" t="n">
-        <v>99.72539999999999</v>
-      </c>
-      <c r="H28" t="n">
-        <v>4.6</v>
-      </c>
+        <v>41.266</v>
+      </c>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>baseline_dynstock2</t>
+          <t>baseline_dynstocknoabs2</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1233,105 +1235,107 @@
         <v>2</v>
       </c>
       <c r="D29" t="n">
-        <v>0.2488</v>
+        <v>0.8228</v>
       </c>
       <c r="E29" t="n">
-        <v>0.2481</v>
+        <v>0.8045</v>
       </c>
       <c r="F29" t="n">
-        <v>0.2496</v>
+        <v>0.8411</v>
       </c>
       <c r="G29" t="n">
-        <v>147.1485</v>
+        <v>44.527</v>
       </c>
       <c r="H29" t="n">
-        <v>2.8</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>baseline_stock16</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>60</v>
       </c>
       <c r="C30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>0.2302</v>
+        <v>0.7467</v>
       </c>
       <c r="E30" t="n">
-        <v>0.2295</v>
+        <v>0.7467</v>
       </c>
       <c r="F30" t="n">
-        <v>0.2309</v>
+        <v>0.7467</v>
       </c>
       <c r="G30" t="n">
-        <v>159.0684</v>
+        <v>49.0416</v>
       </c>
       <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>avg_g_window</t>
+          <t>band_g_mix_b20o1</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>60</v>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D31" t="n">
-        <v>0.2283</v>
+        <v>0.7231</v>
       </c>
       <c r="E31" t="n">
-        <v>0.2276</v>
+        <v>0.4061</v>
       </c>
       <c r="F31" t="n">
-        <v>0.2291</v>
+        <v>1.0401</v>
       </c>
       <c r="G31" t="n">
-        <v>160.3908</v>
+        <v>62.6864</v>
       </c>
       <c r="H31" t="n">
-        <v>3.2</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>60</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>0.2258</v>
+        <v>0.4106</v>
       </c>
       <c r="E32" t="n">
-        <v>0.2252</v>
+        <v>0.2278</v>
       </c>
       <c r="F32" t="n">
-        <v>0.2263</v>
+        <v>0.7759</v>
       </c>
       <c r="G32" t="n">
-        <v>162.2099</v>
-      </c>
-      <c r="H32" t="inlineStr"/>
+        <v>122.7889</v>
+      </c>
+      <c r="H32" t="n">
+        <v>2.1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>peak_g_norpm</t>
+          <t>baseline_dynnoimu</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1341,23 +1345,25 @@
         <v>2</v>
       </c>
       <c r="D33" t="n">
-        <v>0.2245</v>
+        <v>0.3672</v>
       </c>
       <c r="E33" t="n">
-        <v>0.2238</v>
+        <v>0.3661</v>
       </c>
       <c r="F33" t="n">
-        <v>0.2252</v>
+        <v>0.3683</v>
       </c>
       <c r="G33" t="n">
-        <v>163.1152</v>
-      </c>
-      <c r="H33" t="inlineStr"/>
+        <v>99.72539999999999</v>
+      </c>
+      <c r="H33" t="n">
+        <v>4.6</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>baseline_dynstock</t>
+          <t>baseline_dynstock2</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1367,25 +1373,25 @@
         <v>2</v>
       </c>
       <c r="D34" t="n">
-        <v>0.2241</v>
+        <v>0.2488</v>
       </c>
       <c r="E34" t="n">
-        <v>0.2235</v>
+        <v>0.2481</v>
       </c>
       <c r="F34" t="n">
-        <v>0.2247</v>
+        <v>0.2496</v>
       </c>
       <c r="G34" t="n">
-        <v>163.3969</v>
+        <v>147.1485</v>
       </c>
       <c r="H34" t="n">
-        <v>3.05</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs</t>
+          <t>peak_g</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1395,183 +1401,187 @@
         <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>0.1982</v>
+        <v>0.2302</v>
       </c>
       <c r="E35" t="n">
-        <v>0.198</v>
+        <v>0.2295</v>
       </c>
       <c r="F35" t="n">
-        <v>0.1985</v>
+        <v>0.2309</v>
       </c>
       <c r="G35" t="n">
-        <v>184.7105</v>
-      </c>
-      <c r="H35" t="n">
-        <v>3.75</v>
-      </c>
+        <v>159.0684</v>
+      </c>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>avg_g_window_hg</t>
+          <t>avg_g_window</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>1.0148</v>
+        <v>0.2283</v>
       </c>
       <c r="E36" t="n">
-        <v>1.0148</v>
+        <v>0.2276</v>
       </c>
       <c r="F36" t="n">
-        <v>1.0148</v>
+        <v>0.2291</v>
       </c>
       <c r="G36" t="n">
-        <v>64.18680000000001</v>
+        <v>160.3908</v>
       </c>
       <c r="H36" t="n">
-        <v>3.8</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>yaw_intent</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C37" t="n">
         <v>2</v>
       </c>
       <c r="D37" t="n">
-        <v>1.011</v>
+        <v>0.2258</v>
       </c>
       <c r="E37" t="n">
-        <v>1.0062</v>
+        <v>0.2252</v>
       </c>
       <c r="F37" t="n">
-        <v>1.0158</v>
+        <v>0.2263</v>
       </c>
       <c r="G37" t="n">
-        <v>50.3918</v>
+        <v>162.2099</v>
       </c>
       <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>peak_g_norpm</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" t="n">
-        <v>0.9869</v>
+        <v>0.2245</v>
       </c>
       <c r="E38" t="n">
-        <v>0.9869</v>
+        <v>0.2238</v>
       </c>
       <c r="F38" t="n">
-        <v>0.9869</v>
+        <v>0.2252</v>
       </c>
       <c r="G38" t="n">
-        <v>66.0052</v>
+        <v>163.1152</v>
       </c>
       <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>combined</t>
+          <t>baseline_dynstock</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2276</v>
+        <v>0.2241</v>
       </c>
       <c r="E39" t="n">
-        <v>0.2276</v>
+        <v>0.2235</v>
       </c>
       <c r="F39" t="n">
-        <v>0.2276</v>
+        <v>0.2247</v>
       </c>
       <c r="G39" t="n">
-        <v>160.9226</v>
-      </c>
-      <c r="H39" t="inlineStr"/>
+        <v>163.3969</v>
+      </c>
+      <c r="H39" t="n">
+        <v>3.05</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>baseline_dynstocknoabs</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C40" t="n">
         <v>2</v>
       </c>
       <c r="D40" t="n">
-        <v>0.2159</v>
+        <v>0.1982</v>
       </c>
       <c r="E40" t="n">
-        <v>0.2156</v>
+        <v>0.198</v>
       </c>
       <c r="F40" t="n">
-        <v>0.2162</v>
+        <v>0.1985</v>
       </c>
       <c r="G40" t="n">
-        <v>301.7328</v>
-      </c>
-      <c r="H40" t="inlineStr"/>
+        <v>184.7105</v>
+      </c>
+      <c r="H40" t="n">
+        <v>3.75</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>avg_g_window_hg</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>80</v>
       </c>
       <c r="C41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>0.1782</v>
+        <v>1.0148</v>
       </c>
       <c r="E41" t="n">
-        <v>0.1779</v>
+        <v>1.0148</v>
       </c>
       <c r="F41" t="n">
-        <v>0.1784</v>
+        <v>1.0148</v>
       </c>
       <c r="G41" t="n">
-        <v>365.637</v>
-      </c>
-      <c r="H41" t="inlineStr"/>
+        <v>64.18680000000001</v>
+      </c>
+      <c r="H41" t="n">
+        <v>3.8</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>avg_g_window</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1581,44 +1591,174 @@
         <v>2</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1778</v>
+        <v>1.011</v>
       </c>
       <c r="E42" t="n">
-        <v>0.1776</v>
+        <v>1.0062</v>
       </c>
       <c r="F42" t="n">
-        <v>0.178</v>
+        <v>1.0158</v>
       </c>
       <c r="G42" t="n">
-        <v>366.3356</v>
+        <v>50.3918</v>
       </c>
       <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>80</v>
       </c>
       <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.9869</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.9869</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.9869</v>
+      </c>
+      <c r="G43" t="n">
+        <v>66.0052</v>
+      </c>
+      <c r="H43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>combined</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>80</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0.2276</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.2276</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.2276</v>
+      </c>
+      <c r="G44" t="n">
+        <v>160.9226</v>
+      </c>
+      <c r="H44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>80</v>
+      </c>
+      <c r="C45" t="n">
         <v>2</v>
       </c>
-      <c r="D43" t="n">
+      <c r="D45" t="n">
+        <v>0.2159</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.2156</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.2162</v>
+      </c>
+      <c r="G45" t="n">
+        <v>301.7328</v>
+      </c>
+      <c r="H45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>peak_g</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>80</v>
+      </c>
+      <c r="C46" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0.1782</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.1779</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.1784</v>
+      </c>
+      <c r="G46" t="n">
+        <v>365.637</v>
+      </c>
+      <c r="H46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>avg_g_window</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>80</v>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0.1778</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.1776</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="G47" t="n">
+        <v>366.3356</v>
+      </c>
+      <c r="H47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>yaw_intent</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>80</v>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" t="n">
         <v>0.1766</v>
       </c>
-      <c r="E43" t="n">
+      <c r="E48" t="n">
         <v>0.1766</v>
       </c>
-      <c r="F43" t="n">
+      <c r="F48" t="n">
         <v>0.1766</v>
       </c>
-      <c r="G43" t="n">
+      <c r="G48" t="n">
         <v>368.9042</v>
       </c>
-      <c r="H43" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1631,7 +1771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4624,37 +4764,31 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>bandsweep</t>
+          <t>pairedseeds</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>band_g_mix_b20o1</t>
+          <t>band_g_mix_b1o1_s1</t>
         </is>
       </c>
       <c r="D83" t="n">
         <v>60</v>
       </c>
       <c r="E83" t="n">
-        <v>0.4061</v>
+        <v>1.0684</v>
       </c>
       <c r="F83" t="n">
-        <v>90.16759999999999</v>
+        <v>34.2738</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>1788404151-0011</t>
-        </is>
-      </c>
-      <c r="H83" t="n">
-        <v>90.17</v>
-      </c>
-      <c r="I83" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="J83" t="n">
-        <v>5.28</v>
-      </c>
+          <t>1788406434-0001</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4664,36 +4798,36 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>bandsweep</t>
+          <t>pairedseeds</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>band_g_mix_b20o1</t>
+          <t>band_g_mix_b1o1_s1</t>
         </is>
       </c>
       <c r="D84" t="n">
         <v>60</v>
       </c>
       <c r="E84" t="n">
-        <v>1.0401</v>
+        <v>1.0722</v>
       </c>
       <c r="F84" t="n">
-        <v>35.2051</v>
+        <v>34.1511</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>1788404187-0012</t>
+          <t>1788406467-0002</t>
         </is>
       </c>
       <c r="H84" t="n">
-        <v>35.21</v>
+        <v>34.15</v>
       </c>
       <c r="I84" t="n">
-        <v>1.3</v>
+        <v>2.1</v>
       </c>
       <c r="J84" t="n">
-        <v>2.55</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="85">
@@ -4704,36 +4838,36 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>bandsweep</t>
+          <t>pairedseeds</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>band_g_mix_b2p5o2</t>
+          <t>band_g_mix_b1o1_s2</t>
         </is>
       </c>
       <c r="D85" t="n">
         <v>60</v>
       </c>
       <c r="E85" t="n">
-        <v>1.0823</v>
+        <v>1.1391</v>
       </c>
       <c r="F85" t="n">
-        <v>33.8327</v>
+        <v>32.146</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>1788403874-0003</t>
+          <t>1788406503-0003</t>
         </is>
       </c>
       <c r="H85" t="n">
-        <v>33.83</v>
+        <v>32.15</v>
       </c>
       <c r="I85" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="J85" t="n">
-        <v>2.47</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="86">
@@ -4744,36 +4878,36 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>bandsweep</t>
+          <t>pairedseeds</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>band_g_mix_b2p5o2</t>
+          <t>band_g_mix_b1o1_s2</t>
         </is>
       </c>
       <c r="D86" t="n">
         <v>60</v>
       </c>
       <c r="E86" t="n">
-        <v>1.0944</v>
+        <v>1.1556</v>
       </c>
       <c r="F86" t="n">
-        <v>33.4601</v>
+        <v>31.6868</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>1788403907-0004</t>
+          <t>1788406537-0004</t>
         </is>
       </c>
       <c r="H86" t="n">
-        <v>33.46</v>
+        <v>31.69</v>
       </c>
       <c r="I86" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="J86" t="n">
-        <v>2.45</v>
+        <v>2.31</v>
       </c>
     </row>
     <row r="87">
@@ -4784,37 +4918,31 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>bandsweep</t>
+          <t>pairedseeds</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>band_g_mix_b5o2</t>
+          <t>band_g_mix_b1o1_s3</t>
         </is>
       </c>
       <c r="D87" t="n">
         <v>60</v>
       </c>
       <c r="E87" t="n">
-        <v>1.0612</v>
+        <v>1.0395</v>
       </c>
       <c r="F87" t="n">
-        <v>34.5049</v>
+        <v>35.2276</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>1788403944-0005</t>
-        </is>
-      </c>
-      <c r="H87" t="n">
-        <v>34.51</v>
-      </c>
-      <c r="I87" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="J87" t="n">
-        <v>2.48</v>
-      </c>
+          <t>1788405673-0002</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4824,36 +4952,36 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>bandsweep</t>
+          <t>pairedseeds</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>band_g_mix_b5o2</t>
+          <t>band_g_mix_b1o1_s3</t>
         </is>
       </c>
       <c r="D88" t="n">
         <v>60</v>
       </c>
       <c r="E88" t="n">
-        <v>1.0546</v>
+        <v>1.0168</v>
       </c>
       <c r="F88" t="n">
-        <v>34.7221</v>
+        <v>36.0148</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>1788403976-0006</t>
+          <t>1788405701-0001</t>
         </is>
       </c>
       <c r="H88" t="n">
-        <v>34.72</v>
+        <v>36.01</v>
       </c>
       <c r="I88" t="n">
-        <v>4.9</v>
+        <v>3.2</v>
       </c>
       <c r="J88" t="n">
-        <v>2.49</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="89">
@@ -4864,37 +4992,31 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>bandsweep</t>
+          <t>pairedseeds</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>band_g_mix_b7p5o3</t>
+          <t>band_g_mix_b1o1_s3</t>
         </is>
       </c>
       <c r="D89" t="n">
         <v>60</v>
       </c>
       <c r="E89" t="n">
-        <v>1.048</v>
+        <v>1.0165</v>
       </c>
       <c r="F89" t="n">
-        <v>34.9402</v>
+        <v>36.0244</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>1788404012-0007</t>
-        </is>
-      </c>
-      <c r="H89" t="n">
-        <v>34.94</v>
-      </c>
-      <c r="I89" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="J89" t="n">
-        <v>2.6</v>
-      </c>
+          <t>1788406573-0005</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4904,37 +5026,31 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>bandsweep</t>
+          <t>pairedseeds</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>band_g_mix_b7p5o3</t>
+          <t>band_g_mix_b1o1_s3</t>
         </is>
       </c>
       <c r="D90" t="n">
         <v>60</v>
       </c>
       <c r="E90" t="n">
-        <v>1.0741</v>
+        <v>1.0203</v>
       </c>
       <c r="F90" t="n">
-        <v>34.0931</v>
+        <v>35.8884</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>1788404045-0008</t>
-        </is>
-      </c>
-      <c r="H90" t="n">
-        <v>34.09</v>
-      </c>
-      <c r="I90" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="J90" t="n">
-        <v>2.41</v>
-      </c>
+          <t>1788406606-0006</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4944,36 +5060,36 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>ensemble</t>
+          <t>bandsweep</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_b20o1</t>
         </is>
       </c>
       <c r="D91" t="n">
         <v>60</v>
       </c>
       <c r="E91" t="n">
-        <v>1.0488</v>
+        <v>0.4061</v>
       </c>
       <c r="F91" t="n">
-        <v>34.9145</v>
+        <v>90.16759999999999</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>1788401068-0005</t>
+          <t>1788404151-0011</t>
         </is>
       </c>
       <c r="H91" t="n">
-        <v>34.91</v>
+        <v>90.17</v>
       </c>
       <c r="I91" t="n">
-        <v>3.5</v>
+        <v>2.6</v>
       </c>
       <c r="J91" t="n">
-        <v>2.48</v>
+        <v>5.28</v>
       </c>
     </row>
     <row r="92">
@@ -4984,36 +5100,36 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ensemble</t>
+          <t>bandsweep</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_b20o1</t>
         </is>
       </c>
       <c r="D92" t="n">
         <v>60</v>
       </c>
       <c r="E92" t="n">
-        <v>1.0376</v>
+        <v>1.0401</v>
       </c>
       <c r="F92" t="n">
-        <v>35.29</v>
+        <v>35.2051</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>1788401101-0006</t>
+          <t>1788404187-0012</t>
         </is>
       </c>
       <c r="H92" t="n">
-        <v>35.29</v>
+        <v>35.21</v>
       </c>
       <c r="I92" t="n">
-        <v>2.3</v>
+        <v>1.3</v>
       </c>
       <c r="J92" t="n">
-        <v>2.5</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="93">
@@ -5024,36 +5140,36 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>restructure</t>
+          <t>bandsweep</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
+          <t>band_g_mix_b2p5o2</t>
         </is>
       </c>
       <c r="D93" t="n">
         <v>60</v>
       </c>
       <c r="E93" t="n">
-        <v>1.1085</v>
+        <v>1.0823</v>
       </c>
       <c r="F93" t="n">
-        <v>33.0351</v>
+        <v>33.8327</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>1788399311-0002</t>
+          <t>1788403874-0003</t>
         </is>
       </c>
       <c r="H93" t="n">
-        <v>33.04</v>
+        <v>33.83</v>
       </c>
       <c r="I93" t="n">
-        <v>4.8</v>
+        <v>1.5</v>
       </c>
       <c r="J93" t="n">
-        <v>2.4</v>
+        <v>2.47</v>
       </c>
     </row>
     <row r="94">
@@ -5064,36 +5180,36 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>ensemble</t>
+          <t>bandsweep</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>ens_band_g_mix5</t>
+          <t>band_g_mix_b2p5o2</t>
         </is>
       </c>
       <c r="D94" t="n">
         <v>60</v>
       </c>
       <c r="E94" t="n">
-        <v>1.0736</v>
+        <v>1.0944</v>
       </c>
       <c r="F94" t="n">
-        <v>34.1079</v>
+        <v>33.4601</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>1788400929-0001</t>
+          <t>1788403907-0004</t>
         </is>
       </c>
       <c r="H94" t="n">
-        <v>34.11</v>
+        <v>33.46</v>
       </c>
       <c r="I94" t="n">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="J94" t="n">
-        <v>2.44</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="95">
@@ -5104,35 +5220,509 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
+          <t>bandsweep</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>band_g_mix_b5o2</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>60</v>
+      </c>
+      <c r="E95" t="n">
+        <v>1.0612</v>
+      </c>
+      <c r="F95" t="n">
+        <v>34.5049</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>1788403944-0005</t>
+        </is>
+      </c>
+      <c r="H95" t="n">
+        <v>34.51</v>
+      </c>
+      <c r="I95" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J95" t="n">
+        <v>2.48</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>bandsweep</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>band_g_mix_b5o2</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>60</v>
+      </c>
+      <c r="E96" t="n">
+        <v>1.0546</v>
+      </c>
+      <c r="F96" t="n">
+        <v>34.7221</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>1788403976-0006</t>
+        </is>
+      </c>
+      <c r="H96" t="n">
+        <v>34.72</v>
+      </c>
+      <c r="I96" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="J96" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>bandsweep</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>band_g_mix_b7p5o3</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>60</v>
+      </c>
+      <c r="E97" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="F97" t="n">
+        <v>34.9402</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>1788404012-0007</t>
+        </is>
+      </c>
+      <c r="H97" t="n">
+        <v>34.94</v>
+      </c>
+      <c r="I97" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J97" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>bandsweep</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>band_g_mix_b7p5o3</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>60</v>
+      </c>
+      <c r="E98" t="n">
+        <v>1.0741</v>
+      </c>
+      <c r="F98" t="n">
+        <v>34.0931</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>1788404045-0008</t>
+        </is>
+      </c>
+      <c r="H98" t="n">
+        <v>34.09</v>
+      </c>
+      <c r="I98" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J98" t="n">
+        <v>2.41</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
           <t>ensemble</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>band_g_mix_s1</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>60</v>
+      </c>
+      <c r="E99" t="n">
+        <v>1.0488</v>
+      </c>
+      <c r="F99" t="n">
+        <v>34.9145</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>1788401068-0005</t>
+        </is>
+      </c>
+      <c r="H99" t="n">
+        <v>34.91</v>
+      </c>
+      <c r="I99" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J99" t="n">
+        <v>2.48</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>band_g_mix_s1</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>60</v>
+      </c>
+      <c r="E100" t="n">
+        <v>1.0376</v>
+      </c>
+      <c r="F100" t="n">
+        <v>35.29</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>1788401101-0006</t>
+        </is>
+      </c>
+      <c r="H100" t="n">
+        <v>35.29</v>
+      </c>
+      <c r="I100" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J100" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>pairedseeds</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>band_g_mix_s2</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>60</v>
+      </c>
+      <c r="E101" t="n">
+        <v>1.0923</v>
+      </c>
+      <c r="F101" t="n">
+        <v>33.5239</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>1788406643-0007</t>
+        </is>
+      </c>
+      <c r="H101" t="n">
+        <v>33.53</v>
+      </c>
+      <c r="I101" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="J101" t="n">
+        <v>2.42</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>pairedseeds</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>band_g_mix_s2</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>60</v>
+      </c>
+      <c r="E102" t="n">
+        <v>1.0916</v>
+      </c>
+      <c r="F102" t="n">
+        <v>33.5441</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>1788406677-0008</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>pairedseeds</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>band_g_mix_s3</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>60</v>
+      </c>
+      <c r="E103" t="n">
+        <v>1.0346</v>
+      </c>
+      <c r="F103" t="n">
+        <v>35.3941</v>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>1788406714-0009</t>
+        </is>
+      </c>
+      <c r="H103" t="n">
+        <v>35.39</v>
+      </c>
+      <c r="I103" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J103" t="n">
+        <v>2.53</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>pairedseeds</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>band_g_mix_s3</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>60</v>
+      </c>
+      <c r="E104" t="n">
+        <v>1.076</v>
+      </c>
+      <c r="F104" t="n">
+        <v>34.0309</v>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>1788406747-0010</t>
+        </is>
+      </c>
+      <c r="H104" t="n">
+        <v>34.03</v>
+      </c>
+      <c r="I104" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J104" t="n">
+        <v>2.56</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>restructure</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>baseline_dyn</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>60</v>
+      </c>
+      <c r="E105" t="n">
+        <v>1.1085</v>
+      </c>
+      <c r="F105" t="n">
+        <v>33.0351</v>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>1788399311-0002</t>
+        </is>
+      </c>
+      <c r="H105" t="n">
+        <v>33.04</v>
+      </c>
+      <c r="I105" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="J105" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
         <is>
           <t>ens_band_g_mix5</t>
         </is>
       </c>
-      <c r="D95" t="n">
-        <v>60</v>
-      </c>
-      <c r="E95" t="n">
+      <c r="D106" t="n">
+        <v>60</v>
+      </c>
+      <c r="E106" t="n">
+        <v>1.0736</v>
+      </c>
+      <c r="F106" t="n">
+        <v>34.1079</v>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>1788400929-0001</t>
+        </is>
+      </c>
+      <c r="H106" t="n">
+        <v>34.11</v>
+      </c>
+      <c r="I106" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J106" t="n">
+        <v>2.44</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>ens_band_g_mix5</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>60</v>
+      </c>
+      <c r="E107" t="n">
         <v>1.0538</v>
       </c>
-      <c r="F95" t="n">
+      <c r="F107" t="n">
         <v>34.7482</v>
       </c>
-      <c r="G95" t="inlineStr">
+      <c r="G107" t="inlineStr">
         <is>
           <t>1788400962-0002</t>
         </is>
       </c>
-      <c r="H95" t="n">
+      <c r="H107" t="n">
         <v>34.75</v>
       </c>
-      <c r="I95" t="n">
+      <c r="I107" t="n">
         <v>2</v>
       </c>
-      <c r="J95" t="n">
+      <c r="J107" t="n">
         <v>2.48</v>
       </c>
     </row>
@@ -5147,7 +5737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N38"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -5473,7 +6063,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>band_g_mix_b20o1</t>
+          <t>band_g_mix_b1o1_s1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5483,7 +6073,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-02T19:48:58</t>
+          <t>2026-09-02T20:06:30</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -5511,7 +6101,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
         <v>1</v>
@@ -5521,7 +6111,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>[0.14187, 0.15222, 0.16616, 0.16821]</t>
+          <t>[0.14701, 0.15565, 0.16829, 0.16836]</t>
         </is>
       </c>
       <c r="N9" t="inlineStr"/>
@@ -5529,7 +6119,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>band_g_mix_b2p5o2</t>
+          <t>band_g_mix_b1o1_s2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -5539,7 +6129,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-09-02T19:43:04</t>
+          <t>2026-09-02T20:08:01</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -5567,17 +6157,17 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L10" t="n">
         <v>2289</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>[0.14979, 0.15205, 0.16831, 0.16794]</t>
+          <t>[0.15093, 0.15348, 0.17001, 0.16992]</t>
         </is>
       </c>
       <c r="N10" t="inlineStr"/>
@@ -5585,7 +6175,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>band_g_mix_b5o2</t>
+          <t>band_g_mix_b1o1_s3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -5595,7 +6185,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-02T19:44:39</t>
+          <t>2026-09-02T20:09:51</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -5623,17 +6213,17 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
         <v>2289</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>[0.14764, 0.15345, 0.16899, 0.16945]</t>
+          <t>[0.15026, 0.15413, 0.1668, 0.16767]</t>
         </is>
       </c>
       <c r="N11" t="inlineStr"/>
@@ -5641,7 +6231,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>band_g_mix_b7p5o3</t>
+          <t>band_g_mix_b20o1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -5651,7 +6241,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-09-02T19:46:11</t>
+          <t>2026-09-02T19:48:58</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -5679,17 +6269,17 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>7.5</v>
+        <v>20</v>
       </c>
       <c r="K12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L12" t="n">
         <v>2289</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>[0.14858, 0.15176, 0.1686, 0.16846]</t>
+          <t>[0.14187, 0.15222, 0.16616, 0.16821]</t>
         </is>
       </c>
       <c r="N12" t="inlineStr"/>
@@ -5697,7 +6287,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_b2p5o2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -5707,7 +6297,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-09-02T18:54:00</t>
+          <t>2026-09-02T19:43:04</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -5735,17 +6325,17 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="K13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L13" t="n">
         <v>2289</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>[0.14226, 0.15404, 0.16814, 0.16762]</t>
+          <t>[0.14979, 0.15205, 0.16831, 0.16794]</t>
         </is>
       </c>
       <c r="N13" t="inlineStr"/>
@@ -5753,7 +6343,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>band_g_mix_s2</t>
+          <t>band_g_mix_b5o2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -5763,7 +6353,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-09-02T18:55:36</t>
+          <t>2026-09-02T19:44:39</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -5794,14 +6384,14 @@
         <v>5</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L14" t="n">
         <v>2289</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>[0.15115, 0.15324, 0.16928, 0.16978]</t>
+          <t>[0.14764, 0.15345, 0.16899, 0.16945]</t>
         </is>
       </c>
       <c r="N14" t="inlineStr"/>
@@ -5809,7 +6399,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>band_g_mix_s3</t>
+          <t>band_g_mix_b7p5o3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -5819,7 +6409,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-09-02T18:57:18</t>
+          <t>2026-09-02T19:46:11</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -5847,17 +6437,17 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>7.5</v>
       </c>
       <c r="K15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L15" t="n">
         <v>2289</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>[0.15575, 0.16054, 0.1713, 0.17144]</t>
+          <t>[0.14858, 0.15176, 0.1686, 0.16846]</t>
         </is>
       </c>
       <c r="N15" t="inlineStr"/>
@@ -5865,7 +6455,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>band_g_mix_s4</t>
+          <t>band_g_mix_s1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -5875,7 +6465,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-09-02T18:58:55</t>
+          <t>2026-09-02T18:54:00</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -5913,7 +6503,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>[0.14723, 0.15025, 0.16854, 0.16772]</t>
+          <t>[0.14226, 0.15404, 0.16814, 0.16762]</t>
         </is>
       </c>
       <c r="N16" t="inlineStr"/>
@@ -5921,7 +6511,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>band_g_mix_s5</t>
+          <t>band_g_mix_s2</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -5931,7 +6521,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-09-02T19:00:42</t>
+          <t>2026-09-02T18:55:36</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -5969,7 +6559,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>[0.14491, 0.15532, 0.16904, 0.16805]</t>
+          <t>[0.15115, 0.15324, 0.16928, 0.16978]</t>
         </is>
       </c>
       <c r="N17" t="inlineStr"/>
@@ -5977,79 +6567,175 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>band_gy_dyn</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
+          <t>band_g_mix_s3</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:57:18</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>5</v>
+      </c>
+      <c r="K18" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>[0.15575, 0.16054, 0.1713, 0.17144]</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>band_gy_mix</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
+          <t>band_g_mix_s4</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:58:55</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>5</v>
+      </c>
+      <c r="K19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>[0.14723, 0.15025, 0.16854, 0.16772]</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>baseline</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
+          <t>band_g_mix_s5</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-09-02T19:00:42</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>5</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>[0.14491, 0.15532, 0.16904, 0.16805]</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
+          <t>band_gy_dyn</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -6073,7 +6759,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>baseline_dynnoimu</t>
+          <t>band_gy_mix</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -6097,7 +6783,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>baseline_dynstock2</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -6121,7 +6807,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>baseline_dynstock</t>
+          <t>baseline_dyn</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -6145,7 +6831,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs2</t>
+          <t>baseline_dynnoimu</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -6169,7 +6855,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs</t>
+          <t>baseline_dynstock2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -6193,7 +6879,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>baseline_hg</t>
+          <t>baseline_dynstock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -6217,7 +6903,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>baseline_norpm</t>
+          <t>baseline_dynstocknoabs2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -6241,7 +6927,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>baseline_stock16</t>
+          <t>baseline_dynstocknoabs</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -6265,7 +6951,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>baseline_hg</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -6289,7 +6975,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>baseline_stock</t>
+          <t>baseline_norpm</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -6313,7 +6999,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>baseline_stocknorpm</t>
+          <t>baseline_stock16</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -6337,7 +7023,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>combined</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -6361,7 +7047,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>baseline_stock</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -6385,7 +7071,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>curation_hg</t>
+          <t>baseline_stocknorpm</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -6409,7 +7095,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>combined</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -6433,7 +7119,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>peak_g_norpm</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -6457,7 +7143,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>curation_hg</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -6478,6 +7164,78 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>peak_g</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>peak_g_norpm</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>yaw_intent</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Slip-band and yaw-match tick weights: lock_sy holds slip 0.02-0.29 to 5mph, 1.14g / 1.7deg yaw vs 1.10g / 4.5deg
</commit_message>
<xml_diff>
--- a/results/LSTM_ABS_RESULTS.xlsx
+++ b/results/LSTM_ABS_RESULTS.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -529,91 +529,91 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>band_g_mix</t>
+          <t>band_g_mix_lock_sy</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>60</v>
       </c>
       <c r="C4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>1.14</v>
+        <v>1.1428</v>
       </c>
       <c r="E4" t="n">
-        <v>1.1067</v>
+        <v>1.1392</v>
       </c>
       <c r="F4" t="n">
-        <v>1.16</v>
+        <v>1.1464</v>
       </c>
       <c r="G4" t="n">
-        <v>32.1309</v>
+        <v>32.0418</v>
       </c>
       <c r="H4" t="n">
-        <v>2.85</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
+          <t>band_g_mix</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>60</v>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" t="n">
-        <v>1.1232</v>
+        <v>1.1305</v>
       </c>
       <c r="E5" t="n">
-        <v>1.1085</v>
+        <v>1.0904</v>
       </c>
       <c r="F5" t="n">
-        <v>1.1351</v>
+        <v>1.16</v>
       </c>
       <c r="G5" t="n">
-        <v>32.6046</v>
+        <v>32.4067</v>
       </c>
       <c r="H5" t="n">
-        <v>4.7</v>
+        <v>3.0625</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>band_gy_mix</t>
+          <t>baseline_dyn</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>60</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>1.1219</v>
+        <v>1.1232</v>
       </c>
       <c r="E6" t="n">
-        <v>1.1198</v>
+        <v>1.1085</v>
       </c>
       <c r="F6" t="n">
-        <v>1.124</v>
+        <v>1.1351</v>
       </c>
       <c r="G6" t="n">
-        <v>32.6393</v>
+        <v>32.6046</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1</t>
+          <t>band_gy_mix</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -623,53 +623,53 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>1.1018</v>
+        <v>1.1219</v>
       </c>
       <c r="E7" t="n">
-        <v>1.0902</v>
+        <v>1.1198</v>
       </c>
       <c r="F7" t="n">
-        <v>1.1133</v>
+        <v>1.124</v>
       </c>
       <c r="G7" t="n">
-        <v>33.2398</v>
+        <v>32.6393</v>
       </c>
       <c r="H7" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>band_g_mix_s2</t>
+          <t>band_g_mix_lock</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>60</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>1.092</v>
+        <v>1.1088</v>
       </c>
       <c r="E8" t="n">
-        <v>1.0916</v>
+        <v>1.0995</v>
       </c>
       <c r="F8" t="n">
-        <v>1.0923</v>
+        <v>1.1277</v>
       </c>
       <c r="G8" t="n">
-        <v>33.534</v>
+        <v>33.0293</v>
       </c>
       <c r="H8" t="n">
-        <v>4.9</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>band_g_mix_b2p5o2</t>
+          <t>band_g_mix_b1o1</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -679,25 +679,25 @@
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>1.0884</v>
+        <v>1.1018</v>
       </c>
       <c r="E9" t="n">
-        <v>1.0823</v>
+        <v>1.0902</v>
       </c>
       <c r="F9" t="n">
-        <v>1.0944</v>
+        <v>1.1133</v>
       </c>
       <c r="G9" t="n">
-        <v>33.6464</v>
+        <v>33.2398</v>
       </c>
       <c r="H9" t="n">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1_s1</t>
+          <t>band_g_mix_s2</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -707,53 +707,53 @@
         <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>1.0703</v>
+        <v>1.092</v>
       </c>
       <c r="E10" t="n">
-        <v>1.0684</v>
+        <v>1.0916</v>
       </c>
       <c r="F10" t="n">
-        <v>1.0722</v>
+        <v>1.0923</v>
       </c>
       <c r="G10" t="n">
-        <v>34.2125</v>
+        <v>33.534</v>
       </c>
       <c r="H10" t="n">
-        <v>2.1</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>band_g_mix_b2p5o2</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>60</v>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>1.0671</v>
+        <v>1.0884</v>
       </c>
       <c r="E11" t="n">
-        <v>1.0582</v>
+        <v>1.0823</v>
       </c>
       <c r="F11" t="n">
-        <v>1.0716</v>
+        <v>1.0944</v>
       </c>
       <c r="G11" t="n">
-        <v>34.3171</v>
+        <v>33.6464</v>
       </c>
       <c r="H11" t="n">
-        <v>2.3667</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ens_band_g_mix5</t>
+          <t>baseline_dyn_lock</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -763,53 +763,53 @@
         <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>1.0637</v>
+        <v>1.0787</v>
       </c>
       <c r="E12" t="n">
-        <v>1.0538</v>
+        <v>1.0756</v>
       </c>
       <c r="F12" t="n">
-        <v>1.0736</v>
+        <v>1.0817</v>
       </c>
       <c r="G12" t="n">
-        <v>34.428</v>
+        <v>33.9476</v>
       </c>
       <c r="H12" t="n">
-        <v>2.2</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>band_g_dyn</t>
+          <t>band_g_mix_lock_s</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>60</v>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>1.0636</v>
+        <v>1.0736</v>
       </c>
       <c r="E13" t="n">
-        <v>1.0628</v>
+        <v>1.0691</v>
       </c>
       <c r="F13" t="n">
-        <v>1.0644</v>
+        <v>1.0781</v>
       </c>
       <c r="G13" t="n">
-        <v>34.4297</v>
+        <v>34.1097</v>
       </c>
       <c r="H13" t="n">
-        <v>4.15</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>band_g_mix_b7p5o3</t>
+          <t>band_g_mix_b1o1_s1</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -819,53 +819,53 @@
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>1.061</v>
+        <v>1.0703</v>
       </c>
       <c r="E14" t="n">
-        <v>1.048</v>
+        <v>1.0684</v>
       </c>
       <c r="F14" t="n">
-        <v>1.0741</v>
+        <v>1.0722</v>
       </c>
       <c r="G14" t="n">
-        <v>34.5166</v>
+        <v>34.2125</v>
       </c>
       <c r="H14" t="n">
-        <v>1.45</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>band_g_mix_b10o1</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>60</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>1.0608</v>
+        <v>1.0671</v>
       </c>
       <c r="E15" t="n">
-        <v>1.0578</v>
+        <v>1.0582</v>
       </c>
       <c r="F15" t="n">
-        <v>1.0639</v>
+        <v>1.0716</v>
       </c>
       <c r="G15" t="n">
-        <v>34.5166</v>
+        <v>34.3171</v>
       </c>
       <c r="H15" t="n">
-        <v>2.4</v>
+        <v>2.3667</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>band_g_mix_b5o2</t>
+          <t>ens_band_g_mix5</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -875,25 +875,25 @@
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>1.0579</v>
+        <v>1.0637</v>
       </c>
       <c r="E16" t="n">
-        <v>1.0546</v>
+        <v>1.0538</v>
       </c>
       <c r="F16" t="n">
-        <v>1.0612</v>
+        <v>1.0736</v>
       </c>
       <c r="G16" t="n">
-        <v>34.6135</v>
+        <v>34.428</v>
       </c>
       <c r="H16" t="n">
-        <v>4.05</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>band_g_mix_s3</t>
+          <t>band_g_dyn</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -903,25 +903,25 @@
         <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>1.0553</v>
+        <v>1.0636</v>
       </c>
       <c r="E17" t="n">
-        <v>1.0346</v>
+        <v>1.0628</v>
       </c>
       <c r="F17" t="n">
-        <v>1.076</v>
+        <v>1.0644</v>
       </c>
       <c r="G17" t="n">
-        <v>34.7125</v>
+        <v>34.4297</v>
       </c>
       <c r="H17" t="n">
-        <v>2.15</v>
+        <v>4.15</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>band_gy_dyn</t>
+          <t>band_g_mix_b7p5o3</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -931,25 +931,25 @@
         <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>1.0506</v>
+        <v>1.061</v>
       </c>
       <c r="E18" t="n">
-        <v>1.0459</v>
+        <v>1.048</v>
       </c>
       <c r="F18" t="n">
-        <v>1.0554</v>
+        <v>1.0741</v>
       </c>
       <c r="G18" t="n">
-        <v>34.8533</v>
+        <v>34.5166</v>
       </c>
       <c r="H18" t="n">
-        <v>2.6</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_b10o1</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -959,25 +959,25 @@
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>1.0432</v>
+        <v>1.0608</v>
       </c>
       <c r="E19" t="n">
-        <v>1.0376</v>
+        <v>1.0578</v>
       </c>
       <c r="F19" t="n">
-        <v>1.0488</v>
+        <v>1.0639</v>
       </c>
       <c r="G19" t="n">
-        <v>35.1022</v>
+        <v>34.5166</v>
       </c>
       <c r="H19" t="n">
-        <v>2.9</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>avg_g_window_hg</t>
+          <t>band_g_mix_b5o2</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -987,53 +987,53 @@
         <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>1.0301</v>
+        <v>1.0579</v>
       </c>
       <c r="E20" t="n">
-        <v>1.0294</v>
+        <v>1.0546</v>
       </c>
       <c r="F20" t="n">
-        <v>1.0308</v>
+        <v>1.0612</v>
       </c>
       <c r="G20" t="n">
-        <v>35.5482</v>
+        <v>34.6135</v>
       </c>
       <c r="H20" t="n">
-        <v>2.55</v>
+        <v>4.05</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>band_g_mix_s3</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>60</v>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>1.0292</v>
+        <v>1.0553</v>
       </c>
       <c r="E21" t="n">
-        <v>1.0039</v>
+        <v>1.0346</v>
       </c>
       <c r="F21" t="n">
-        <v>1.066</v>
+        <v>1.076</v>
       </c>
       <c r="G21" t="n">
-        <v>35.6013</v>
+        <v>34.7125</v>
       </c>
       <c r="H21" t="n">
-        <v>0.8</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>avg_g_window_stock</t>
+          <t>band_gy_dyn</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1043,51 +1043,53 @@
         <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>1.029</v>
+        <v>1.0506</v>
       </c>
       <c r="E22" t="n">
-        <v>1.026</v>
+        <v>1.0459</v>
       </c>
       <c r="F22" t="n">
-        <v>1.0319</v>
+        <v>1.0554</v>
       </c>
       <c r="G22" t="n">
-        <v>35.5875</v>
-      </c>
-      <c r="H22" t="inlineStr"/>
+        <v>34.8533</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2.6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1_s3</t>
+          <t>band_g_mix_s1</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>60</v>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>1.0233</v>
+        <v>1.0432</v>
       </c>
       <c r="E23" t="n">
-        <v>1.0165</v>
+        <v>1.0376</v>
       </c>
       <c r="F23" t="n">
-        <v>1.0395</v>
+        <v>1.0488</v>
       </c>
       <c r="G23" t="n">
-        <v>35.7888</v>
+        <v>35.1022</v>
       </c>
       <c r="H23" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>baseline_hg</t>
+          <t>avg_g_window_hg</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1097,109 +1099,107 @@
         <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>1.0162</v>
+        <v>1.0301</v>
       </c>
       <c r="E24" t="n">
-        <v>1.0147</v>
+        <v>1.0294</v>
       </c>
       <c r="F24" t="n">
-        <v>1.0177</v>
+        <v>1.0308</v>
       </c>
       <c r="G24" t="n">
-        <v>36.0347</v>
+        <v>35.5482</v>
       </c>
       <c r="H24" t="n">
-        <v>3</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>baseline FORCE_CMD=1.0</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>60</v>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D25" t="n">
-        <v>1.0017</v>
+        <v>1.0292</v>
       </c>
       <c r="E25" t="n">
-        <v>1.0017</v>
+        <v>1.0039</v>
       </c>
       <c r="F25" t="n">
-        <v>1.0017</v>
+        <v>1.066</v>
       </c>
       <c r="G25" t="n">
-        <v>36.5572</v>
+        <v>35.6013</v>
       </c>
       <c r="H25" t="n">
-        <v>3.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>baseline_stocknorpm</t>
+          <t>avg_g_window_stock</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>60</v>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.029</v>
       </c>
       <c r="E26" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.026</v>
       </c>
       <c r="F26" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.0319</v>
       </c>
       <c r="G26" t="n">
-        <v>37.0845</v>
-      </c>
-      <c r="H26" t="n">
-        <v>1</v>
-      </c>
+        <v>35.5875</v>
+      </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>baseline_stock</t>
+          <t>band_g_mix_b1o1_s3</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>60</v>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D27" t="n">
-        <v>0.8937</v>
+        <v>1.0233</v>
       </c>
       <c r="E27" t="n">
-        <v>0.8933</v>
+        <v>1.0165</v>
       </c>
       <c r="F27" t="n">
-        <v>0.8942</v>
+        <v>1.0395</v>
       </c>
       <c r="G27" t="n">
-        <v>40.9724</v>
+        <v>35.7888</v>
       </c>
       <c r="H27" t="n">
-        <v>3.5667</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>curation_hg</t>
+          <t>baseline_hg</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1209,51 +1209,53 @@
         <v>2</v>
       </c>
       <c r="D28" t="n">
-        <v>0.8874</v>
+        <v>1.0162</v>
       </c>
       <c r="E28" t="n">
-        <v>0.8813</v>
+        <v>1.0147</v>
       </c>
       <c r="F28" t="n">
-        <v>0.8935</v>
+        <v>1.0177</v>
       </c>
       <c r="G28" t="n">
-        <v>41.266</v>
-      </c>
-      <c r="H28" t="inlineStr"/>
+        <v>36.0347</v>
+      </c>
+      <c r="H28" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs2</t>
+          <t>baseline FORCE_CMD=1.0</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>60</v>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>0.8228</v>
+        <v>1.0017</v>
       </c>
       <c r="E29" t="n">
-        <v>0.8045</v>
+        <v>1.0017</v>
       </c>
       <c r="F29" t="n">
-        <v>0.8411</v>
+        <v>1.0017</v>
       </c>
       <c r="G29" t="n">
-        <v>44.527</v>
+        <v>36.5572</v>
       </c>
       <c r="H29" t="n">
-        <v>1.9</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>baseline_stock16</t>
+          <t>baseline_stocknorpm</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1263,79 +1265,79 @@
         <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>0.7467</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="E30" t="n">
-        <v>0.7467</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="F30" t="n">
-        <v>0.7467</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="G30" t="n">
-        <v>49.0416</v>
-      </c>
-      <c r="H30" t="inlineStr"/>
+        <v>37.0845</v>
+      </c>
+      <c r="H30" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>band_g_mix_b20o1</t>
+          <t>baseline_stock</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>60</v>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>0.7231</v>
+        <v>0.8937</v>
       </c>
       <c r="E31" t="n">
-        <v>0.4061</v>
+        <v>0.8933</v>
       </c>
       <c r="F31" t="n">
-        <v>1.0401</v>
+        <v>0.8942</v>
       </c>
       <c r="G31" t="n">
-        <v>62.6864</v>
+        <v>40.9724</v>
       </c>
       <c r="H31" t="n">
-        <v>1.95</v>
+        <v>3.5667</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>curation_hg</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>60</v>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
-        <v>0.4106</v>
+        <v>0.8874</v>
       </c>
       <c r="E32" t="n">
-        <v>0.2278</v>
+        <v>0.8813</v>
       </c>
       <c r="F32" t="n">
-        <v>0.7759</v>
+        <v>0.8935</v>
       </c>
       <c r="G32" t="n">
-        <v>122.7889</v>
-      </c>
-      <c r="H32" t="n">
-        <v>2.1</v>
-      </c>
+        <v>41.266</v>
+      </c>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>baseline_dynnoimu</t>
+          <t>baseline_dynstocknoabs2</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1345,53 +1347,51 @@
         <v>2</v>
       </c>
       <c r="D33" t="n">
-        <v>0.3672</v>
+        <v>0.8228</v>
       </c>
       <c r="E33" t="n">
-        <v>0.3661</v>
+        <v>0.8045</v>
       </c>
       <c r="F33" t="n">
-        <v>0.3683</v>
+        <v>0.8411</v>
       </c>
       <c r="G33" t="n">
-        <v>99.72539999999999</v>
+        <v>44.527</v>
       </c>
       <c r="H33" t="n">
-        <v>4.6</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>baseline_dynstock2</t>
+          <t>baseline_stock16</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>60</v>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>0.2488</v>
+        <v>0.7467</v>
       </c>
       <c r="E34" t="n">
-        <v>0.2481</v>
+        <v>0.7467</v>
       </c>
       <c r="F34" t="n">
-        <v>0.2496</v>
+        <v>0.7467</v>
       </c>
       <c r="G34" t="n">
-        <v>147.1485</v>
-      </c>
-      <c r="H34" t="n">
-        <v>2.8</v>
-      </c>
+        <v>49.0416</v>
+      </c>
+      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>band_g_mix_b20o1</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1401,23 +1401,25 @@
         <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>0.2302</v>
+        <v>0.7231</v>
       </c>
       <c r="E35" t="n">
-        <v>0.2295</v>
+        <v>0.4061</v>
       </c>
       <c r="F35" t="n">
-        <v>0.2309</v>
+        <v>1.0401</v>
       </c>
       <c r="G35" t="n">
-        <v>159.0684</v>
-      </c>
-      <c r="H35" t="inlineStr"/>
+        <v>62.6864</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1.95</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>avg_g_window</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1427,25 +1429,25 @@
         <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>0.2283</v>
+        <v>0.4106</v>
       </c>
       <c r="E36" t="n">
-        <v>0.2276</v>
+        <v>0.2278</v>
       </c>
       <c r="F36" t="n">
-        <v>0.2291</v>
+        <v>0.7759</v>
       </c>
       <c r="G36" t="n">
-        <v>160.3908</v>
+        <v>122.7889</v>
       </c>
       <c r="H36" t="n">
-        <v>3.2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>baseline_dynnoimu</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1455,23 +1457,25 @@
         <v>2</v>
       </c>
       <c r="D37" t="n">
-        <v>0.2258</v>
+        <v>0.3672</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2252</v>
+        <v>0.3661</v>
       </c>
       <c r="F37" t="n">
-        <v>0.2263</v>
+        <v>0.3683</v>
       </c>
       <c r="G37" t="n">
-        <v>162.2099</v>
-      </c>
-      <c r="H37" t="inlineStr"/>
+        <v>99.72539999999999</v>
+      </c>
+      <c r="H37" t="n">
+        <v>4.6</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>peak_g_norpm</t>
+          <t>baseline_dynstock2</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1481,23 +1485,25 @@
         <v>2</v>
       </c>
       <c r="D38" t="n">
-        <v>0.2245</v>
+        <v>0.2488</v>
       </c>
       <c r="E38" t="n">
-        <v>0.2238</v>
+        <v>0.2481</v>
       </c>
       <c r="F38" t="n">
-        <v>0.2252</v>
+        <v>0.2496</v>
       </c>
       <c r="G38" t="n">
-        <v>163.1152</v>
-      </c>
-      <c r="H38" t="inlineStr"/>
+        <v>147.1485</v>
+      </c>
+      <c r="H38" t="n">
+        <v>2.8</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>baseline_dynstock</t>
+          <t>peak_g</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1507,185 +1513,187 @@
         <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2241</v>
+        <v>0.2302</v>
       </c>
       <c r="E39" t="n">
-        <v>0.2235</v>
+        <v>0.2295</v>
       </c>
       <c r="F39" t="n">
-        <v>0.2247</v>
+        <v>0.2309</v>
       </c>
       <c r="G39" t="n">
-        <v>163.3969</v>
-      </c>
-      <c r="H39" t="n">
-        <v>3.05</v>
-      </c>
+        <v>159.0684</v>
+      </c>
+      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs</t>
+          <t>avg_g_window</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>60</v>
       </c>
       <c r="C40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D40" t="n">
-        <v>0.1982</v>
+        <v>0.2283</v>
       </c>
       <c r="E40" t="n">
-        <v>0.198</v>
+        <v>0.2276</v>
       </c>
       <c r="F40" t="n">
-        <v>0.1985</v>
+        <v>0.2291</v>
       </c>
       <c r="G40" t="n">
-        <v>184.7105</v>
+        <v>160.3908</v>
       </c>
       <c r="H40" t="n">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>avg_g_window_hg</t>
+          <t>yaw_intent</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D41" t="n">
-        <v>1.0148</v>
+        <v>0.2258</v>
       </c>
       <c r="E41" t="n">
-        <v>1.0148</v>
+        <v>0.2252</v>
       </c>
       <c r="F41" t="n">
-        <v>1.0148</v>
+        <v>0.2263</v>
       </c>
       <c r="G41" t="n">
-        <v>64.18680000000001</v>
-      </c>
-      <c r="H41" t="n">
-        <v>3.8</v>
-      </c>
+        <v>162.2099</v>
+      </c>
+      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>peak_g_norpm</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C42" t="n">
         <v>2</v>
       </c>
       <c r="D42" t="n">
-        <v>1.011</v>
+        <v>0.2245</v>
       </c>
       <c r="E42" t="n">
-        <v>1.0062</v>
+        <v>0.2238</v>
       </c>
       <c r="F42" t="n">
-        <v>1.0158</v>
+        <v>0.2252</v>
       </c>
       <c r="G42" t="n">
-        <v>50.3918</v>
+        <v>163.1152</v>
       </c>
       <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>baseline_dynstock</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D43" t="n">
-        <v>0.9869</v>
+        <v>0.2241</v>
       </c>
       <c r="E43" t="n">
-        <v>0.9869</v>
+        <v>0.2235</v>
       </c>
       <c r="F43" t="n">
-        <v>0.9869</v>
+        <v>0.2247</v>
       </c>
       <c r="G43" t="n">
-        <v>66.0052</v>
-      </c>
-      <c r="H43" t="inlineStr"/>
+        <v>163.3969</v>
+      </c>
+      <c r="H43" t="n">
+        <v>3.05</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>combined</t>
+          <t>baseline_dynstocknoabs</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D44" t="n">
-        <v>0.2276</v>
+        <v>0.1982</v>
       </c>
       <c r="E44" t="n">
-        <v>0.2276</v>
+        <v>0.198</v>
       </c>
       <c r="F44" t="n">
-        <v>0.2276</v>
+        <v>0.1985</v>
       </c>
       <c r="G44" t="n">
-        <v>160.9226</v>
-      </c>
-      <c r="H44" t="inlineStr"/>
+        <v>184.7105</v>
+      </c>
+      <c r="H44" t="n">
+        <v>3.75</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>avg_g_window_hg</t>
         </is>
       </c>
       <c r="B45" t="n">
         <v>80</v>
       </c>
       <c r="C45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>0.2159</v>
+        <v>1.0148</v>
       </c>
       <c r="E45" t="n">
-        <v>0.2156</v>
+        <v>1.0148</v>
       </c>
       <c r="F45" t="n">
-        <v>0.2162</v>
+        <v>1.0148</v>
       </c>
       <c r="G45" t="n">
-        <v>301.7328</v>
-      </c>
-      <c r="H45" t="inlineStr"/>
+        <v>64.18680000000001</v>
+      </c>
+      <c r="H45" t="n">
+        <v>3.8</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1695,70 +1703,174 @@
         <v>2</v>
       </c>
       <c r="D46" t="n">
-        <v>0.1782</v>
+        <v>1.011</v>
       </c>
       <c r="E46" t="n">
-        <v>0.1779</v>
+        <v>1.0062</v>
       </c>
       <c r="F46" t="n">
-        <v>0.1784</v>
+        <v>1.0158</v>
       </c>
       <c r="G46" t="n">
-        <v>365.637</v>
+        <v>50.3918</v>
       </c>
       <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>avg_g_window</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>80</v>
       </c>
       <c r="C47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>0.1778</v>
+        <v>0.9869</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1776</v>
+        <v>0.9869</v>
       </c>
       <c r="F47" t="n">
-        <v>0.178</v>
+        <v>0.9869</v>
       </c>
       <c r="G47" t="n">
-        <v>366.3356</v>
+        <v>66.0052</v>
       </c>
       <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>combined</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>80</v>
       </c>
       <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.2276</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.2276</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.2276</v>
+      </c>
+      <c r="G48" t="n">
+        <v>160.9226</v>
+      </c>
+      <c r="H48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>80</v>
+      </c>
+      <c r="C49" t="n">
         <v>2</v>
       </c>
-      <c r="D48" t="n">
+      <c r="D49" t="n">
+        <v>0.2159</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.2156</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.2162</v>
+      </c>
+      <c r="G49" t="n">
+        <v>301.7328</v>
+      </c>
+      <c r="H49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>peak_g</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>80</v>
+      </c>
+      <c r="C50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0.1782</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.1779</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.1784</v>
+      </c>
+      <c r="G50" t="n">
+        <v>365.637</v>
+      </c>
+      <c r="H50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>avg_g_window</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>80</v>
+      </c>
+      <c r="C51" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.1778</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.1776</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="G51" t="n">
+        <v>366.3356</v>
+      </c>
+      <c r="H51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>yaw_intent</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>80</v>
+      </c>
+      <c r="C52" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" t="n">
         <v>0.1766</v>
       </c>
-      <c r="E48" t="n">
+      <c r="E52" t="n">
         <v>0.1766</v>
       </c>
-      <c r="F48" t="n">
+      <c r="F52" t="n">
         <v>0.1766</v>
       </c>
-      <c r="G48" t="n">
+      <c r="G52" t="n">
         <v>368.9042</v>
       </c>
-      <c r="H48" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1771,7 +1883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J107"/>
+  <dimension ref="A1:J121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4604,36 +4716,36 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>bandsweep</t>
+          <t>lockweight</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>band_g_mix_b10o1</t>
+          <t>band_g_mix</t>
         </is>
       </c>
       <c r="D79" t="n">
         <v>60</v>
       </c>
       <c r="E79" t="n">
-        <v>1.0639</v>
+        <v>1.1135</v>
       </c>
       <c r="F79" t="n">
-        <v>34.4174</v>
+        <v>32.8853</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>1788404082-0009</t>
+          <t>1788409274-0005</t>
         </is>
       </c>
       <c r="H79" t="n">
-        <v>34.42</v>
+        <v>32.89</v>
       </c>
       <c r="I79" t="n">
-        <v>2.8</v>
+        <v>3.3</v>
       </c>
       <c r="J79" t="n">
-        <v>2.47</v>
+        <v>2.37</v>
       </c>
     </row>
     <row r="80">
@@ -4644,36 +4756,36 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>bandsweep</t>
+          <t>lockweight</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>band_g_mix_b10o1</t>
+          <t>band_g_mix</t>
         </is>
       </c>
       <c r="D80" t="n">
         <v>60</v>
       </c>
       <c r="E80" t="n">
-        <v>1.0578</v>
+        <v>1.0904</v>
       </c>
       <c r="F80" t="n">
-        <v>34.6159</v>
+        <v>33.5831</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>1788404114-0010</t>
+          <t>1788409307-0006</t>
         </is>
       </c>
       <c r="H80" t="n">
-        <v>34.62</v>
+        <v>33.59</v>
       </c>
       <c r="I80" t="n">
-        <v>2</v>
+        <v>4.1</v>
       </c>
       <c r="J80" t="n">
-        <v>2.48</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="81">
@@ -4689,31 +4801,31 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1</t>
+          <t>band_g_mix_b10o1</t>
         </is>
       </c>
       <c r="D81" t="n">
         <v>60</v>
       </c>
       <c r="E81" t="n">
-        <v>1.0902</v>
+        <v>1.0639</v>
       </c>
       <c r="F81" t="n">
-        <v>33.5875</v>
+        <v>34.4174</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>1788403804-0001</t>
+          <t>1788404082-0009</t>
         </is>
       </c>
       <c r="H81" t="n">
-        <v>33.59</v>
+        <v>34.42</v>
       </c>
       <c r="I81" t="n">
-        <v>1.6</v>
+        <v>2.8</v>
       </c>
       <c r="J81" t="n">
-        <v>2.62</v>
+        <v>2.47</v>
       </c>
     </row>
     <row r="82">
@@ -4729,31 +4841,31 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1</t>
+          <t>band_g_mix_b10o1</t>
         </is>
       </c>
       <c r="D82" t="n">
         <v>60</v>
       </c>
       <c r="E82" t="n">
-        <v>1.1133</v>
+        <v>1.0578</v>
       </c>
       <c r="F82" t="n">
-        <v>32.8921</v>
+        <v>34.6159</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>1788403836-0002</t>
+          <t>1788404114-0010</t>
         </is>
       </c>
       <c r="H82" t="n">
-        <v>32.89</v>
+        <v>34.62</v>
       </c>
       <c r="I82" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="J82" t="n">
-        <v>2.55</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="83">
@@ -4764,31 +4876,37 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>pairedseeds</t>
+          <t>bandsweep</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1_s1</t>
+          <t>band_g_mix_b1o1</t>
         </is>
       </c>
       <c r="D83" t="n">
         <v>60</v>
       </c>
       <c r="E83" t="n">
-        <v>1.0684</v>
+        <v>1.0902</v>
       </c>
       <c r="F83" t="n">
-        <v>34.2738</v>
+        <v>33.5875</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>1788406434-0001</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
+          <t>1788403804-0001</t>
+        </is>
+      </c>
+      <c r="H83" t="n">
+        <v>33.59</v>
+      </c>
+      <c r="I83" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J83" t="n">
+        <v>2.62</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4798,36 +4916,36 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>pairedseeds</t>
+          <t>bandsweep</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1_s1</t>
+          <t>band_g_mix_b1o1</t>
         </is>
       </c>
       <c r="D84" t="n">
         <v>60</v>
       </c>
       <c r="E84" t="n">
-        <v>1.0722</v>
+        <v>1.1133</v>
       </c>
       <c r="F84" t="n">
-        <v>34.1511</v>
+        <v>32.8921</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>1788406467-0002</t>
+          <t>1788403836-0002</t>
         </is>
       </c>
       <c r="H84" t="n">
-        <v>34.15</v>
+        <v>32.89</v>
       </c>
       <c r="I84" t="n">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="J84" t="n">
-        <v>2.44</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="85">
@@ -4843,32 +4961,26 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1_s2</t>
+          <t>band_g_mix_b1o1_s1</t>
         </is>
       </c>
       <c r="D85" t="n">
         <v>60</v>
       </c>
       <c r="E85" t="n">
-        <v>1.1391</v>
+        <v>1.0684</v>
       </c>
       <c r="F85" t="n">
-        <v>32.146</v>
+        <v>34.2738</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>1788406503-0003</t>
-        </is>
-      </c>
-      <c r="H85" t="n">
-        <v>32.15</v>
-      </c>
-      <c r="I85" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="J85" t="n">
-        <v>2.35</v>
-      </c>
+          <t>1788406434-0001</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4883,31 +4995,31 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1_s2</t>
+          <t>band_g_mix_b1o1_s1</t>
         </is>
       </c>
       <c r="D86" t="n">
         <v>60</v>
       </c>
       <c r="E86" t="n">
-        <v>1.1556</v>
+        <v>1.0722</v>
       </c>
       <c r="F86" t="n">
-        <v>31.6868</v>
+        <v>34.1511</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>1788406537-0004</t>
+          <t>1788406467-0002</t>
         </is>
       </c>
       <c r="H86" t="n">
-        <v>31.69</v>
+        <v>34.15</v>
       </c>
       <c r="I86" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="J86" t="n">
-        <v>2.31</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="87">
@@ -4923,26 +5035,32 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1_s3</t>
+          <t>band_g_mix_b1o1_s2</t>
         </is>
       </c>
       <c r="D87" t="n">
         <v>60</v>
       </c>
       <c r="E87" t="n">
-        <v>1.0395</v>
+        <v>1.1391</v>
       </c>
       <c r="F87" t="n">
-        <v>35.2276</v>
+        <v>32.146</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>1788405673-0002</t>
-        </is>
-      </c>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
+          <t>1788406503-0003</t>
+        </is>
+      </c>
+      <c r="H87" t="n">
+        <v>32.15</v>
+      </c>
+      <c r="I87" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="J87" t="n">
+        <v>2.35</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4957,31 +5075,31 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1_s3</t>
+          <t>band_g_mix_b1o1_s2</t>
         </is>
       </c>
       <c r="D88" t="n">
         <v>60</v>
       </c>
       <c r="E88" t="n">
-        <v>1.0168</v>
+        <v>1.1556</v>
       </c>
       <c r="F88" t="n">
-        <v>36.0148</v>
+        <v>31.6868</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>1788405701-0001</t>
+          <t>1788406537-0004</t>
         </is>
       </c>
       <c r="H88" t="n">
-        <v>36.01</v>
+        <v>31.69</v>
       </c>
       <c r="I88" t="n">
-        <v>3.2</v>
+        <v>1.8</v>
       </c>
       <c r="J88" t="n">
-        <v>2.56</v>
+        <v>2.31</v>
       </c>
     </row>
     <row r="89">
@@ -5004,14 +5122,14 @@
         <v>60</v>
       </c>
       <c r="E89" t="n">
-        <v>1.0165</v>
+        <v>1.0395</v>
       </c>
       <c r="F89" t="n">
-        <v>36.0244</v>
+        <v>35.2276</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>1788406573-0005</t>
+          <t>1788405673-0002</t>
         </is>
       </c>
       <c r="H89" t="inlineStr"/>
@@ -5038,19 +5156,25 @@
         <v>60</v>
       </c>
       <c r="E90" t="n">
-        <v>1.0203</v>
+        <v>1.0168</v>
       </c>
       <c r="F90" t="n">
-        <v>35.8884</v>
+        <v>36.0148</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>1788406606-0006</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
+          <t>1788405701-0001</t>
+        </is>
+      </c>
+      <c r="H90" t="n">
+        <v>36.01</v>
+      </c>
+      <c r="I90" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J90" t="n">
+        <v>2.56</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5060,37 +5184,31 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>bandsweep</t>
+          <t>pairedseeds</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>band_g_mix_b20o1</t>
+          <t>band_g_mix_b1o1_s3</t>
         </is>
       </c>
       <c r="D91" t="n">
         <v>60</v>
       </c>
       <c r="E91" t="n">
-        <v>0.4061</v>
+        <v>1.0165</v>
       </c>
       <c r="F91" t="n">
-        <v>90.16759999999999</v>
+        <v>36.0244</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>1788404151-0011</t>
-        </is>
-      </c>
-      <c r="H91" t="n">
-        <v>90.17</v>
-      </c>
-      <c r="I91" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="J91" t="n">
-        <v>5.28</v>
-      </c>
+          <t>1788406573-0005</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5100,37 +5218,31 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>bandsweep</t>
+          <t>pairedseeds</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>band_g_mix_b20o1</t>
+          <t>band_g_mix_b1o1_s3</t>
         </is>
       </c>
       <c r="D92" t="n">
         <v>60</v>
       </c>
       <c r="E92" t="n">
-        <v>1.0401</v>
+        <v>1.0203</v>
       </c>
       <c r="F92" t="n">
-        <v>35.2051</v>
+        <v>35.8884</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>1788404187-0012</t>
-        </is>
-      </c>
-      <c r="H92" t="n">
-        <v>35.21</v>
-      </c>
-      <c r="I92" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="J92" t="n">
-        <v>2.55</v>
-      </c>
+          <t>1788406606-0006</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5145,31 +5257,31 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>band_g_mix_b2p5o2</t>
+          <t>band_g_mix_b20o1</t>
         </is>
       </c>
       <c r="D93" t="n">
         <v>60</v>
       </c>
       <c r="E93" t="n">
-        <v>1.0823</v>
+        <v>0.4061</v>
       </c>
       <c r="F93" t="n">
-        <v>33.8327</v>
+        <v>90.16759999999999</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>1788403874-0003</t>
+          <t>1788404151-0011</t>
         </is>
       </c>
       <c r="H93" t="n">
-        <v>33.83</v>
+        <v>90.17</v>
       </c>
       <c r="I93" t="n">
-        <v>1.5</v>
+        <v>2.6</v>
       </c>
       <c r="J93" t="n">
-        <v>2.47</v>
+        <v>5.28</v>
       </c>
     </row>
     <row r="94">
@@ -5185,31 +5297,31 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>band_g_mix_b2p5o2</t>
+          <t>band_g_mix_b20o1</t>
         </is>
       </c>
       <c r="D94" t="n">
         <v>60</v>
       </c>
       <c r="E94" t="n">
-        <v>1.0944</v>
+        <v>1.0401</v>
       </c>
       <c r="F94" t="n">
-        <v>33.4601</v>
+        <v>35.2051</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>1788403907-0004</t>
+          <t>1788404187-0012</t>
         </is>
       </c>
       <c r="H94" t="n">
-        <v>33.46</v>
+        <v>35.21</v>
       </c>
       <c r="I94" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
       <c r="J94" t="n">
-        <v>2.45</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="95">
@@ -5225,31 +5337,31 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>band_g_mix_b5o2</t>
+          <t>band_g_mix_b2p5o2</t>
         </is>
       </c>
       <c r="D95" t="n">
         <v>60</v>
       </c>
       <c r="E95" t="n">
-        <v>1.0612</v>
+        <v>1.0823</v>
       </c>
       <c r="F95" t="n">
-        <v>34.5049</v>
+        <v>33.8327</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>1788403944-0005</t>
+          <t>1788403874-0003</t>
         </is>
       </c>
       <c r="H95" t="n">
-        <v>34.51</v>
+        <v>33.83</v>
       </c>
       <c r="I95" t="n">
-        <v>3.2</v>
+        <v>1.5</v>
       </c>
       <c r="J95" t="n">
-        <v>2.48</v>
+        <v>2.47</v>
       </c>
     </row>
     <row r="96">
@@ -5265,31 +5377,31 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>band_g_mix_b5o2</t>
+          <t>band_g_mix_b2p5o2</t>
         </is>
       </c>
       <c r="D96" t="n">
         <v>60</v>
       </c>
       <c r="E96" t="n">
-        <v>1.0546</v>
+        <v>1.0944</v>
       </c>
       <c r="F96" t="n">
-        <v>34.7221</v>
+        <v>33.4601</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>1788403976-0006</t>
+          <t>1788403907-0004</t>
         </is>
       </c>
       <c r="H96" t="n">
-        <v>34.72</v>
+        <v>33.46</v>
       </c>
       <c r="I96" t="n">
-        <v>4.9</v>
+        <v>1.6</v>
       </c>
       <c r="J96" t="n">
-        <v>2.49</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="97">
@@ -5305,31 +5417,31 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>band_g_mix_b7p5o3</t>
+          <t>band_g_mix_b5o2</t>
         </is>
       </c>
       <c r="D97" t="n">
         <v>60</v>
       </c>
       <c r="E97" t="n">
-        <v>1.048</v>
+        <v>1.0612</v>
       </c>
       <c r="F97" t="n">
-        <v>34.9402</v>
+        <v>34.5049</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>1788404012-0007</t>
+          <t>1788403944-0005</t>
         </is>
       </c>
       <c r="H97" t="n">
-        <v>34.94</v>
+        <v>34.51</v>
       </c>
       <c r="I97" t="n">
-        <v>1.5</v>
+        <v>3.2</v>
       </c>
       <c r="J97" t="n">
-        <v>2.6</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="98">
@@ -5345,31 +5457,31 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>band_g_mix_b7p5o3</t>
+          <t>band_g_mix_b5o2</t>
         </is>
       </c>
       <c r="D98" t="n">
         <v>60</v>
       </c>
       <c r="E98" t="n">
-        <v>1.0741</v>
+        <v>1.0546</v>
       </c>
       <c r="F98" t="n">
-        <v>34.0931</v>
+        <v>34.7221</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>1788404045-0008</t>
+          <t>1788403976-0006</t>
         </is>
       </c>
       <c r="H98" t="n">
-        <v>34.09</v>
+        <v>34.72</v>
       </c>
       <c r="I98" t="n">
-        <v>1.4</v>
+        <v>4.9</v>
       </c>
       <c r="J98" t="n">
-        <v>2.41</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="99">
@@ -5380,36 +5492,36 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ensemble</t>
+          <t>bandsweep</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_b7p5o3</t>
         </is>
       </c>
       <c r="D99" t="n">
         <v>60</v>
       </c>
       <c r="E99" t="n">
-        <v>1.0488</v>
+        <v>1.048</v>
       </c>
       <c r="F99" t="n">
-        <v>34.9145</v>
+        <v>34.9402</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>1788401068-0005</t>
+          <t>1788404012-0007</t>
         </is>
       </c>
       <c r="H99" t="n">
-        <v>34.91</v>
+        <v>34.94</v>
       </c>
       <c r="I99" t="n">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="J99" t="n">
-        <v>2.48</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="100">
@@ -5420,36 +5532,36 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ensemble</t>
+          <t>bandsweep</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_b7p5o3</t>
         </is>
       </c>
       <c r="D100" t="n">
         <v>60</v>
       </c>
       <c r="E100" t="n">
-        <v>1.0376</v>
+        <v>1.0741</v>
       </c>
       <c r="F100" t="n">
-        <v>35.29</v>
+        <v>34.0931</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>1788401101-0006</t>
+          <t>1788404045-0008</t>
         </is>
       </c>
       <c r="H100" t="n">
-        <v>35.29</v>
+        <v>34.09</v>
       </c>
       <c r="I100" t="n">
-        <v>2.3</v>
+        <v>1.4</v>
       </c>
       <c r="J100" t="n">
-        <v>2.5</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="101">
@@ -5460,36 +5572,36 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>pairedseeds</t>
+          <t>lockweight</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>band_g_mix_s2</t>
+          <t>band_g_mix_lock</t>
         </is>
       </c>
       <c r="D101" t="n">
         <v>60</v>
       </c>
       <c r="E101" t="n">
-        <v>1.0923</v>
+        <v>1.1277</v>
       </c>
       <c r="F101" t="n">
-        <v>33.5239</v>
+        <v>32.4713</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>1788406643-0007</t>
+          <t>1788409135-0001</t>
         </is>
       </c>
       <c r="H101" t="n">
-        <v>33.53</v>
+        <v>32.47</v>
       </c>
       <c r="I101" t="n">
-        <v>4.9</v>
+        <v>1.5</v>
       </c>
       <c r="J101" t="n">
-        <v>2.42</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="102">
@@ -5500,31 +5612,37 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>pairedseeds</t>
+          <t>lockweight</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>band_g_mix_s2</t>
+          <t>band_g_mix_lock</t>
         </is>
       </c>
       <c r="D102" t="n">
         <v>60</v>
       </c>
       <c r="E102" t="n">
-        <v>1.0916</v>
+        <v>1.1072</v>
       </c>
       <c r="F102" t="n">
-        <v>33.5441</v>
+        <v>33.0721</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>1788406677-0008</t>
-        </is>
-      </c>
-      <c r="H102" t="inlineStr"/>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
+          <t>1788409168-0002</t>
+        </is>
+      </c>
+      <c r="H102" t="n">
+        <v>33.07</v>
+      </c>
+      <c r="I102" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J102" t="n">
+        <v>2.38</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5534,37 +5652,31 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>pairedseeds</t>
+          <t>slipyaw3</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>band_g_mix_s3</t>
+          <t>band_g_mix_lock</t>
         </is>
       </c>
       <c r="D103" t="n">
         <v>60</v>
       </c>
       <c r="E103" t="n">
-        <v>1.0346</v>
+        <v>1.1007</v>
       </c>
       <c r="F103" t="n">
-        <v>35.3941</v>
+        <v>33.2682</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>1788406714-0009</t>
-        </is>
-      </c>
-      <c r="H103" t="n">
-        <v>35.39</v>
-      </c>
-      <c r="I103" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="J103" t="n">
-        <v>2.53</v>
-      </c>
+          <t>1788412341-0003</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5574,36 +5686,36 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>pairedseeds</t>
+          <t>slipyaw3</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>band_g_mix_s3</t>
+          <t>band_g_mix_lock</t>
         </is>
       </c>
       <c r="D104" t="n">
         <v>60</v>
       </c>
       <c r="E104" t="n">
-        <v>1.076</v>
+        <v>1.0995</v>
       </c>
       <c r="F104" t="n">
-        <v>34.0309</v>
+        <v>33.3055</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>1788406747-0010</t>
+          <t>1788412373-0004</t>
         </is>
       </c>
       <c r="H104" t="n">
-        <v>34.03</v>
+        <v>33.31</v>
       </c>
       <c r="I104" t="n">
-        <v>1.1</v>
+        <v>4.5</v>
       </c>
       <c r="J104" t="n">
-        <v>2.56</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="105">
@@ -5614,36 +5726,36 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>restructure</t>
+          <t>slipyaw</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
+          <t>band_g_mix_lock_s</t>
         </is>
       </c>
       <c r="D105" t="n">
         <v>60</v>
       </c>
       <c r="E105" t="n">
-        <v>1.1085</v>
+        <v>1.0781</v>
       </c>
       <c r="F105" t="n">
-        <v>33.0351</v>
+        <v>33.9666</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>1788399311-0002</t>
+          <t>1788410563-0002</t>
         </is>
       </c>
       <c r="H105" t="n">
-        <v>33.04</v>
+        <v>33.97</v>
       </c>
       <c r="I105" t="n">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
       <c r="J105" t="n">
-        <v>2.4</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="106">
@@ -5654,33 +5766,33 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>ensemble</t>
+          <t>slipyaw</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ens_band_g_mix5</t>
+          <t>band_g_mix_lock_s</t>
         </is>
       </c>
       <c r="D106" t="n">
         <v>60</v>
       </c>
       <c r="E106" t="n">
-        <v>1.0736</v>
+        <v>1.0781</v>
       </c>
       <c r="F106" t="n">
-        <v>34.1079</v>
+        <v>33.9666</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>1788400929-0001</t>
+          <t>1788410563-0002</t>
         </is>
       </c>
       <c r="H106" t="n">
-        <v>34.11</v>
+        <v>33.97</v>
       </c>
       <c r="I106" t="n">
-        <v>2.4</v>
+        <v>3.9</v>
       </c>
       <c r="J106" t="n">
         <v>2.44</v>
@@ -5694,35 +5806,589 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
+          <t>slipyaw</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>band_g_mix_lock_s</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>60</v>
+      </c>
+      <c r="E107" t="n">
+        <v>1.0691</v>
+      </c>
+      <c r="F107" t="n">
+        <v>34.2528</v>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>1788410595-0003</t>
+        </is>
+      </c>
+      <c r="H107" t="n">
+        <v>34.25</v>
+      </c>
+      <c r="I107" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J107" t="n">
+        <v>2.45</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>slipyaw</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>band_g_mix_lock_s</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>60</v>
+      </c>
+      <c r="E108" t="n">
+        <v>1.0691</v>
+      </c>
+      <c r="F108" t="n">
+        <v>34.2528</v>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>1788410595-0003</t>
+        </is>
+      </c>
+      <c r="H108" t="n">
+        <v>34.25</v>
+      </c>
+      <c r="I108" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J108" t="n">
+        <v>2.45</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>slipyaw3</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>band_g_mix_lock_sy</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>60</v>
+      </c>
+      <c r="E109" t="n">
+        <v>1.1392</v>
+      </c>
+      <c r="F109" t="n">
+        <v>32.1429</v>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>1788412271-0001</t>
+        </is>
+      </c>
+      <c r="H109" t="n">
+        <v>32.14</v>
+      </c>
+      <c r="I109" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="J109" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>slipyaw3</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>band_g_mix_lock_sy</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>60</v>
+      </c>
+      <c r="E110" t="n">
+        <v>1.1464</v>
+      </c>
+      <c r="F110" t="n">
+        <v>31.9408</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>1788412304-0002</t>
+        </is>
+      </c>
+      <c r="H110" t="n">
+        <v>31.94</v>
+      </c>
+      <c r="I110" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J110" t="n">
+        <v>2.33</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
           <t>ensemble</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>band_g_mix_s1</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>60</v>
+      </c>
+      <c r="E111" t="n">
+        <v>1.0488</v>
+      </c>
+      <c r="F111" t="n">
+        <v>34.9145</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>1788401068-0005</t>
+        </is>
+      </c>
+      <c r="H111" t="n">
+        <v>34.91</v>
+      </c>
+      <c r="I111" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J111" t="n">
+        <v>2.48</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>band_g_mix_s1</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>60</v>
+      </c>
+      <c r="E112" t="n">
+        <v>1.0376</v>
+      </c>
+      <c r="F112" t="n">
+        <v>35.29</v>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>1788401101-0006</t>
+        </is>
+      </c>
+      <c r="H112" t="n">
+        <v>35.29</v>
+      </c>
+      <c r="I112" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J112" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>pairedseeds</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>band_g_mix_s2</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>60</v>
+      </c>
+      <c r="E113" t="n">
+        <v>1.0923</v>
+      </c>
+      <c r="F113" t="n">
+        <v>33.5239</v>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>1788406643-0007</t>
+        </is>
+      </c>
+      <c r="H113" t="n">
+        <v>33.53</v>
+      </c>
+      <c r="I113" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="J113" t="n">
+        <v>2.42</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>pairedseeds</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>band_g_mix_s2</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>60</v>
+      </c>
+      <c r="E114" t="n">
+        <v>1.0916</v>
+      </c>
+      <c r="F114" t="n">
+        <v>33.5441</v>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>1788406677-0008</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>pairedseeds</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>band_g_mix_s3</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>60</v>
+      </c>
+      <c r="E115" t="n">
+        <v>1.0346</v>
+      </c>
+      <c r="F115" t="n">
+        <v>35.3941</v>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>1788406714-0009</t>
+        </is>
+      </c>
+      <c r="H115" t="n">
+        <v>35.39</v>
+      </c>
+      <c r="I115" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J115" t="n">
+        <v>2.53</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>pairedseeds</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>band_g_mix_s3</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>60</v>
+      </c>
+      <c r="E116" t="n">
+        <v>1.076</v>
+      </c>
+      <c r="F116" t="n">
+        <v>34.0309</v>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>1788406747-0010</t>
+        </is>
+      </c>
+      <c r="H116" t="n">
+        <v>34.03</v>
+      </c>
+      <c r="I116" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J116" t="n">
+        <v>2.56</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>restructure</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>baseline_dyn</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>60</v>
+      </c>
+      <c r="E117" t="n">
+        <v>1.1085</v>
+      </c>
+      <c r="F117" t="n">
+        <v>33.0351</v>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>1788399311-0002</t>
+        </is>
+      </c>
+      <c r="H117" t="n">
+        <v>33.04</v>
+      </c>
+      <c r="I117" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="J117" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>lockweight</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>baseline_dyn_lock</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>60</v>
+      </c>
+      <c r="E118" t="n">
+        <v>1.0756</v>
+      </c>
+      <c r="F118" t="n">
+        <v>34.0434</v>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>1788409205-0003</t>
+        </is>
+      </c>
+      <c r="H118" t="n">
+        <v>34.04</v>
+      </c>
+      <c r="I118" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J118" t="n">
+        <v>2.45</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>lockweight</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>baseline_dyn_lock</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>60</v>
+      </c>
+      <c r="E119" t="n">
+        <v>1.0817</v>
+      </c>
+      <c r="F119" t="n">
+        <v>33.8519</v>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>1788409238-0004</t>
+        </is>
+      </c>
+      <c r="H119" t="n">
+        <v>33.85</v>
+      </c>
+      <c r="I119" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J119" t="n">
+        <v>2.43</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
         <is>
           <t>ens_band_g_mix5</t>
         </is>
       </c>
-      <c r="D107" t="n">
-        <v>60</v>
-      </c>
-      <c r="E107" t="n">
+      <c r="D120" t="n">
+        <v>60</v>
+      </c>
+      <c r="E120" t="n">
+        <v>1.0736</v>
+      </c>
+      <c r="F120" t="n">
+        <v>34.1079</v>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>1788400929-0001</t>
+        </is>
+      </c>
+      <c r="H120" t="n">
+        <v>34.11</v>
+      </c>
+      <c r="I120" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J120" t="n">
+        <v>2.44</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>ens_band_g_mix5</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>60</v>
+      </c>
+      <c r="E121" t="n">
         <v>1.0538</v>
       </c>
-      <c r="F107" t="n">
+      <c r="F121" t="n">
         <v>34.7482</v>
       </c>
-      <c r="G107" t="inlineStr">
+      <c r="G121" t="inlineStr">
         <is>
           <t>1788400962-0002</t>
         </is>
       </c>
-      <c r="H107" t="n">
+      <c r="H121" t="n">
         <v>34.75</v>
       </c>
-      <c r="I107" t="n">
+      <c r="I121" t="n">
         <v>2</v>
       </c>
-      <c r="J107" t="n">
+      <c r="J121" t="n">
         <v>2.48</v>
       </c>
     </row>
@@ -5737,7 +6403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -6455,7 +7121,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_lock</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6465,7 +7131,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-09-02T18:54:00</t>
+          <t>2026-09-02T21:16:23</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -6503,7 +7169,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>[0.14226, 0.15404, 0.16814, 0.16762]</t>
+          <t>[0.15058, 0.15519, 0.171, 0.17031]</t>
         </is>
       </c>
       <c r="N16" t="inlineStr"/>
@@ -6511,7 +7177,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>band_g_mix_s2</t>
+          <t>band_g_mix_lock_s</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6521,7 +7187,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-09-02T18:55:36</t>
+          <t>2026-09-02T21:26:40</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -6559,7 +7225,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>[0.15115, 0.15324, 0.16928, 0.16978]</t>
+          <t>[0.1511, 0.15729, 0.1708, 0.16893]</t>
         </is>
       </c>
       <c r="N17" t="inlineStr"/>
@@ -6567,7 +7233,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>band_g_mix_s3</t>
+          <t>band_g_mix_lock_sy</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -6577,7 +7243,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-09-02T18:57:18</t>
+          <t>2026-09-02T21:28:05</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -6615,7 +7281,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>[0.15575, 0.16054, 0.1713, 0.17144]</t>
+          <t>[0.15131, 0.15295, 0.1697, 0.16946]</t>
         </is>
       </c>
       <c r="N18" t="inlineStr"/>
@@ -6623,7 +7289,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>band_g_mix_s4</t>
+          <t>band_g_mix_s1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -6633,7 +7299,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-09-02T18:58:55</t>
+          <t>2026-09-02T18:54:00</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -6671,7 +7337,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>[0.14723, 0.15025, 0.16854, 0.16772]</t>
+          <t>[0.14226, 0.15404, 0.16814, 0.16762]</t>
         </is>
       </c>
       <c r="N19" t="inlineStr"/>
@@ -6679,7 +7345,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>band_g_mix_s5</t>
+          <t>band_g_mix_s2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -6689,7 +7355,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-09-02T19:00:42</t>
+          <t>2026-09-02T18:55:36</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -6727,7 +7393,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>[0.14491, 0.15532, 0.16904, 0.16805]</t>
+          <t>[0.15115, 0.15324, 0.16928, 0.16978]</t>
         </is>
       </c>
       <c r="N20" t="inlineStr"/>
@@ -6735,79 +7401,175 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>band_gy_dyn</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
+          <t>band_g_mix_s3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:57:18</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>5</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>[0.15575, 0.16054, 0.1713, 0.17144]</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>band_gy_mix</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
+          <t>band_g_mix_s4</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:58:55</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>5</v>
+      </c>
+      <c r="K22" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>[0.14723, 0.15025, 0.16854, 0.16772]</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>baseline</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
+          <t>band_g_mix_s5</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-09-02T19:00:42</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>5</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1</v>
+      </c>
+      <c r="L23" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>[0.14491, 0.15532, 0.16904, 0.16805]</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
+          <t>band_gy_dyn</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -6831,7 +7593,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>baseline_dynnoimu</t>
+          <t>band_gy_mix</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -6855,7 +7617,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>baseline_dynstock2</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -6879,7 +7641,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>baseline_dynstock</t>
+          <t>baseline_dyn</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -6903,31 +7665,63 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs2</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
+          <t>baseline_dyn_lock</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026-09-02T21:17:44</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>dyn_abs</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>5</v>
+      </c>
+      <c r="K28" t="n">
+        <v>1</v>
+      </c>
+      <c r="L28" t="n">
+        <v>1129</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>[0.13261, 0.15194, 0.08818, 0.08624]</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs</t>
+          <t>baseline_dynnoimu</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -6951,7 +7745,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>baseline_hg</t>
+          <t>baseline_dynstock2</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -6975,7 +7769,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>baseline_norpm</t>
+          <t>baseline_dynstock</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -6999,7 +7793,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>baseline_stock16</t>
+          <t>baseline_dynstocknoabs2</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -7023,7 +7817,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>baseline_dynstocknoabs</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -7047,7 +7841,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>baseline_stock</t>
+          <t>baseline_hg</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -7071,7 +7865,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>baseline_stocknorpm</t>
+          <t>baseline_norpm</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -7095,7 +7889,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>combined</t>
+          <t>baseline_stock16</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -7119,7 +7913,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -7143,7 +7937,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>curation_hg</t>
+          <t>baseline_stock</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -7167,7 +7961,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>baseline_stocknorpm</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -7191,7 +7985,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>peak_g_norpm</t>
+          <t>combined</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -7215,7 +8009,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -7236,6 +8030,102 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>curation_hg</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>peak_g</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>peak_g_norpm</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>yaw_intent</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
In-band slip retention weight (grip plateau 0.05-0.25 over a 100ms forward window), 3 seeds plus yaw combo
</commit_message>
<xml_diff>
--- a/results/LSTM_ABS_RESULTS.xlsx
+++ b/results/LSTM_ABS_RESULTS.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -613,63 +613,63 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
+          <t>band_g_mix_keep_s0</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>60</v>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>1.1232</v>
+        <v>1.1259</v>
       </c>
       <c r="E7" t="n">
-        <v>1.1085</v>
+        <v>1.1204</v>
       </c>
       <c r="F7" t="n">
-        <v>1.1351</v>
+        <v>1.1314</v>
       </c>
       <c r="G7" t="n">
-        <v>32.6046</v>
+        <v>32.5238</v>
       </c>
       <c r="H7" t="n">
-        <v>4.7</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>band_gy_mix</t>
+          <t>baseline_dyn</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>60</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D8" t="n">
-        <v>1.1219</v>
+        <v>1.1232</v>
       </c>
       <c r="E8" t="n">
-        <v>1.1198</v>
+        <v>1.1085</v>
       </c>
       <c r="F8" t="n">
-        <v>1.124</v>
+        <v>1.1351</v>
       </c>
       <c r="G8" t="n">
-        <v>32.6393</v>
+        <v>32.6046</v>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>band_g_mix_b1_sy_s2</t>
+          <t>band_gy_mix</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -679,25 +679,25 @@
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>1.12</v>
+        <v>1.1219</v>
       </c>
       <c r="E9" t="n">
-        <v>1.1184</v>
+        <v>1.1198</v>
       </c>
       <c r="F9" t="n">
-        <v>1.1215</v>
+        <v>1.124</v>
       </c>
       <c r="G9" t="n">
-        <v>32.6967</v>
+        <v>32.6393</v>
       </c>
       <c r="H9" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>band_g_mix_b1_sy_s0</t>
+          <t>band_g_mix_b1_sy_s2</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -707,79 +707,81 @@
         <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>1.1102</v>
+        <v>1.12</v>
       </c>
       <c r="E10" t="n">
-        <v>1.0997</v>
+        <v>1.1184</v>
       </c>
       <c r="F10" t="n">
-        <v>1.1207</v>
+        <v>1.1215</v>
       </c>
       <c r="G10" t="n">
-        <v>32.987</v>
+        <v>32.6967</v>
       </c>
       <c r="H10" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>band_g_mix_lock</t>
+          <t>band_g_mix_b1_sy_s0</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>60</v>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>1.1088</v>
+        <v>1.1102</v>
       </c>
       <c r="E11" t="n">
-        <v>1.0995</v>
+        <v>1.0997</v>
       </c>
       <c r="F11" t="n">
-        <v>1.1277</v>
+        <v>1.1207</v>
       </c>
       <c r="G11" t="n">
-        <v>33.0293</v>
+        <v>32.987</v>
       </c>
       <c r="H11" t="n">
-        <v>3.5</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s2</t>
+          <t>band_g_mix_lock</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>60</v>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D12" t="n">
-        <v>1.1067</v>
+        <v>1.1088</v>
       </c>
       <c r="E12" t="n">
-        <v>1.1048</v>
+        <v>1.0995</v>
       </c>
       <c r="F12" t="n">
-        <v>1.1085</v>
+        <v>1.1277</v>
       </c>
       <c r="G12" t="n">
-        <v>33.0898</v>
-      </c>
-      <c r="H12" t="inlineStr"/>
+        <v>33.0293</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_y</t>
+          <t>band_g_mix_lock_s2</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -789,25 +791,23 @@
         <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>1.1056</v>
+        <v>1.1067</v>
       </c>
       <c r="E13" t="n">
-        <v>1.1035</v>
+        <v>1.1048</v>
       </c>
       <c r="F13" t="n">
-        <v>1.1077</v>
+        <v>1.1085</v>
       </c>
       <c r="G13" t="n">
-        <v>33.1212</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1.7</v>
-      </c>
+        <v>33.0898</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>band_g_mix_b1_y_s0</t>
+          <t>band_g_mix_lock_y</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -817,25 +817,25 @@
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>1.1024</v>
+        <v>1.1056</v>
       </c>
       <c r="E14" t="n">
-        <v>1.0999</v>
+        <v>1.1035</v>
       </c>
       <c r="F14" t="n">
-        <v>1.1048</v>
+        <v>1.1077</v>
       </c>
       <c r="G14" t="n">
-        <v>33.2183</v>
+        <v>33.1212</v>
       </c>
       <c r="H14" t="n">
-        <v>1.45</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1</t>
+          <t>band_g_mix_keep_s2</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -845,25 +845,25 @@
         <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>1.1018</v>
+        <v>1.1047</v>
       </c>
       <c r="E15" t="n">
-        <v>1.0902</v>
+        <v>1.1017</v>
       </c>
       <c r="F15" t="n">
-        <v>1.1133</v>
+        <v>1.1077</v>
       </c>
       <c r="G15" t="n">
-        <v>33.2398</v>
+        <v>33.1475</v>
       </c>
       <c r="H15" t="n">
-        <v>1.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>band_g_mix_b1_y_s1</t>
+          <t>band_g_mix_b1_y_s0</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -873,23 +873,25 @@
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>1.0992</v>
+        <v>1.1024</v>
       </c>
       <c r="E16" t="n">
-        <v>1.0948</v>
+        <v>1.0999</v>
       </c>
       <c r="F16" t="n">
-        <v>1.1036</v>
+        <v>1.1048</v>
       </c>
       <c r="G16" t="n">
-        <v>33.3144</v>
-      </c>
-      <c r="H16" t="inlineStr"/>
+        <v>33.2183</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1.45</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s1</t>
+          <t>band_g_mix_b1o1</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -899,25 +901,25 @@
         <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>1.0984</v>
+        <v>1.1018</v>
       </c>
       <c r="E17" t="n">
-        <v>1.0895</v>
+        <v>1.0902</v>
       </c>
       <c r="F17" t="n">
-        <v>1.1072</v>
+        <v>1.1133</v>
       </c>
       <c r="G17" t="n">
-        <v>33.3413</v>
+        <v>33.2398</v>
       </c>
       <c r="H17" t="n">
-        <v>3.2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>band_g_mix_s2</t>
+          <t>band_g_mix_b1_y_s1</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -927,25 +929,23 @@
         <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>1.092</v>
+        <v>1.0992</v>
       </c>
       <c r="E18" t="n">
-        <v>1.0916</v>
+        <v>1.0948</v>
       </c>
       <c r="F18" t="n">
-        <v>1.0923</v>
+        <v>1.1036</v>
       </c>
       <c r="G18" t="n">
-        <v>33.534</v>
-      </c>
-      <c r="H18" t="n">
-        <v>4.9</v>
-      </c>
+        <v>33.3144</v>
+      </c>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>band_g_mix_b2p5o2</t>
+          <t>band_g_mix_lock_s1</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -955,25 +955,25 @@
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>1.0884</v>
+        <v>1.0984</v>
       </c>
       <c r="E19" t="n">
-        <v>1.0823</v>
+        <v>1.0895</v>
       </c>
       <c r="F19" t="n">
-        <v>1.0944</v>
+        <v>1.1072</v>
       </c>
       <c r="G19" t="n">
-        <v>33.6464</v>
+        <v>33.3413</v>
       </c>
       <c r="H19" t="n">
-        <v>1.55</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>band_g_mix_b1_sy_s1</t>
+          <t>band_g_mix_s2</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -983,23 +983,25 @@
         <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>1.0866</v>
+        <v>1.092</v>
       </c>
       <c r="E20" t="n">
-        <v>1.0848</v>
+        <v>1.0916</v>
       </c>
       <c r="F20" t="n">
-        <v>1.0884</v>
+        <v>1.0923</v>
       </c>
       <c r="G20" t="n">
-        <v>33.7008</v>
-      </c>
-      <c r="H20" t="inlineStr"/>
+        <v>33.534</v>
+      </c>
+      <c r="H20" t="n">
+        <v>4.9</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>baseline_dyn_lock</t>
+          <t>band_g_mix_b2p5o2</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1009,25 +1011,25 @@
         <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>1.0787</v>
+        <v>1.0884</v>
       </c>
       <c r="E21" t="n">
-        <v>1.0756</v>
+        <v>1.0823</v>
       </c>
       <c r="F21" t="n">
-        <v>1.0817</v>
+        <v>1.0944</v>
       </c>
       <c r="G21" t="n">
-        <v>33.9476</v>
+        <v>33.6464</v>
       </c>
       <c r="H21" t="n">
-        <v>4.4</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_sy_s2</t>
+          <t>band_g_mix_keepy_s0</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1037,51 +1039,51 @@
         <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>1.0742</v>
+        <v>1.0882</v>
       </c>
       <c r="E22" t="n">
-        <v>1.0712</v>
+        <v>1.0873</v>
       </c>
       <c r="F22" t="n">
-        <v>1.0771</v>
+        <v>1.0891</v>
       </c>
       <c r="G22" t="n">
-        <v>34.0912</v>
-      </c>
-      <c r="H22" t="inlineStr"/>
+        <v>33.6494</v>
+      </c>
+      <c r="H22" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s</t>
+          <t>band_g_mix_b1_sy_s1</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>60</v>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>1.0736</v>
+        <v>1.0866</v>
       </c>
       <c r="E23" t="n">
-        <v>1.0691</v>
+        <v>1.0848</v>
       </c>
       <c r="F23" t="n">
-        <v>1.0781</v>
+        <v>1.0884</v>
       </c>
       <c r="G23" t="n">
-        <v>34.1097</v>
-      </c>
-      <c r="H23" t="n">
-        <v>3.25</v>
-      </c>
+        <v>33.7008</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1_s1</t>
+          <t>baseline_dyn_lock</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1091,81 +1093,79 @@
         <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>1.0703</v>
+        <v>1.0787</v>
       </c>
       <c r="E24" t="n">
-        <v>1.0684</v>
+        <v>1.0756</v>
       </c>
       <c r="F24" t="n">
-        <v>1.0722</v>
+        <v>1.0817</v>
       </c>
       <c r="G24" t="n">
-        <v>34.2125</v>
+        <v>33.9476</v>
       </c>
       <c r="H24" t="n">
-        <v>2.1</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>band_g_mix_lock_sy_s2</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>60</v>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D25" t="n">
-        <v>1.0671</v>
+        <v>1.0742</v>
       </c>
       <c r="E25" t="n">
-        <v>1.0582</v>
+        <v>1.0712</v>
       </c>
       <c r="F25" t="n">
-        <v>1.0716</v>
+        <v>1.0771</v>
       </c>
       <c r="G25" t="n">
-        <v>34.3171</v>
-      </c>
-      <c r="H25" t="n">
-        <v>2.3667</v>
-      </c>
+        <v>34.0912</v>
+      </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ens_band_g_mix5</t>
+          <t>band_g_mix_lock_s</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>60</v>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D26" t="n">
-        <v>1.0637</v>
+        <v>1.0736</v>
       </c>
       <c r="E26" t="n">
-        <v>1.0538</v>
+        <v>1.0691</v>
       </c>
       <c r="F26" t="n">
-        <v>1.0736</v>
+        <v>1.0781</v>
       </c>
       <c r="G26" t="n">
-        <v>34.428</v>
+        <v>34.1097</v>
       </c>
       <c r="H26" t="n">
-        <v>2.2</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>band_g_dyn</t>
+          <t>band_g_mix_b1o1_s1</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1175,53 +1175,53 @@
         <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>1.0636</v>
+        <v>1.0703</v>
       </c>
       <c r="E27" t="n">
-        <v>1.0628</v>
+        <v>1.0684</v>
       </c>
       <c r="F27" t="n">
-        <v>1.0644</v>
+        <v>1.0722</v>
       </c>
       <c r="G27" t="n">
-        <v>34.4297</v>
+        <v>34.2125</v>
       </c>
       <c r="H27" t="n">
-        <v>4.15</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>band_g_mix_b7p5o3</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>60</v>
       </c>
       <c r="C28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>1.061</v>
+        <v>1.0671</v>
       </c>
       <c r="E28" t="n">
-        <v>1.048</v>
+        <v>1.0582</v>
       </c>
       <c r="F28" t="n">
-        <v>1.0741</v>
+        <v>1.0716</v>
       </c>
       <c r="G28" t="n">
-        <v>34.5166</v>
+        <v>34.3171</v>
       </c>
       <c r="H28" t="n">
-        <v>1.45</v>
+        <v>2.3667</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>band_g_mix_b10o1</t>
+          <t>ens_band_g_mix5</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1231,25 +1231,25 @@
         <v>2</v>
       </c>
       <c r="D29" t="n">
-        <v>1.0608</v>
+        <v>1.0637</v>
       </c>
       <c r="E29" t="n">
-        <v>1.0578</v>
+        <v>1.0538</v>
       </c>
       <c r="F29" t="n">
-        <v>1.0639</v>
+        <v>1.0736</v>
       </c>
       <c r="G29" t="n">
-        <v>34.5166</v>
+        <v>34.428</v>
       </c>
       <c r="H29" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>band_g_mix_b5o2</t>
+          <t>band_g_dyn</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1259,25 +1259,25 @@
         <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>1.0579</v>
+        <v>1.0636</v>
       </c>
       <c r="E30" t="n">
-        <v>1.0546</v>
+        <v>1.0628</v>
       </c>
       <c r="F30" t="n">
-        <v>1.0612</v>
+        <v>1.0644</v>
       </c>
       <c r="G30" t="n">
-        <v>34.6135</v>
+        <v>34.4297</v>
       </c>
       <c r="H30" t="n">
-        <v>4.05</v>
+        <v>4.15</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>band_g_mix_s3</t>
+          <t>band_g_mix_b7p5o3</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1287,25 +1287,25 @@
         <v>2</v>
       </c>
       <c r="D31" t="n">
-        <v>1.0553</v>
+        <v>1.061</v>
       </c>
       <c r="E31" t="n">
-        <v>1.0346</v>
+        <v>1.048</v>
       </c>
       <c r="F31" t="n">
-        <v>1.076</v>
+        <v>1.0741</v>
       </c>
       <c r="G31" t="n">
-        <v>34.7125</v>
+        <v>34.5166</v>
       </c>
       <c r="H31" t="n">
-        <v>2.15</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>band_gy_dyn</t>
+          <t>band_g_mix_b10o1</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1315,25 +1315,25 @@
         <v>2</v>
       </c>
       <c r="D32" t="n">
-        <v>1.0506</v>
+        <v>1.0608</v>
       </c>
       <c r="E32" t="n">
-        <v>1.0459</v>
+        <v>1.0578</v>
       </c>
       <c r="F32" t="n">
-        <v>1.0554</v>
+        <v>1.0639</v>
       </c>
       <c r="G32" t="n">
-        <v>34.8533</v>
+        <v>34.5166</v>
       </c>
       <c r="H32" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_b5o2</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1343,25 +1343,25 @@
         <v>2</v>
       </c>
       <c r="D33" t="n">
-        <v>1.0432</v>
+        <v>1.0579</v>
       </c>
       <c r="E33" t="n">
-        <v>1.0376</v>
+        <v>1.0546</v>
       </c>
       <c r="F33" t="n">
-        <v>1.0488</v>
+        <v>1.0612</v>
       </c>
       <c r="G33" t="n">
-        <v>35.1022</v>
+        <v>34.6135</v>
       </c>
       <c r="H33" t="n">
-        <v>2.9</v>
+        <v>4.05</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>band_g_mix_b1_y_s2</t>
+          <t>band_g_mix_s3</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1371,25 +1371,25 @@
         <v>2</v>
       </c>
       <c r="D34" t="n">
-        <v>1.0352</v>
+        <v>1.0553</v>
       </c>
       <c r="E34" t="n">
-        <v>1.0338</v>
+        <v>1.0346</v>
       </c>
       <c r="F34" t="n">
-        <v>1.0365</v>
+        <v>1.076</v>
       </c>
       <c r="G34" t="n">
-        <v>35.3747</v>
+        <v>34.7125</v>
       </c>
       <c r="H34" t="n">
-        <v>2.95</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>avg_g_window_hg</t>
+          <t>band_gy_dyn</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1399,53 +1399,53 @@
         <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>1.0301</v>
+        <v>1.0506</v>
       </c>
       <c r="E35" t="n">
-        <v>1.0294</v>
+        <v>1.0459</v>
       </c>
       <c r="F35" t="n">
-        <v>1.0308</v>
+        <v>1.0554</v>
       </c>
       <c r="G35" t="n">
-        <v>35.5482</v>
+        <v>34.8533</v>
       </c>
       <c r="H35" t="n">
-        <v>2.55</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>band_g_mix_s1</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>60</v>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>1.0292</v>
+        <v>1.0432</v>
       </c>
       <c r="E36" t="n">
-        <v>1.0039</v>
+        <v>1.0376</v>
       </c>
       <c r="F36" t="n">
-        <v>1.066</v>
+        <v>1.0488</v>
       </c>
       <c r="G36" t="n">
-        <v>35.6013</v>
+        <v>35.1022</v>
       </c>
       <c r="H36" t="n">
-        <v>0.8</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>avg_g_window_stock</t>
+          <t>band_g_mix_keep_s1</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1455,51 +1455,51 @@
         <v>2</v>
       </c>
       <c r="D37" t="n">
-        <v>1.029</v>
+        <v>1.0388</v>
       </c>
       <c r="E37" t="n">
-        <v>1.026</v>
+        <v>1.0357</v>
       </c>
       <c r="F37" t="n">
-        <v>1.0319</v>
+        <v>1.0419</v>
       </c>
       <c r="G37" t="n">
-        <v>35.5875</v>
+        <v>35.2519</v>
       </c>
       <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1_s3</t>
+          <t>band_g_mix_b1_y_s2</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>60</v>
       </c>
       <c r="C38" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D38" t="n">
-        <v>1.0233</v>
+        <v>1.0352</v>
       </c>
       <c r="E38" t="n">
-        <v>1.0165</v>
+        <v>1.0338</v>
       </c>
       <c r="F38" t="n">
-        <v>1.0395</v>
+        <v>1.0365</v>
       </c>
       <c r="G38" t="n">
-        <v>35.7888</v>
+        <v>35.3747</v>
       </c>
       <c r="H38" t="n">
-        <v>3.2</v>
+        <v>2.95</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>baseline_hg</t>
+          <t>avg_g_window_hg</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1509,109 +1509,107 @@
         <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>1.0162</v>
+        <v>1.0301</v>
       </c>
       <c r="E39" t="n">
-        <v>1.0147</v>
+        <v>1.0294</v>
       </c>
       <c r="F39" t="n">
-        <v>1.0177</v>
+        <v>1.0308</v>
       </c>
       <c r="G39" t="n">
-        <v>36.0347</v>
+        <v>35.5482</v>
       </c>
       <c r="H39" t="n">
-        <v>3</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>baseline FORCE_CMD=1.0</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>60</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D40" t="n">
-        <v>1.0017</v>
+        <v>1.0292</v>
       </c>
       <c r="E40" t="n">
-        <v>1.0017</v>
+        <v>1.0039</v>
       </c>
       <c r="F40" t="n">
-        <v>1.0017</v>
+        <v>1.066</v>
       </c>
       <c r="G40" t="n">
-        <v>36.5572</v>
+        <v>35.6013</v>
       </c>
       <c r="H40" t="n">
-        <v>3.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>baseline_stocknorpm</t>
+          <t>avg_g_window_stock</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>60</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D41" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.029</v>
       </c>
       <c r="E41" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.026</v>
       </c>
       <c r="F41" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.0319</v>
       </c>
       <c r="G41" t="n">
-        <v>37.0845</v>
-      </c>
-      <c r="H41" t="n">
-        <v>1</v>
-      </c>
+        <v>35.5875</v>
+      </c>
+      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>baseline_stock</t>
+          <t>band_g_mix_b1o1_s3</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>60</v>
       </c>
       <c r="C42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D42" t="n">
-        <v>0.8937</v>
+        <v>1.0233</v>
       </c>
       <c r="E42" t="n">
-        <v>0.8933</v>
+        <v>1.0165</v>
       </c>
       <c r="F42" t="n">
-        <v>0.8942</v>
+        <v>1.0395</v>
       </c>
       <c r="G42" t="n">
-        <v>40.9724</v>
+        <v>35.7888</v>
       </c>
       <c r="H42" t="n">
-        <v>3.5667</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>curation_hg</t>
+          <t>baseline_hg</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1621,51 +1619,53 @@
         <v>2</v>
       </c>
       <c r="D43" t="n">
-        <v>0.8874</v>
+        <v>1.0162</v>
       </c>
       <c r="E43" t="n">
-        <v>0.8813</v>
+        <v>1.0147</v>
       </c>
       <c r="F43" t="n">
-        <v>0.8935</v>
+        <v>1.0177</v>
       </c>
       <c r="G43" t="n">
-        <v>41.266</v>
-      </c>
-      <c r="H43" t="inlineStr"/>
+        <v>36.0347</v>
+      </c>
+      <c r="H43" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs2</t>
+          <t>baseline FORCE_CMD=1.0</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>60</v>
       </c>
       <c r="C44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>0.8228</v>
+        <v>1.0017</v>
       </c>
       <c r="E44" t="n">
-        <v>0.8045</v>
+        <v>1.0017</v>
       </c>
       <c r="F44" t="n">
-        <v>0.8411</v>
+        <v>1.0017</v>
       </c>
       <c r="G44" t="n">
-        <v>44.527</v>
+        <v>36.5572</v>
       </c>
       <c r="H44" t="n">
-        <v>1.9</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>baseline_stock16</t>
+          <t>baseline_stocknorpm</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1675,79 +1675,79 @@
         <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>0.7467</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="E45" t="n">
-        <v>0.7467</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="F45" t="n">
-        <v>0.7467</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="G45" t="n">
-        <v>49.0416</v>
-      </c>
-      <c r="H45" t="inlineStr"/>
+        <v>37.0845</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>band_g_mix_b20o1</t>
+          <t>baseline_stock</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>60</v>
       </c>
       <c r="C46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D46" t="n">
-        <v>0.7231</v>
+        <v>0.8937</v>
       </c>
       <c r="E46" t="n">
-        <v>0.4061</v>
+        <v>0.8933</v>
       </c>
       <c r="F46" t="n">
-        <v>1.0401</v>
+        <v>0.8942</v>
       </c>
       <c r="G46" t="n">
-        <v>62.6864</v>
+        <v>40.9724</v>
       </c>
       <c r="H46" t="n">
-        <v>1.95</v>
+        <v>3.5667</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>curation_hg</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>60</v>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D47" t="n">
-        <v>0.4106</v>
+        <v>0.8874</v>
       </c>
       <c r="E47" t="n">
-        <v>0.2278</v>
+        <v>0.8813</v>
       </c>
       <c r="F47" t="n">
-        <v>0.7759</v>
+        <v>0.8935</v>
       </c>
       <c r="G47" t="n">
-        <v>122.7889</v>
-      </c>
-      <c r="H47" t="n">
-        <v>2.1</v>
-      </c>
+        <v>41.266</v>
+      </c>
+      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>baseline_dynnoimu</t>
+          <t>baseline_dynstocknoabs2</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1757,53 +1757,51 @@
         <v>2</v>
       </c>
       <c r="D48" t="n">
-        <v>0.3672</v>
+        <v>0.8228</v>
       </c>
       <c r="E48" t="n">
-        <v>0.3661</v>
+        <v>0.8045</v>
       </c>
       <c r="F48" t="n">
-        <v>0.3683</v>
+        <v>0.8411</v>
       </c>
       <c r="G48" t="n">
-        <v>99.72539999999999</v>
+        <v>44.527</v>
       </c>
       <c r="H48" t="n">
-        <v>4.6</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>baseline_dynstock2</t>
+          <t>baseline_stock16</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>60</v>
       </c>
       <c r="C49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D49" t="n">
-        <v>0.2488</v>
+        <v>0.7467</v>
       </c>
       <c r="E49" t="n">
-        <v>0.2481</v>
+        <v>0.7467</v>
       </c>
       <c r="F49" t="n">
-        <v>0.2496</v>
+        <v>0.7467</v>
       </c>
       <c r="G49" t="n">
-        <v>147.1485</v>
-      </c>
-      <c r="H49" t="n">
-        <v>2.8</v>
-      </c>
+        <v>49.0416</v>
+      </c>
+      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>band_g_mix_b20o1</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1813,23 +1811,25 @@
         <v>2</v>
       </c>
       <c r="D50" t="n">
-        <v>0.2302</v>
+        <v>0.7231</v>
       </c>
       <c r="E50" t="n">
-        <v>0.2295</v>
+        <v>0.4061</v>
       </c>
       <c r="F50" t="n">
-        <v>0.2309</v>
+        <v>1.0401</v>
       </c>
       <c r="G50" t="n">
-        <v>159.0684</v>
-      </c>
-      <c r="H50" t="inlineStr"/>
+        <v>62.6864</v>
+      </c>
+      <c r="H50" t="n">
+        <v>1.95</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>avg_g_window</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1839,25 +1839,25 @@
         <v>3</v>
       </c>
       <c r="D51" t="n">
-        <v>0.2283</v>
+        <v>0.4106</v>
       </c>
       <c r="E51" t="n">
-        <v>0.2276</v>
+        <v>0.2278</v>
       </c>
       <c r="F51" t="n">
-        <v>0.2291</v>
+        <v>0.7759</v>
       </c>
       <c r="G51" t="n">
-        <v>160.3908</v>
+        <v>122.7889</v>
       </c>
       <c r="H51" t="n">
-        <v>3.2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>baseline_dynnoimu</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1867,23 +1867,25 @@
         <v>2</v>
       </c>
       <c r="D52" t="n">
-        <v>0.2258</v>
+        <v>0.3672</v>
       </c>
       <c r="E52" t="n">
-        <v>0.2252</v>
+        <v>0.3661</v>
       </c>
       <c r="F52" t="n">
-        <v>0.2263</v>
+        <v>0.3683</v>
       </c>
       <c r="G52" t="n">
-        <v>162.2099</v>
-      </c>
-      <c r="H52" t="inlineStr"/>
+        <v>99.72539999999999</v>
+      </c>
+      <c r="H52" t="n">
+        <v>4.6</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>peak_g_norpm</t>
+          <t>baseline_dynstock2</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1893,23 +1895,25 @@
         <v>2</v>
       </c>
       <c r="D53" t="n">
-        <v>0.2245</v>
+        <v>0.2488</v>
       </c>
       <c r="E53" t="n">
-        <v>0.2238</v>
+        <v>0.2481</v>
       </c>
       <c r="F53" t="n">
-        <v>0.2252</v>
+        <v>0.2496</v>
       </c>
       <c r="G53" t="n">
-        <v>163.1152</v>
-      </c>
-      <c r="H53" t="inlineStr"/>
+        <v>147.1485</v>
+      </c>
+      <c r="H53" t="n">
+        <v>2.8</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>baseline_dynstock</t>
+          <t>peak_g</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1919,185 +1923,187 @@
         <v>2</v>
       </c>
       <c r="D54" t="n">
-        <v>0.2241</v>
+        <v>0.2302</v>
       </c>
       <c r="E54" t="n">
-        <v>0.2235</v>
+        <v>0.2295</v>
       </c>
       <c r="F54" t="n">
-        <v>0.2247</v>
+        <v>0.2309</v>
       </c>
       <c r="G54" t="n">
-        <v>163.3969</v>
-      </c>
-      <c r="H54" t="n">
-        <v>3.05</v>
-      </c>
+        <v>159.0684</v>
+      </c>
+      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs</t>
+          <t>avg_g_window</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>60</v>
       </c>
       <c r="C55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D55" t="n">
-        <v>0.1982</v>
+        <v>0.2283</v>
       </c>
       <c r="E55" t="n">
-        <v>0.198</v>
+        <v>0.2276</v>
       </c>
       <c r="F55" t="n">
-        <v>0.1985</v>
+        <v>0.2291</v>
       </c>
       <c r="G55" t="n">
-        <v>184.7105</v>
+        <v>160.3908</v>
       </c>
       <c r="H55" t="n">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>avg_g_window_hg</t>
+          <t>yaw_intent</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D56" t="n">
-        <v>1.0148</v>
+        <v>0.2258</v>
       </c>
       <c r="E56" t="n">
-        <v>1.0148</v>
+        <v>0.2252</v>
       </c>
       <c r="F56" t="n">
-        <v>1.0148</v>
+        <v>0.2263</v>
       </c>
       <c r="G56" t="n">
-        <v>64.18680000000001</v>
-      </c>
-      <c r="H56" t="n">
-        <v>3.8</v>
-      </c>
+        <v>162.2099</v>
+      </c>
+      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>peak_g_norpm</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C57" t="n">
         <v>2</v>
       </c>
       <c r="D57" t="n">
-        <v>1.011</v>
+        <v>0.2245</v>
       </c>
       <c r="E57" t="n">
-        <v>1.0062</v>
+        <v>0.2238</v>
       </c>
       <c r="F57" t="n">
-        <v>1.0158</v>
+        <v>0.2252</v>
       </c>
       <c r="G57" t="n">
-        <v>50.3918</v>
+        <v>163.1152</v>
       </c>
       <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>baseline_dynstock</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D58" t="n">
-        <v>0.9869</v>
+        <v>0.2241</v>
       </c>
       <c r="E58" t="n">
-        <v>0.9869</v>
+        <v>0.2235</v>
       </c>
       <c r="F58" t="n">
-        <v>0.9869</v>
+        <v>0.2247</v>
       </c>
       <c r="G58" t="n">
-        <v>66.0052</v>
-      </c>
-      <c r="H58" t="inlineStr"/>
+        <v>163.3969</v>
+      </c>
+      <c r="H58" t="n">
+        <v>3.05</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>combined</t>
+          <t>baseline_dynstocknoabs</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D59" t="n">
-        <v>0.2276</v>
+        <v>0.1982</v>
       </c>
       <c r="E59" t="n">
-        <v>0.2276</v>
+        <v>0.198</v>
       </c>
       <c r="F59" t="n">
-        <v>0.2276</v>
+        <v>0.1985</v>
       </c>
       <c r="G59" t="n">
-        <v>160.9226</v>
-      </c>
-      <c r="H59" t="inlineStr"/>
+        <v>184.7105</v>
+      </c>
+      <c r="H59" t="n">
+        <v>3.75</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>avg_g_window_hg</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>80</v>
       </c>
       <c r="C60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D60" t="n">
-        <v>0.2159</v>
+        <v>1.0148</v>
       </c>
       <c r="E60" t="n">
-        <v>0.2156</v>
+        <v>1.0148</v>
       </c>
       <c r="F60" t="n">
-        <v>0.2162</v>
+        <v>1.0148</v>
       </c>
       <c r="G60" t="n">
-        <v>301.7328</v>
-      </c>
-      <c r="H60" t="inlineStr"/>
+        <v>64.18680000000001</v>
+      </c>
+      <c r="H60" t="n">
+        <v>3.8</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2107,70 +2113,174 @@
         <v>2</v>
       </c>
       <c r="D61" t="n">
-        <v>0.1782</v>
+        <v>1.011</v>
       </c>
       <c r="E61" t="n">
-        <v>0.1779</v>
+        <v>1.0062</v>
       </c>
       <c r="F61" t="n">
-        <v>0.1784</v>
+        <v>1.0158</v>
       </c>
       <c r="G61" t="n">
-        <v>365.637</v>
+        <v>50.3918</v>
       </c>
       <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>avg_g_window</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>80</v>
       </c>
       <c r="C62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D62" t="n">
-        <v>0.1778</v>
+        <v>0.9869</v>
       </c>
       <c r="E62" t="n">
-        <v>0.1776</v>
+        <v>0.9869</v>
       </c>
       <c r="F62" t="n">
-        <v>0.178</v>
+        <v>0.9869</v>
       </c>
       <c r="G62" t="n">
-        <v>366.3356</v>
+        <v>66.0052</v>
       </c>
       <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>combined</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>80</v>
       </c>
       <c r="C63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0.2276</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0.2276</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.2276</v>
+      </c>
+      <c r="G63" t="n">
+        <v>160.9226</v>
+      </c>
+      <c r="H63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>80</v>
+      </c>
+      <c r="C64" t="n">
         <v>2</v>
       </c>
-      <c r="D63" t="n">
+      <c r="D64" t="n">
+        <v>0.2159</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0.2156</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.2162</v>
+      </c>
+      <c r="G64" t="n">
+        <v>301.7328</v>
+      </c>
+      <c r="H64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>peak_g</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>80</v>
+      </c>
+      <c r="C65" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0.1782</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0.1779</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0.1784</v>
+      </c>
+      <c r="G65" t="n">
+        <v>365.637</v>
+      </c>
+      <c r="H65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>avg_g_window</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>80</v>
+      </c>
+      <c r="C66" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0.1778</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0.1776</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="G66" t="n">
+        <v>366.3356</v>
+      </c>
+      <c r="H66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>yaw_intent</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>80</v>
+      </c>
+      <c r="C67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D67" t="n">
         <v>0.1766</v>
       </c>
-      <c r="E63" t="n">
+      <c r="E67" t="n">
         <v>0.1766</v>
       </c>
-      <c r="F63" t="n">
+      <c r="F67" t="n">
         <v>0.1766</v>
       </c>
-      <c r="G63" t="n">
+      <c r="G67" t="n">
         <v>368.9042</v>
       </c>
-      <c r="H63" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2183,7 +2293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J143"/>
+  <dimension ref="A1:J151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6323,38 +6433,38 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>lockweight</t>
+          <t>slipkeep</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>band_g_mix_lock</t>
+          <t>band_g_mix_keep_s0</t>
         </is>
       </c>
       <c r="D113" t="n">
         <v>60</v>
       </c>
       <c r="E113" t="n">
-        <v>1.1277</v>
+        <v>1.1314</v>
       </c>
       <c r="F113" t="n">
-        <v>32.4713</v>
+        <v>32.365</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>1788409135-0001</t>
+          <t>1788469731-0001</t>
         </is>
       </c>
       <c r="H113" t="n">
-        <v>32.47</v>
+        <v>32.37</v>
       </c>
       <c r="I113" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="J113" t="n">
         <v>2.35</v>
@@ -6363,71 +6473,71 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>lockweight</t>
+          <t>slipkeep</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>band_g_mix_lock</t>
+          <t>band_g_mix_keep_s0</t>
         </is>
       </c>
       <c r="D114" t="n">
         <v>60</v>
       </c>
       <c r="E114" t="n">
-        <v>1.1072</v>
+        <v>1.1204</v>
       </c>
       <c r="F114" t="n">
-        <v>33.0721</v>
+        <v>32.6826</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>1788409168-0002</t>
+          <t>1788469763-0002</t>
         </is>
       </c>
       <c r="H114" t="n">
-        <v>33.07</v>
+        <v>32.68</v>
       </c>
       <c r="I114" t="n">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="J114" t="n">
-        <v>2.38</v>
+        <v>2.37</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>slipyaw3</t>
+          <t>slipkeep</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>band_g_mix_lock</t>
+          <t>band_g_mix_keep_s1</t>
         </is>
       </c>
       <c r="D115" t="n">
         <v>60</v>
       </c>
       <c r="E115" t="n">
-        <v>1.1007</v>
+        <v>1.0419</v>
       </c>
       <c r="F115" t="n">
-        <v>33.2682</v>
+        <v>35.1468</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>1788412341-0003</t>
+          <t>1788469799-0003</t>
         </is>
       </c>
       <c r="H115" t="inlineStr"/>
@@ -6437,42 +6547,36 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>slipyaw3</t>
+          <t>slipkeep</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>band_g_mix_lock</t>
+          <t>band_g_mix_keep_s1</t>
         </is>
       </c>
       <c r="D116" t="n">
         <v>60</v>
       </c>
       <c r="E116" t="n">
-        <v>1.0995</v>
+        <v>1.0357</v>
       </c>
       <c r="F116" t="n">
-        <v>33.3055</v>
+        <v>35.357</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>1788412373-0004</t>
-        </is>
-      </c>
-      <c r="H116" t="n">
-        <v>33.31</v>
-      </c>
-      <c r="I116" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="J116" t="n">
-        <v>2.39</v>
-      </c>
+          <t>1788469832-0004</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -6482,36 +6586,36 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>yawseeds</t>
+          <t>slipkeep</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s1</t>
+          <t>band_g_mix_keep_s2</t>
         </is>
       </c>
       <c r="D117" t="n">
         <v>60</v>
       </c>
       <c r="E117" t="n">
-        <v>1.1072</v>
+        <v>1.1017</v>
       </c>
       <c r="F117" t="n">
-        <v>33.0728</v>
+        <v>33.237</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>1788419867-0005</t>
+          <t>1788469869-0005</t>
         </is>
       </c>
       <c r="H117" t="n">
-        <v>33.08</v>
+        <v>33.24</v>
       </c>
       <c r="I117" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="J117" t="n">
-        <v>2.37</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="118">
@@ -6522,36 +6626,36 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>yawseeds</t>
+          <t>slipkeep</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s1</t>
+          <t>band_g_mix_keep_s2</t>
         </is>
       </c>
       <c r="D118" t="n">
         <v>60</v>
       </c>
       <c r="E118" t="n">
-        <v>1.0895</v>
+        <v>1.1077</v>
       </c>
       <c r="F118" t="n">
-        <v>33.6098</v>
+        <v>33.058</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>1788419899-0006</t>
+          <t>1788469902-0006</t>
         </is>
       </c>
       <c r="H118" t="n">
-        <v>33.61</v>
+        <v>33.06</v>
       </c>
       <c r="I118" t="n">
-        <v>2.8</v>
+        <v>3.6</v>
       </c>
       <c r="J118" t="n">
-        <v>2.42</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="119">
@@ -6562,31 +6666,37 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>yawseeds</t>
+          <t>slipkeep</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s2</t>
+          <t>band_g_mix_keepy_s0</t>
         </is>
       </c>
       <c r="D119" t="n">
         <v>60</v>
       </c>
       <c r="E119" t="n">
-        <v>1.1048</v>
+        <v>1.0891</v>
       </c>
       <c r="F119" t="n">
-        <v>33.1457</v>
+        <v>33.6213</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>1788419936-0007</t>
-        </is>
-      </c>
-      <c r="H119" t="inlineStr"/>
-      <c r="I119" t="inlineStr"/>
-      <c r="J119" t="inlineStr"/>
+          <t>1788469939-0007</t>
+        </is>
+      </c>
+      <c r="H119" t="n">
+        <v>33.63</v>
+      </c>
+      <c r="I119" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J119" t="n">
+        <v>2.41</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -6596,31 +6706,37 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>yawseeds</t>
+          <t>slipkeep</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s2</t>
+          <t>band_g_mix_keepy_s0</t>
         </is>
       </c>
       <c r="D120" t="n">
         <v>60</v>
       </c>
       <c r="E120" t="n">
-        <v>1.1085</v>
+        <v>1.0873</v>
       </c>
       <c r="F120" t="n">
-        <v>33.034</v>
+        <v>33.6774</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>1788419968-0008</t>
-        </is>
-      </c>
-      <c r="H120" t="inlineStr"/>
-      <c r="I120" t="inlineStr"/>
-      <c r="J120" t="inlineStr"/>
+          <t>1788469972-0008</t>
+        </is>
+      </c>
+      <c r="H120" t="n">
+        <v>33.68</v>
+      </c>
+      <c r="I120" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="J120" t="n">
+        <v>2.41</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -6630,36 +6746,36 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>slipyaw</t>
+          <t>lockweight</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s</t>
+          <t>band_g_mix_lock</t>
         </is>
       </c>
       <c r="D121" t="n">
         <v>60</v>
       </c>
       <c r="E121" t="n">
-        <v>1.0781</v>
+        <v>1.1277</v>
       </c>
       <c r="F121" t="n">
-        <v>33.9666</v>
+        <v>32.4713</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>1788410563-0002</t>
+          <t>1788409135-0001</t>
         </is>
       </c>
       <c r="H121" t="n">
-        <v>33.97</v>
+        <v>32.47</v>
       </c>
       <c r="I121" t="n">
-        <v>3.9</v>
+        <v>1.5</v>
       </c>
       <c r="J121" t="n">
-        <v>2.44</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="122">
@@ -6670,36 +6786,36 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>slipyaw</t>
+          <t>lockweight</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s</t>
+          <t>band_g_mix_lock</t>
         </is>
       </c>
       <c r="D122" t="n">
         <v>60</v>
       </c>
       <c r="E122" t="n">
-        <v>1.0781</v>
+        <v>1.1072</v>
       </c>
       <c r="F122" t="n">
-        <v>33.9666</v>
+        <v>33.0721</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>1788410563-0002</t>
+          <t>1788409168-0002</t>
         </is>
       </c>
       <c r="H122" t="n">
-        <v>33.97</v>
+        <v>33.07</v>
       </c>
       <c r="I122" t="n">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="J122" t="n">
-        <v>2.44</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="123">
@@ -6710,37 +6826,31 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>slipyaw</t>
+          <t>slipyaw3</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s</t>
+          <t>band_g_mix_lock</t>
         </is>
       </c>
       <c r="D123" t="n">
         <v>60</v>
       </c>
       <c r="E123" t="n">
-        <v>1.0691</v>
+        <v>1.1007</v>
       </c>
       <c r="F123" t="n">
-        <v>34.2528</v>
+        <v>33.2682</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>1788410595-0003</t>
-        </is>
-      </c>
-      <c r="H123" t="n">
-        <v>34.25</v>
-      </c>
-      <c r="I123" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="J123" t="n">
-        <v>2.45</v>
-      </c>
+          <t>1788412341-0003</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6750,116 +6860,116 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>slipyaw</t>
+          <t>slipyaw3</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s</t>
+          <t>band_g_mix_lock</t>
         </is>
       </c>
       <c r="D124" t="n">
         <v>60</v>
       </c>
       <c r="E124" t="n">
-        <v>1.0691</v>
+        <v>1.0995</v>
       </c>
       <c r="F124" t="n">
-        <v>34.2528</v>
+        <v>33.3055</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>1788410595-0003</t>
+          <t>1788412373-0004</t>
         </is>
       </c>
       <c r="H124" t="n">
-        <v>34.25</v>
+        <v>33.31</v>
       </c>
       <c r="I124" t="n">
-        <v>2.6</v>
+        <v>4.5</v>
       </c>
       <c r="J124" t="n">
-        <v>2.45</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>slipyaw3</t>
+          <t>yawseeds</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_sy</t>
+          <t>band_g_mix_lock_s1</t>
         </is>
       </c>
       <c r="D125" t="n">
         <v>60</v>
       </c>
       <c r="E125" t="n">
-        <v>1.1392</v>
+        <v>1.1072</v>
       </c>
       <c r="F125" t="n">
-        <v>32.1429</v>
+        <v>33.0728</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>1788412271-0001</t>
+          <t>1788419867-0005</t>
         </is>
       </c>
       <c r="H125" t="n">
-        <v>32.14</v>
+        <v>33.08</v>
       </c>
       <c r="I125" t="n">
-        <v>1.8</v>
+        <v>3.6</v>
       </c>
       <c r="J125" t="n">
-        <v>2.4</v>
+        <v>2.37</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>slipyaw3</t>
+          <t>yawseeds</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_sy</t>
+          <t>band_g_mix_lock_s1</t>
         </is>
       </c>
       <c r="D126" t="n">
         <v>60</v>
       </c>
       <c r="E126" t="n">
-        <v>1.1464</v>
+        <v>1.0895</v>
       </c>
       <c r="F126" t="n">
-        <v>31.9408</v>
+        <v>33.6098</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>1788412304-0002</t>
+          <t>1788419899-0006</t>
         </is>
       </c>
       <c r="H126" t="n">
-        <v>31.94</v>
+        <v>33.61</v>
       </c>
       <c r="I126" t="n">
-        <v>1.7</v>
+        <v>2.8</v>
       </c>
       <c r="J126" t="n">
-        <v>2.33</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="127">
@@ -6875,32 +6985,26 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_sy_s1</t>
+          <t>band_g_mix_lock_s2</t>
         </is>
       </c>
       <c r="D127" t="n">
         <v>60</v>
       </c>
       <c r="E127" t="n">
-        <v>1.1342</v>
+        <v>1.1048</v>
       </c>
       <c r="F127" t="n">
-        <v>32.2846</v>
+        <v>33.1457</v>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>1788419727-0001</t>
-        </is>
-      </c>
-      <c r="H127" t="n">
-        <v>32.29</v>
-      </c>
-      <c r="I127" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="J127" t="n">
-        <v>2.36</v>
-      </c>
+          <t>1788419936-0007</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -6915,179 +7019,185 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_sy_s1</t>
+          <t>band_g_mix_lock_s2</t>
         </is>
       </c>
       <c r="D128" t="n">
         <v>60</v>
       </c>
       <c r="E128" t="n">
-        <v>1.1413</v>
+        <v>1.1085</v>
       </c>
       <c r="F128" t="n">
-        <v>32.0846</v>
+        <v>33.034</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>1788419760-0002</t>
-        </is>
-      </c>
-      <c r="H128" t="n">
-        <v>32.09</v>
-      </c>
-      <c r="I128" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="J128" t="n">
-        <v>2.3</v>
-      </c>
+          <t>1788419968-0008</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>yawseeds</t>
+          <t>slipyaw</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_sy_s2</t>
+          <t>band_g_mix_lock_s</t>
         </is>
       </c>
       <c r="D129" t="n">
         <v>60</v>
       </c>
       <c r="E129" t="n">
-        <v>1.0771</v>
+        <v>1.0781</v>
       </c>
       <c r="F129" t="n">
-        <v>33.9969</v>
+        <v>33.9666</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>1788419797-0003</t>
-        </is>
-      </c>
-      <c r="H129" t="inlineStr"/>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
+          <t>1788410563-0002</t>
+        </is>
+      </c>
+      <c r="H129" t="n">
+        <v>33.97</v>
+      </c>
+      <c r="I129" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="J129" t="n">
+        <v>2.44</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>yawseeds</t>
+          <t>slipyaw</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_sy_s2</t>
+          <t>band_g_mix_lock_s</t>
         </is>
       </c>
       <c r="D130" t="n">
         <v>60</v>
       </c>
       <c r="E130" t="n">
-        <v>1.0712</v>
+        <v>1.0781</v>
       </c>
       <c r="F130" t="n">
-        <v>34.1856</v>
+        <v>33.9666</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>1788419829-0004</t>
-        </is>
-      </c>
-      <c r="H130" t="inlineStr"/>
-      <c r="I130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
+          <t>1788410563-0002</t>
+        </is>
+      </c>
+      <c r="H130" t="n">
+        <v>33.97</v>
+      </c>
+      <c r="I130" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="J130" t="n">
+        <v>2.44</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>yawseeds</t>
+          <t>slipyaw</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_y</t>
+          <t>band_g_mix_lock_s</t>
         </is>
       </c>
       <c r="D131" t="n">
         <v>60</v>
       </c>
       <c r="E131" t="n">
-        <v>1.1035</v>
+        <v>1.0691</v>
       </c>
       <c r="F131" t="n">
-        <v>33.183</v>
+        <v>34.2528</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>1788420005-0009</t>
+          <t>1788410595-0003</t>
         </is>
       </c>
       <c r="H131" t="n">
-        <v>33.18</v>
+        <v>34.25</v>
       </c>
       <c r="I131" t="n">
-        <v>1.6</v>
+        <v>2.6</v>
       </c>
       <c r="J131" t="n">
-        <v>2.53</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>yawseeds</t>
+          <t>slipyaw</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_y</t>
+          <t>band_g_mix_lock_s</t>
         </is>
       </c>
       <c r="D132" t="n">
         <v>60</v>
       </c>
       <c r="E132" t="n">
-        <v>1.1077</v>
+        <v>1.0691</v>
       </c>
       <c r="F132" t="n">
-        <v>33.0594</v>
+        <v>34.2528</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>1788420037-0010</t>
+          <t>1788410595-0003</t>
         </is>
       </c>
       <c r="H132" t="n">
-        <v>33.06</v>
+        <v>34.25</v>
       </c>
       <c r="I132" t="n">
-        <v>1.8</v>
+        <v>2.6</v>
       </c>
       <c r="J132" t="n">
-        <v>2.51</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="133">
@@ -7098,36 +7208,36 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>ensemble</t>
+          <t>slipyaw3</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_lock_sy</t>
         </is>
       </c>
       <c r="D133" t="n">
         <v>60</v>
       </c>
       <c r="E133" t="n">
-        <v>1.0488</v>
+        <v>1.1392</v>
       </c>
       <c r="F133" t="n">
-        <v>34.9145</v>
+        <v>32.1429</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>1788401068-0005</t>
+          <t>1788412271-0001</t>
         </is>
       </c>
       <c r="H133" t="n">
-        <v>34.91</v>
+        <v>32.14</v>
       </c>
       <c r="I133" t="n">
-        <v>3.5</v>
+        <v>1.8</v>
       </c>
       <c r="J133" t="n">
-        <v>2.48</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="134">
@@ -7138,270 +7248,264 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>ensemble</t>
+          <t>slipyaw3</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_lock_sy</t>
         </is>
       </c>
       <c r="D134" t="n">
         <v>60</v>
       </c>
       <c r="E134" t="n">
-        <v>1.0376</v>
+        <v>1.1464</v>
       </c>
       <c r="F134" t="n">
-        <v>35.29</v>
+        <v>31.9408</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>1788401101-0006</t>
+          <t>1788412304-0002</t>
         </is>
       </c>
       <c r="H134" t="n">
-        <v>35.29</v>
+        <v>31.94</v>
       </c>
       <c r="I134" t="n">
-        <v>2.3</v>
+        <v>1.7</v>
       </c>
       <c r="J134" t="n">
-        <v>2.5</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>pairedseeds</t>
+          <t>yawseeds</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>band_g_mix_s2</t>
+          <t>band_g_mix_lock_sy_s1</t>
         </is>
       </c>
       <c r="D135" t="n">
         <v>60</v>
       </c>
       <c r="E135" t="n">
-        <v>1.0923</v>
+        <v>1.1342</v>
       </c>
       <c r="F135" t="n">
-        <v>33.5239</v>
+        <v>32.2846</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>1788406643-0007</t>
+          <t>1788419727-0001</t>
         </is>
       </c>
       <c r="H135" t="n">
-        <v>33.53</v>
+        <v>32.29</v>
       </c>
       <c r="I135" t="n">
-        <v>4.9</v>
+        <v>2.2</v>
       </c>
       <c r="J135" t="n">
-        <v>2.42</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>pairedseeds</t>
+          <t>yawseeds</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>band_g_mix_s2</t>
+          <t>band_g_mix_lock_sy_s1</t>
         </is>
       </c>
       <c r="D136" t="n">
         <v>60</v>
       </c>
       <c r="E136" t="n">
-        <v>1.0916</v>
+        <v>1.1413</v>
       </c>
       <c r="F136" t="n">
-        <v>33.5441</v>
+        <v>32.0846</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>1788406677-0008</t>
-        </is>
-      </c>
-      <c r="H136" t="inlineStr"/>
-      <c r="I136" t="inlineStr"/>
-      <c r="J136" t="inlineStr"/>
+          <t>1788419760-0002</t>
+        </is>
+      </c>
+      <c r="H136" t="n">
+        <v>32.09</v>
+      </c>
+      <c r="I136" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J136" t="n">
+        <v>2.3</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>pairedseeds</t>
+          <t>yawseeds</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>band_g_mix_s3</t>
+          <t>band_g_mix_lock_sy_s2</t>
         </is>
       </c>
       <c r="D137" t="n">
         <v>60</v>
       </c>
       <c r="E137" t="n">
-        <v>1.0346</v>
+        <v>1.0771</v>
       </c>
       <c r="F137" t="n">
-        <v>35.3941</v>
+        <v>33.9969</v>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>1788406714-0009</t>
-        </is>
-      </c>
-      <c r="H137" t="n">
-        <v>35.39</v>
-      </c>
-      <c r="I137" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="J137" t="n">
-        <v>2.53</v>
-      </c>
+          <t>1788419797-0003</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>pairedseeds</t>
+          <t>yawseeds</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>band_g_mix_s3</t>
+          <t>band_g_mix_lock_sy_s2</t>
         </is>
       </c>
       <c r="D138" t="n">
         <v>60</v>
       </c>
       <c r="E138" t="n">
-        <v>1.076</v>
+        <v>1.0712</v>
       </c>
       <c r="F138" t="n">
-        <v>34.0309</v>
+        <v>34.1856</v>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>1788406747-0010</t>
-        </is>
-      </c>
-      <c r="H138" t="n">
-        <v>34.03</v>
-      </c>
-      <c r="I138" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="J138" t="n">
-        <v>2.56</v>
-      </c>
+          <t>1788419829-0004</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>restructure</t>
+          <t>yawseeds</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
+          <t>band_g_mix_lock_y</t>
         </is>
       </c>
       <c r="D139" t="n">
         <v>60</v>
       </c>
       <c r="E139" t="n">
-        <v>1.1085</v>
+        <v>1.1035</v>
       </c>
       <c r="F139" t="n">
-        <v>33.0351</v>
+        <v>33.183</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>1788399311-0002</t>
+          <t>1788420005-0009</t>
         </is>
       </c>
       <c r="H139" t="n">
-        <v>33.04</v>
+        <v>33.18</v>
       </c>
       <c r="I139" t="n">
-        <v>4.8</v>
+        <v>1.6</v>
       </c>
       <c r="J139" t="n">
-        <v>2.4</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>lockweight</t>
+          <t>yawseeds</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>baseline_dyn_lock</t>
+          <t>band_g_mix_lock_y</t>
         </is>
       </c>
       <c r="D140" t="n">
         <v>60</v>
       </c>
       <c r="E140" t="n">
-        <v>1.0756</v>
+        <v>1.1077</v>
       </c>
       <c r="F140" t="n">
-        <v>34.0434</v>
+        <v>33.0594</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>1788409205-0003</t>
+          <t>1788420037-0010</t>
         </is>
       </c>
       <c r="H140" t="n">
-        <v>34.04</v>
+        <v>33.06</v>
       </c>
       <c r="I140" t="n">
-        <v>4.5</v>
+        <v>1.8</v>
       </c>
       <c r="J140" t="n">
-        <v>2.45</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="141">
@@ -7412,36 +7516,36 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>lockweight</t>
+          <t>ensemble</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>baseline_dyn_lock</t>
+          <t>band_g_mix_s1</t>
         </is>
       </c>
       <c r="D141" t="n">
         <v>60</v>
       </c>
       <c r="E141" t="n">
-        <v>1.0817</v>
+        <v>1.0488</v>
       </c>
       <c r="F141" t="n">
-        <v>33.8519</v>
+        <v>34.9145</v>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>1788409238-0004</t>
+          <t>1788401068-0005</t>
         </is>
       </c>
       <c r="H141" t="n">
-        <v>33.85</v>
+        <v>34.91</v>
       </c>
       <c r="I141" t="n">
-        <v>4.3</v>
+        <v>3.5</v>
       </c>
       <c r="J141" t="n">
-        <v>2.43</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="142">
@@ -7457,31 +7561,31 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>ens_band_g_mix5</t>
+          <t>band_g_mix_s1</t>
         </is>
       </c>
       <c r="D142" t="n">
         <v>60</v>
       </c>
       <c r="E142" t="n">
-        <v>1.0736</v>
+        <v>1.0376</v>
       </c>
       <c r="F142" t="n">
-        <v>34.1079</v>
+        <v>35.29</v>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>1788400929-0001</t>
+          <t>1788401101-0006</t>
         </is>
       </c>
       <c r="H142" t="n">
-        <v>34.11</v>
+        <v>35.29</v>
       </c>
       <c r="I142" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="J142" t="n">
-        <v>2.44</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="143">
@@ -7492,35 +7596,349 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
+          <t>pairedseeds</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>band_g_mix_s2</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>60</v>
+      </c>
+      <c r="E143" t="n">
+        <v>1.0923</v>
+      </c>
+      <c r="F143" t="n">
+        <v>33.5239</v>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>1788406643-0007</t>
+        </is>
+      </c>
+      <c r="H143" t="n">
+        <v>33.53</v>
+      </c>
+      <c r="I143" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="J143" t="n">
+        <v>2.42</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>pairedseeds</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>band_g_mix_s2</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>60</v>
+      </c>
+      <c r="E144" t="n">
+        <v>1.0916</v>
+      </c>
+      <c r="F144" t="n">
+        <v>33.5441</v>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>1788406677-0008</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>pairedseeds</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>band_g_mix_s3</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>60</v>
+      </c>
+      <c r="E145" t="n">
+        <v>1.0346</v>
+      </c>
+      <c r="F145" t="n">
+        <v>35.3941</v>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>1788406714-0009</t>
+        </is>
+      </c>
+      <c r="H145" t="n">
+        <v>35.39</v>
+      </c>
+      <c r="I145" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J145" t="n">
+        <v>2.53</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>pairedseeds</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>band_g_mix_s3</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>60</v>
+      </c>
+      <c r="E146" t="n">
+        <v>1.076</v>
+      </c>
+      <c r="F146" t="n">
+        <v>34.0309</v>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>1788406747-0010</t>
+        </is>
+      </c>
+      <c r="H146" t="n">
+        <v>34.03</v>
+      </c>
+      <c r="I146" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J146" t="n">
+        <v>2.56</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>restructure</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>baseline_dyn</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>60</v>
+      </c>
+      <c r="E147" t="n">
+        <v>1.1085</v>
+      </c>
+      <c r="F147" t="n">
+        <v>33.0351</v>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>1788399311-0002</t>
+        </is>
+      </c>
+      <c r="H147" t="n">
+        <v>33.04</v>
+      </c>
+      <c r="I147" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="J147" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>lockweight</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>baseline_dyn_lock</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>60</v>
+      </c>
+      <c r="E148" t="n">
+        <v>1.0756</v>
+      </c>
+      <c r="F148" t="n">
+        <v>34.0434</v>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>1788409205-0003</t>
+        </is>
+      </c>
+      <c r="H148" t="n">
+        <v>34.04</v>
+      </c>
+      <c r="I148" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J148" t="n">
+        <v>2.45</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>lockweight</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>baseline_dyn_lock</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>60</v>
+      </c>
+      <c r="E149" t="n">
+        <v>1.0817</v>
+      </c>
+      <c r="F149" t="n">
+        <v>33.8519</v>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>1788409238-0004</t>
+        </is>
+      </c>
+      <c r="H149" t="n">
+        <v>33.85</v>
+      </c>
+      <c r="I149" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J149" t="n">
+        <v>2.43</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
           <t>ensemble</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr">
+      <c r="C150" t="inlineStr">
         <is>
           <t>ens_band_g_mix5</t>
         </is>
       </c>
-      <c r="D143" t="n">
-        <v>60</v>
-      </c>
-      <c r="E143" t="n">
+      <c r="D150" t="n">
+        <v>60</v>
+      </c>
+      <c r="E150" t="n">
+        <v>1.0736</v>
+      </c>
+      <c r="F150" t="n">
+        <v>34.1079</v>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>1788400929-0001</t>
+        </is>
+      </c>
+      <c r="H150" t="n">
+        <v>34.11</v>
+      </c>
+      <c r="I150" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J150" t="n">
+        <v>2.44</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>ens_band_g_mix5</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>60</v>
+      </c>
+      <c r="E151" t="n">
         <v>1.0538</v>
       </c>
-      <c r="F143" t="n">
+      <c r="F151" t="n">
         <v>34.7482</v>
       </c>
-      <c r="G143" t="inlineStr">
+      <c r="G151" t="inlineStr">
         <is>
           <t>1788400962-0002</t>
         </is>
       </c>
-      <c r="H143" t="n">
+      <c r="H151" t="n">
         <v>34.75</v>
       </c>
-      <c r="I143" t="n">
+      <c r="I151" t="n">
         <v>2</v>
       </c>
-      <c r="J143" t="n">
+      <c r="J151" t="n">
         <v>2.48</v>
       </c>
     </row>
@@ -7535,7 +7953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N56"/>
+  <dimension ref="A1:N60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -8589,7 +9007,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>band_g_mix_lock</t>
+          <t>band_g_mix_keep_s0</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -8599,7 +9017,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-09-02T21:16:23</t>
+          <t>2026-09-03T14:03:19</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -8637,7 +9055,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>[0.15058, 0.15519, 0.171, 0.17031]</t>
+          <t>[0.16033, 0.16304, 0.17293, 0.17217]</t>
         </is>
       </c>
       <c r="N22" t="inlineStr"/>
@@ -8645,7 +9063,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s1</t>
+          <t>band_g_mix_keep_s1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -8655,7 +9073,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-09-03T00:11:14</t>
+          <t>2026-09-03T14:04:42</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -8693,7 +9111,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>[0.152, 0.15449, 0.17063, 0.17097]</t>
+          <t>[0.15514, 0.15842, 0.17031, 0.16974]</t>
         </is>
       </c>
       <c r="N23" t="inlineStr"/>
@@ -8701,7 +9119,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s2</t>
+          <t>band_g_mix_keep_s2</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -8711,7 +9129,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-09-03T00:12:39</t>
+          <t>2026-09-03T14:06:06</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -8749,7 +9167,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>[0.15082, 0.15738, 0.17089, 0.16978]</t>
+          <t>[0.15564, 0.15825, 0.17158, 0.17018]</t>
         </is>
       </c>
       <c r="N24" t="inlineStr"/>
@@ -8757,7 +9175,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s</t>
+          <t>band_g_mix_keepy_s0</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -8767,7 +9185,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-09-02T21:26:40</t>
+          <t>2026-09-03T14:07:29</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -8805,7 +9223,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>[0.1511, 0.15729, 0.1708, 0.16893]</t>
+          <t>[0.15259, 0.15739, 0.17198, 0.17108]</t>
         </is>
       </c>
       <c r="N25" t="inlineStr"/>
@@ -8813,7 +9231,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_sy</t>
+          <t>band_g_mix_lock</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -8823,7 +9241,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-09-02T21:28:05</t>
+          <t>2026-09-02T21:16:23</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -8861,7 +9279,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>[0.15131, 0.15295, 0.1697, 0.16946]</t>
+          <t>[0.15058, 0.15519, 0.171, 0.17031]</t>
         </is>
       </c>
       <c r="N26" t="inlineStr"/>
@@ -8869,7 +9287,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_sy_s1</t>
+          <t>band_g_mix_lock_s1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -8879,7 +9297,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-09-03T00:08:32</t>
+          <t>2026-09-03T00:11:14</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -8917,7 +9335,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>[0.14868, 0.15309, 0.16853, 0.16879]</t>
+          <t>[0.152, 0.15449, 0.17063, 0.17097]</t>
         </is>
       </c>
       <c r="N27" t="inlineStr"/>
@@ -8925,7 +9343,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_sy_s2</t>
+          <t>band_g_mix_lock_s2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -8935,7 +9353,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-09-03T00:09:53</t>
+          <t>2026-09-03T00:12:39</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -8973,7 +9391,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>[0.14937, 0.15545, 0.17107, 0.16995]</t>
+          <t>[0.15082, 0.15738, 0.17089, 0.16978]</t>
         </is>
       </c>
       <c r="N28" t="inlineStr"/>
@@ -8981,7 +9399,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_y</t>
+          <t>band_g_mix_lock_s</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -8991,7 +9409,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-09-03T00:14:01</t>
+          <t>2026-09-02T21:26:40</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -9029,7 +9447,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>[0.15046, 0.15335, 0.17045, 0.16869]</t>
+          <t>[0.1511, 0.15729, 0.1708, 0.16893]</t>
         </is>
       </c>
       <c r="N29" t="inlineStr"/>
@@ -9037,7 +9455,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_g_mix_lock_sy</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -9047,7 +9465,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-09-02T18:54:00</t>
+          <t>2026-09-02T21:28:05</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -9085,7 +9503,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>[0.14226, 0.15404, 0.16814, 0.16762]</t>
+          <t>[0.15131, 0.15295, 0.1697, 0.16946]</t>
         </is>
       </c>
       <c r="N30" t="inlineStr"/>
@@ -9093,7 +9511,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>band_g_mix_s2</t>
+          <t>band_g_mix_lock_sy_s1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -9103,7 +9521,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-09-02T18:55:36</t>
+          <t>2026-09-03T00:08:32</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -9141,7 +9559,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>[0.15115, 0.15324, 0.16928, 0.16978]</t>
+          <t>[0.14868, 0.15309, 0.16853, 0.16879]</t>
         </is>
       </c>
       <c r="N31" t="inlineStr"/>
@@ -9149,7 +9567,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>band_g_mix_s3</t>
+          <t>band_g_mix_lock_sy_s2</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -9159,7 +9577,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-09-02T18:57:18</t>
+          <t>2026-09-03T00:09:53</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -9197,7 +9615,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>[0.15575, 0.16054, 0.1713, 0.17144]</t>
+          <t>[0.14937, 0.15545, 0.17107, 0.16995]</t>
         </is>
       </c>
       <c r="N32" t="inlineStr"/>
@@ -9205,7 +9623,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>band_g_mix_s4</t>
+          <t>band_g_mix_lock_y</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -9215,7 +9633,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-09-02T18:58:55</t>
+          <t>2026-09-03T00:14:01</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -9253,7 +9671,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>[0.14723, 0.15025, 0.16854, 0.16772]</t>
+          <t>[0.15046, 0.15335, 0.17045, 0.16869]</t>
         </is>
       </c>
       <c r="N33" t="inlineStr"/>
@@ -9261,7 +9679,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>band_g_mix_s5</t>
+          <t>band_g_mix_s1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -9271,7 +9689,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-09-02T19:00:42</t>
+          <t>2026-09-02T18:54:00</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -9309,7 +9727,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>[0.14491, 0.15532, 0.16904, 0.16805]</t>
+          <t>[0.14226, 0.15404, 0.16814, 0.16762]</t>
         </is>
       </c>
       <c r="N34" t="inlineStr"/>
@@ -9317,159 +9735,255 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>band_gy_dyn</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
+          <t>band_g_mix_s2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:55:36</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>5</v>
+      </c>
+      <c r="K35" t="n">
+        <v>1</v>
+      </c>
+      <c r="L35" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>[0.15115, 0.15324, 0.16928, 0.16978]</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>band_gy_mix</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
+          <t>band_g_mix_s3</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:57:18</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>5</v>
+      </c>
+      <c r="K36" t="n">
+        <v>1</v>
+      </c>
+      <c r="L36" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>[0.15575, 0.16054, 0.1713, 0.17144]</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>baseline</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
+          <t>band_g_mix_s4</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2026-09-02T18:58:55</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>5</v>
+      </c>
+      <c r="K37" t="n">
+        <v>1</v>
+      </c>
+      <c r="L37" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>[0.14723, 0.15025, 0.16854, 0.16772]</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
+          <t>band_g_mix_s5</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>band_g</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2026-09-02T19:00:42</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>5</v>
+      </c>
+      <c r="K38" t="n">
+        <v>1</v>
+      </c>
+      <c r="L38" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>[0.14491, 0.15532, 0.16904, 0.16805]</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>baseline_dyn_lock</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>baseline</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>2026-09-02T21:17:44</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>dyn_abs</t>
-        </is>
-      </c>
+          <t>band_gy_dyn</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>etk800</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>sensor_z,roll_angle,pitch_angle,gear</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>gy2</t>
-        </is>
-      </c>
-      <c r="J39" t="n">
-        <v>5</v>
-      </c>
-      <c r="K39" t="n">
-        <v>1</v>
-      </c>
-      <c r="L39" t="n">
-        <v>1129</v>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>[0.13261, 0.15194, 0.08818, 0.08624]</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>baseline_dynnoimu</t>
+          <t>band_gy_mix</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -9493,7 +10007,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>baseline_dynstock2</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -9517,7 +10031,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>baseline_dynstock</t>
+          <t>baseline_dyn</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
@@ -9541,31 +10055,63 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs2</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
+          <t>baseline_dyn_lock</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2026-09-02T21:17:44</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>dyn_abs</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>5</v>
+      </c>
+      <c r="K43" t="n">
+        <v>1</v>
+      </c>
+      <c r="L43" t="n">
+        <v>1129</v>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>[0.13261, 0.15194, 0.08818, 0.08624]</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs</t>
+          <t>baseline_dynnoimu</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -9589,7 +10135,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>baseline_hg</t>
+          <t>baseline_dynstock2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
@@ -9613,7 +10159,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>baseline_norpm</t>
+          <t>baseline_dynstock</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
@@ -9637,7 +10183,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>baseline_stock16</t>
+          <t>baseline_dynstocknoabs2</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -9661,7 +10207,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>baseline_dynstocknoabs</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -9685,7 +10231,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>baseline_stock</t>
+          <t>baseline_hg</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -9709,7 +10255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>baseline_stocknorpm</t>
+          <t>baseline_norpm</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -9733,7 +10279,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>combined</t>
+          <t>baseline_stock16</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
@@ -9757,7 +10303,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -9781,7 +10327,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>curation_hg</t>
+          <t>baseline_stock</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
@@ -9805,7 +10351,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>baseline_stocknorpm</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
@@ -9829,7 +10375,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>peak_g_norpm</t>
+          <t>combined</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
@@ -9853,7 +10399,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
@@ -9874,6 +10420,102 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>curation_hg</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>peak_g</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>peak_g_norpm</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>yaw_intent</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Unfiltered high-gain episode-g variant; regenerate README tables
</commit_message>
<xml_diff>
--- a/results/LSTM_ABS_RESULTS.xlsx
+++ b/results/LSTM_ABS_RESULTS.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -753,7 +753,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>band_g_mix_b1_sy_s2</t>
+          <t>baseline_all_epg3_s0</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -763,25 +763,25 @@
         <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>1.12</v>
+        <v>1.1218</v>
       </c>
       <c r="E12" t="n">
-        <v>1.1184</v>
+        <v>1.0915</v>
       </c>
       <c r="F12" t="n">
-        <v>1.1215</v>
+        <v>1.1522</v>
       </c>
       <c r="G12" t="n">
-        <v>32.6967</v>
+        <v>32.6658</v>
       </c>
       <c r="H12" t="n">
-        <v>2.5</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>band_g_mix_b1_sy_s0</t>
+          <t>band_g_mix_b1_sy_s2</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -791,79 +791,81 @@
         <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>1.1102</v>
+        <v>1.12</v>
       </c>
       <c r="E13" t="n">
-        <v>1.0997</v>
+        <v>1.1184</v>
       </c>
       <c r="F13" t="n">
-        <v>1.1207</v>
+        <v>1.1215</v>
       </c>
       <c r="G13" t="n">
-        <v>32.987</v>
+        <v>32.6967</v>
       </c>
       <c r="H13" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>band_g_mix_lock</t>
+          <t>band_g_mix_b1_sy_s0</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>60</v>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>1.1088</v>
+        <v>1.1102</v>
       </c>
       <c r="E14" t="n">
-        <v>1.0995</v>
+        <v>1.0997</v>
       </c>
       <c r="F14" t="n">
-        <v>1.1277</v>
+        <v>1.1207</v>
       </c>
       <c r="G14" t="n">
-        <v>33.0293</v>
+        <v>32.987</v>
       </c>
       <c r="H14" t="n">
-        <v>3.5</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s2</t>
+          <t>band_g_mix_lock</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>60</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>1.1067</v>
+        <v>1.1088</v>
       </c>
       <c r="E15" t="n">
-        <v>1.1048</v>
+        <v>1.0995</v>
       </c>
       <c r="F15" t="n">
-        <v>1.1085</v>
+        <v>1.1277</v>
       </c>
       <c r="G15" t="n">
-        <v>33.0898</v>
-      </c>
-      <c r="H15" t="inlineStr"/>
+        <v>33.0293</v>
+      </c>
+      <c r="H15" t="n">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_y</t>
+          <t>band_g_mix_lock_s2</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -873,25 +875,23 @@
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>1.1056</v>
+        <v>1.1067</v>
       </c>
       <c r="E16" t="n">
-        <v>1.1035</v>
+        <v>1.1048</v>
       </c>
       <c r="F16" t="n">
-        <v>1.1077</v>
+        <v>1.1085</v>
       </c>
       <c r="G16" t="n">
-        <v>33.1212</v>
-      </c>
-      <c r="H16" t="n">
-        <v>1.7</v>
-      </c>
+        <v>33.0898</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>band_g_mix_keep_s2</t>
+          <t>band_g_mix_lock_y</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -901,25 +901,25 @@
         <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>1.1047</v>
+        <v>1.1056</v>
       </c>
       <c r="E17" t="n">
-        <v>1.1017</v>
+        <v>1.1035</v>
       </c>
       <c r="F17" t="n">
         <v>1.1077</v>
       </c>
       <c r="G17" t="n">
-        <v>33.1475</v>
+        <v>33.1212</v>
       </c>
       <c r="H17" t="n">
-        <v>3.7</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>band_g_mix_b1_y_s0</t>
+          <t>band_g_mix_keep_s2</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -929,25 +929,25 @@
         <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>1.1024</v>
+        <v>1.1047</v>
       </c>
       <c r="E18" t="n">
-        <v>1.0999</v>
+        <v>1.1017</v>
       </c>
       <c r="F18" t="n">
-        <v>1.1048</v>
+        <v>1.1077</v>
       </c>
       <c r="G18" t="n">
-        <v>33.2183</v>
+        <v>33.1475</v>
       </c>
       <c r="H18" t="n">
-        <v>1.45</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1</t>
+          <t>band_g_mix_b1_y_s0</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -957,25 +957,25 @@
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>1.1018</v>
+        <v>1.1024</v>
       </c>
       <c r="E19" t="n">
-        <v>1.0902</v>
+        <v>1.0999</v>
       </c>
       <c r="F19" t="n">
-        <v>1.1133</v>
+        <v>1.1048</v>
       </c>
       <c r="G19" t="n">
-        <v>33.2398</v>
+        <v>33.2183</v>
       </c>
       <c r="H19" t="n">
-        <v>1.5</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>band_g_mix_b1_y_s1</t>
+          <t>band_g_mix_b1o1</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -985,23 +985,25 @@
         <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>1.0992</v>
+        <v>1.1018</v>
       </c>
       <c r="E20" t="n">
-        <v>1.0948</v>
+        <v>1.0902</v>
       </c>
       <c r="F20" t="n">
-        <v>1.1036</v>
+        <v>1.1133</v>
       </c>
       <c r="G20" t="n">
-        <v>33.3144</v>
-      </c>
-      <c r="H20" t="inlineStr"/>
+        <v>33.2398</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s1</t>
+          <t>band_g_mix_b1_y_s1</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1011,25 +1013,23 @@
         <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>1.0984</v>
+        <v>1.0992</v>
       </c>
       <c r="E21" t="n">
-        <v>1.0895</v>
+        <v>1.0948</v>
       </c>
       <c r="F21" t="n">
-        <v>1.1072</v>
+        <v>1.1036</v>
       </c>
       <c r="G21" t="n">
-        <v>33.3413</v>
-      </c>
-      <c r="H21" t="n">
-        <v>3.2</v>
-      </c>
+        <v>33.3144</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>band_g_mix_s2</t>
+          <t>band_g_mix_lock_s1</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1039,25 +1039,25 @@
         <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>1.092</v>
+        <v>1.0984</v>
       </c>
       <c r="E22" t="n">
-        <v>1.0916</v>
+        <v>1.0895</v>
       </c>
       <c r="F22" t="n">
-        <v>1.0923</v>
+        <v>1.1072</v>
       </c>
       <c r="G22" t="n">
-        <v>33.534</v>
+        <v>33.3413</v>
       </c>
       <c r="H22" t="n">
-        <v>4.9</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>band_g_mix_b2p5o2</t>
+          <t>band_g_mix_s2</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1067,25 +1067,25 @@
         <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>1.0884</v>
+        <v>1.092</v>
       </c>
       <c r="E23" t="n">
-        <v>1.0823</v>
+        <v>1.0916</v>
       </c>
       <c r="F23" t="n">
-        <v>1.0944</v>
+        <v>1.0923</v>
       </c>
       <c r="G23" t="n">
-        <v>33.6464</v>
+        <v>33.534</v>
       </c>
       <c r="H23" t="n">
-        <v>1.55</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>band_g_mix_keepy_s0</t>
+          <t>band_g_mix_b2p5o2</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1095,25 +1095,25 @@
         <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>1.0882</v>
+        <v>1.0884</v>
       </c>
       <c r="E24" t="n">
-        <v>1.0873</v>
+        <v>1.0823</v>
       </c>
       <c r="F24" t="n">
-        <v>1.0891</v>
+        <v>1.0944</v>
       </c>
       <c r="G24" t="n">
-        <v>33.6494</v>
+        <v>33.6464</v>
       </c>
       <c r="H24" t="n">
-        <v>3.6</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>band_g_mix_b1_sy_s1</t>
+          <t>band_g_mix_keepy_s0</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1123,23 +1123,25 @@
         <v>2</v>
       </c>
       <c r="D25" t="n">
-        <v>1.0866</v>
+        <v>1.0882</v>
       </c>
       <c r="E25" t="n">
-        <v>1.0848</v>
+        <v>1.0873</v>
       </c>
       <c r="F25" t="n">
-        <v>1.0884</v>
+        <v>1.0891</v>
       </c>
       <c r="G25" t="n">
-        <v>33.7008</v>
-      </c>
-      <c r="H25" t="inlineStr"/>
+        <v>33.6494</v>
+      </c>
+      <c r="H25" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>baseline_dyn_lock</t>
+          <t>band_g_mix_b1_sy_s1</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1149,25 +1151,23 @@
         <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>1.0787</v>
+        <v>1.0866</v>
       </c>
       <c r="E26" t="n">
-        <v>1.0756</v>
+        <v>1.0848</v>
       </c>
       <c r="F26" t="n">
-        <v>1.0817</v>
+        <v>1.0884</v>
       </c>
       <c r="G26" t="n">
-        <v>33.9476</v>
-      </c>
-      <c r="H26" t="n">
-        <v>4.4</v>
-      </c>
+        <v>33.7008</v>
+      </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_sy_s2</t>
+          <t>baseline_dyn_lock</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1177,107 +1177,107 @@
         <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>1.0742</v>
+        <v>1.0787</v>
       </c>
       <c r="E27" t="n">
-        <v>1.0712</v>
+        <v>1.0756</v>
       </c>
       <c r="F27" t="n">
-        <v>1.0771</v>
+        <v>1.0817</v>
       </c>
       <c r="G27" t="n">
-        <v>34.0912</v>
-      </c>
-      <c r="H27" t="inlineStr"/>
+        <v>33.9476</v>
+      </c>
+      <c r="H27" t="n">
+        <v>4.4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>band_g_mix_lock_s</t>
+          <t>band_g_mix_lock_sy_s2</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>60</v>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D28" t="n">
-        <v>1.0736</v>
+        <v>1.0742</v>
       </c>
       <c r="E28" t="n">
-        <v>1.0691</v>
+        <v>1.0712</v>
       </c>
       <c r="F28" t="n">
-        <v>1.0781</v>
+        <v>1.0771</v>
       </c>
       <c r="G28" t="n">
-        <v>34.1097</v>
-      </c>
-      <c r="H28" t="n">
-        <v>3.25</v>
-      </c>
+        <v>34.0912</v>
+      </c>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1_s1</t>
+          <t>baseline_all_epg3_s1</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>60</v>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>1.0703</v>
+        <v>1.0741</v>
       </c>
       <c r="E29" t="n">
-        <v>1.0684</v>
+        <v>1.0741</v>
       </c>
       <c r="F29" t="n">
-        <v>1.0722</v>
+        <v>1.0741</v>
       </c>
       <c r="G29" t="n">
-        <v>34.2125</v>
+        <v>34.0906</v>
       </c>
       <c r="H29" t="n">
-        <v>2.1</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>band_g_mix_lock_s</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>60</v>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" t="n">
-        <v>1.0671</v>
+        <v>1.0736</v>
       </c>
       <c r="E30" t="n">
-        <v>1.0582</v>
+        <v>1.0691</v>
       </c>
       <c r="F30" t="n">
-        <v>1.0716</v>
+        <v>1.0781</v>
       </c>
       <c r="G30" t="n">
-        <v>34.3171</v>
+        <v>34.1097</v>
       </c>
       <c r="H30" t="n">
-        <v>2.3667</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ens_band_g_mix5</t>
+          <t>band_g_mix_b1o1_s1</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1287,53 +1287,53 @@
         <v>2</v>
       </c>
       <c r="D31" t="n">
-        <v>1.0637</v>
+        <v>1.0703</v>
       </c>
       <c r="E31" t="n">
-        <v>1.0538</v>
+        <v>1.0684</v>
       </c>
       <c r="F31" t="n">
-        <v>1.0736</v>
+        <v>1.0722</v>
       </c>
       <c r="G31" t="n">
-        <v>34.428</v>
+        <v>34.2125</v>
       </c>
       <c r="H31" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>band_g_dyn</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>60</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>1.0636</v>
+        <v>1.0671</v>
       </c>
       <c r="E32" t="n">
-        <v>1.0628</v>
+        <v>1.0582</v>
       </c>
       <c r="F32" t="n">
-        <v>1.0644</v>
+        <v>1.0716</v>
       </c>
       <c r="G32" t="n">
-        <v>34.4297</v>
+        <v>34.3171</v>
       </c>
       <c r="H32" t="n">
-        <v>4.15</v>
+        <v>2.3667</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>band_g_mix_b7p5o3</t>
+          <t>ens_band_g_mix5</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1343,25 +1343,25 @@
         <v>2</v>
       </c>
       <c r="D33" t="n">
-        <v>1.061</v>
+        <v>1.0637</v>
       </c>
       <c r="E33" t="n">
-        <v>1.048</v>
+        <v>1.0538</v>
       </c>
       <c r="F33" t="n">
-        <v>1.0741</v>
+        <v>1.0736</v>
       </c>
       <c r="G33" t="n">
-        <v>34.5166</v>
+        <v>34.428</v>
       </c>
       <c r="H33" t="n">
-        <v>1.45</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>band_g_mix_b10o1</t>
+          <t>band_g_dyn</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1371,25 +1371,25 @@
         <v>2</v>
       </c>
       <c r="D34" t="n">
-        <v>1.0608</v>
+        <v>1.0636</v>
       </c>
       <c r="E34" t="n">
-        <v>1.0578</v>
+        <v>1.0628</v>
       </c>
       <c r="F34" t="n">
-        <v>1.0639</v>
+        <v>1.0644</v>
       </c>
       <c r="G34" t="n">
-        <v>34.5166</v>
+        <v>34.4297</v>
       </c>
       <c r="H34" t="n">
-        <v>2.4</v>
+        <v>4.15</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>band_g_mix_b5o2</t>
+          <t>band_g_mix_b7p5o3</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1399,25 +1399,25 @@
         <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>1.0579</v>
+        <v>1.061</v>
       </c>
       <c r="E35" t="n">
-        <v>1.0546</v>
+        <v>1.048</v>
       </c>
       <c r="F35" t="n">
-        <v>1.0612</v>
+        <v>1.0741</v>
       </c>
       <c r="G35" t="n">
-        <v>34.6135</v>
+        <v>34.5166</v>
       </c>
       <c r="H35" t="n">
-        <v>4.05</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>band_g_mix_s3</t>
+          <t>band_g_mix_b10o1</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1427,25 +1427,25 @@
         <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>1.0553</v>
+        <v>1.0608</v>
       </c>
       <c r="E36" t="n">
-        <v>1.0346</v>
+        <v>1.0578</v>
       </c>
       <c r="F36" t="n">
-        <v>1.076</v>
+        <v>1.0639</v>
       </c>
       <c r="G36" t="n">
-        <v>34.7125</v>
+        <v>34.5166</v>
       </c>
       <c r="H36" t="n">
-        <v>2.15</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>baseline_mix_epg_s1</t>
+          <t>band_g_mix_b5o2</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1455,25 +1455,25 @@
         <v>2</v>
       </c>
       <c r="D37" t="n">
-        <v>1.0518</v>
+        <v>1.0579</v>
       </c>
       <c r="E37" t="n">
-        <v>1.0512</v>
+        <v>1.0546</v>
       </c>
       <c r="F37" t="n">
-        <v>1.0525</v>
+        <v>1.0612</v>
       </c>
       <c r="G37" t="n">
-        <v>34.8139</v>
+        <v>34.6135</v>
       </c>
       <c r="H37" t="n">
-        <v>2.9</v>
+        <v>4.05</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>band_gy_dyn</t>
+          <t>band_g_mix_s3</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1483,25 +1483,25 @@
         <v>2</v>
       </c>
       <c r="D38" t="n">
-        <v>1.0506</v>
+        <v>1.0553</v>
       </c>
       <c r="E38" t="n">
-        <v>1.0459</v>
+        <v>1.0346</v>
       </c>
       <c r="F38" t="n">
-        <v>1.0554</v>
+        <v>1.076</v>
       </c>
       <c r="G38" t="n">
-        <v>34.8533</v>
+        <v>34.7125</v>
       </c>
       <c r="H38" t="n">
-        <v>2.6</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>band_g_mix_bandepg_s0</t>
+          <t>baseline_mix_epg_s1</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1511,25 +1511,25 @@
         <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>1.0482</v>
+        <v>1.0518</v>
       </c>
       <c r="E39" t="n">
-        <v>1.0446</v>
+        <v>1.0512</v>
       </c>
       <c r="F39" t="n">
-        <v>1.0517</v>
+        <v>1.0525</v>
       </c>
       <c r="G39" t="n">
-        <v>34.936</v>
+        <v>34.8139</v>
       </c>
       <c r="H39" t="n">
-        <v>3.05</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>band_g_mix_s1</t>
+          <t>band_gy_dyn</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1539,25 +1539,25 @@
         <v>2</v>
       </c>
       <c r="D40" t="n">
-        <v>1.0432</v>
+        <v>1.0506</v>
       </c>
       <c r="E40" t="n">
-        <v>1.0376</v>
+        <v>1.0459</v>
       </c>
       <c r="F40" t="n">
-        <v>1.0488</v>
+        <v>1.0554</v>
       </c>
       <c r="G40" t="n">
-        <v>35.1022</v>
+        <v>34.8533</v>
       </c>
       <c r="H40" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>band_g_mix_keep_s1</t>
+          <t>band_g_mix_bandepg_s0</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1567,23 +1567,25 @@
         <v>2</v>
       </c>
       <c r="D41" t="n">
-        <v>1.0388</v>
+        <v>1.0482</v>
       </c>
       <c r="E41" t="n">
-        <v>1.0357</v>
+        <v>1.0446</v>
       </c>
       <c r="F41" t="n">
-        <v>1.0419</v>
+        <v>1.0517</v>
       </c>
       <c r="G41" t="n">
-        <v>35.2519</v>
-      </c>
-      <c r="H41" t="inlineStr"/>
+        <v>34.936</v>
+      </c>
+      <c r="H41" t="n">
+        <v>3.05</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>band_g_mix_b1_y_s2</t>
+          <t>band_g_mix_s1</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1593,25 +1595,25 @@
         <v>2</v>
       </c>
       <c r="D42" t="n">
-        <v>1.0352</v>
+        <v>1.0432</v>
       </c>
       <c r="E42" t="n">
-        <v>1.0338</v>
+        <v>1.0376</v>
       </c>
       <c r="F42" t="n">
-        <v>1.0365</v>
+        <v>1.0488</v>
       </c>
       <c r="G42" t="n">
-        <v>35.3747</v>
+        <v>35.1022</v>
       </c>
       <c r="H42" t="n">
-        <v>2.95</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>avg_g_window_hg</t>
+          <t>band_g_mix_keep_s1</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1621,53 +1623,51 @@
         <v>2</v>
       </c>
       <c r="D43" t="n">
-        <v>1.0301</v>
+        <v>1.0388</v>
       </c>
       <c r="E43" t="n">
-        <v>1.0294</v>
+        <v>1.0357</v>
       </c>
       <c r="F43" t="n">
-        <v>1.0308</v>
+        <v>1.0419</v>
       </c>
       <c r="G43" t="n">
-        <v>35.5482</v>
-      </c>
-      <c r="H43" t="n">
-        <v>2.55</v>
-      </c>
+        <v>35.2519</v>
+      </c>
+      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>band_g_mix_b1_y_s2</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>60</v>
       </c>
       <c r="C44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D44" t="n">
-        <v>1.0292</v>
+        <v>1.0352</v>
       </c>
       <c r="E44" t="n">
-        <v>1.0039</v>
+        <v>1.0338</v>
       </c>
       <c r="F44" t="n">
-        <v>1.066</v>
+        <v>1.0365</v>
       </c>
       <c r="G44" t="n">
-        <v>35.6013</v>
+        <v>35.3747</v>
       </c>
       <c r="H44" t="n">
-        <v>0.8</v>
+        <v>2.95</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>avg_g_window_stock</t>
+          <t>avg_g_window_hg</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1677,51 +1677,53 @@
         <v>2</v>
       </c>
       <c r="D45" t="n">
-        <v>1.029</v>
+        <v>1.0301</v>
       </c>
       <c r="E45" t="n">
-        <v>1.026</v>
+        <v>1.0294</v>
       </c>
       <c r="F45" t="n">
-        <v>1.0319</v>
+        <v>1.0308</v>
       </c>
       <c r="G45" t="n">
-        <v>35.5875</v>
-      </c>
-      <c r="H45" t="inlineStr"/>
+        <v>35.5482</v>
+      </c>
+      <c r="H45" t="n">
+        <v>2.55</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>band_g_mix_b1o1_s3</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>60</v>
       </c>
       <c r="C46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D46" t="n">
-        <v>1.0233</v>
+        <v>1.0292</v>
       </c>
       <c r="E46" t="n">
-        <v>1.0165</v>
+        <v>1.0039</v>
       </c>
       <c r="F46" t="n">
-        <v>1.0395</v>
+        <v>1.066</v>
       </c>
       <c r="G46" t="n">
-        <v>35.7888</v>
+        <v>35.6013</v>
       </c>
       <c r="H46" t="n">
-        <v>3.2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>baseline_hg</t>
+          <t>avg_g_window_stock</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1731,189 +1733,189 @@
         <v>2</v>
       </c>
       <c r="D47" t="n">
-        <v>1.0162</v>
+        <v>1.029</v>
       </c>
       <c r="E47" t="n">
-        <v>1.0147</v>
+        <v>1.026</v>
       </c>
       <c r="F47" t="n">
-        <v>1.0177</v>
+        <v>1.0319</v>
       </c>
       <c r="G47" t="n">
-        <v>36.0347</v>
-      </c>
-      <c r="H47" t="n">
-        <v>3</v>
-      </c>
+        <v>35.5875</v>
+      </c>
+      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>baseline FORCE_CMD=1.0</t>
+          <t>band_g_mix_b1o1_s3</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>60</v>
       </c>
       <c r="C48" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D48" t="n">
-        <v>1.0017</v>
+        <v>1.0233</v>
       </c>
       <c r="E48" t="n">
-        <v>1.0017</v>
+        <v>1.0165</v>
       </c>
       <c r="F48" t="n">
-        <v>1.0017</v>
+        <v>1.0395</v>
       </c>
       <c r="G48" t="n">
-        <v>36.5572</v>
+        <v>35.7888</v>
       </c>
       <c r="H48" t="n">
-        <v>3.5</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>baseline_stocknorpm</t>
+          <t>baseline_hg</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>60</v>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D49" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.0162</v>
       </c>
       <c r="E49" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.0147</v>
       </c>
       <c r="F49" t="n">
-        <v>0.9874000000000001</v>
+        <v>1.0177</v>
       </c>
       <c r="G49" t="n">
-        <v>37.0845</v>
+        <v>36.0347</v>
       </c>
       <c r="H49" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>baseline_stock</t>
+          <t>baseline FORCE_CMD=1.0</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>60</v>
       </c>
       <c r="C50" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>0.8937</v>
+        <v>1.0017</v>
       </c>
       <c r="E50" t="n">
-        <v>0.8933</v>
+        <v>1.0017</v>
       </c>
       <c r="F50" t="n">
-        <v>0.8942</v>
+        <v>1.0017</v>
       </c>
       <c r="G50" t="n">
-        <v>40.9724</v>
+        <v>36.5572</v>
       </c>
       <c r="H50" t="n">
-        <v>3.5667</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>curation_hg</t>
+          <t>baseline_stocknorpm</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>60</v>
       </c>
       <c r="C51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D51" t="n">
-        <v>0.8874</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="E51" t="n">
-        <v>0.8813</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="F51" t="n">
-        <v>0.8935</v>
+        <v>0.9874000000000001</v>
       </c>
       <c r="G51" t="n">
-        <v>41.266</v>
-      </c>
-      <c r="H51" t="inlineStr"/>
+        <v>37.0845</v>
+      </c>
+      <c r="H51" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs2</t>
+          <t>baseline_stock</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>60</v>
       </c>
       <c r="C52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D52" t="n">
-        <v>0.8228</v>
+        <v>0.8937</v>
       </c>
       <c r="E52" t="n">
-        <v>0.8045</v>
+        <v>0.8933</v>
       </c>
       <c r="F52" t="n">
-        <v>0.8411</v>
+        <v>0.8942</v>
       </c>
       <c r="G52" t="n">
-        <v>44.527</v>
+        <v>40.9724</v>
       </c>
       <c r="H52" t="n">
-        <v>1.9</v>
+        <v>3.5667</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>baseline_stock16</t>
+          <t>curation_hg</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>60</v>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D53" t="n">
-        <v>0.7467</v>
+        <v>0.8874</v>
       </c>
       <c r="E53" t="n">
-        <v>0.7467</v>
+        <v>0.8813</v>
       </c>
       <c r="F53" t="n">
-        <v>0.7467</v>
+        <v>0.8935</v>
       </c>
       <c r="G53" t="n">
-        <v>49.0416</v>
+        <v>41.266</v>
       </c>
       <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>band_g_mix_b20o1</t>
+          <t>baseline_dynstocknoabs2</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1923,53 +1925,51 @@
         <v>2</v>
       </c>
       <c r="D54" t="n">
-        <v>0.7231</v>
+        <v>0.8228</v>
       </c>
       <c r="E54" t="n">
-        <v>0.4061</v>
+        <v>0.8045</v>
       </c>
       <c r="F54" t="n">
-        <v>1.0401</v>
+        <v>0.8411</v>
       </c>
       <c r="G54" t="n">
-        <v>62.6864</v>
+        <v>44.527</v>
       </c>
       <c r="H54" t="n">
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>baseline_stock16</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>60</v>
       </c>
       <c r="C55" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>0.4106</v>
+        <v>0.7467</v>
       </c>
       <c r="E55" t="n">
-        <v>0.2278</v>
+        <v>0.7467</v>
       </c>
       <c r="F55" t="n">
-        <v>0.7759</v>
+        <v>0.7467</v>
       </c>
       <c r="G55" t="n">
-        <v>122.7889</v>
-      </c>
-      <c r="H55" t="n">
-        <v>2.1</v>
-      </c>
+        <v>49.0416</v>
+      </c>
+      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>baseline_dynnoimu</t>
+          <t>band_g_mix_b20o1</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1979,53 +1979,53 @@
         <v>2</v>
       </c>
       <c r="D56" t="n">
-        <v>0.3672</v>
+        <v>0.7231</v>
       </c>
       <c r="E56" t="n">
-        <v>0.3661</v>
+        <v>0.4061</v>
       </c>
       <c r="F56" t="n">
-        <v>0.3683</v>
+        <v>1.0401</v>
       </c>
       <c r="G56" t="n">
-        <v>99.72539999999999</v>
+        <v>62.6864</v>
       </c>
       <c r="H56" t="n">
-        <v>4.6</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>baseline_dynstock2</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>60</v>
       </c>
       <c r="C57" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>0.2488</v>
+        <v>0.4106</v>
       </c>
       <c r="E57" t="n">
-        <v>0.2481</v>
+        <v>0.2278</v>
       </c>
       <c r="F57" t="n">
-        <v>0.2496</v>
+        <v>0.7759</v>
       </c>
       <c r="G57" t="n">
-        <v>147.1485</v>
+        <v>122.7889</v>
       </c>
       <c r="H57" t="n">
-        <v>2.8</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>baseline_dynnoimu</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -2035,51 +2035,53 @@
         <v>2</v>
       </c>
       <c r="D58" t="n">
-        <v>0.2302</v>
+        <v>0.3672</v>
       </c>
       <c r="E58" t="n">
-        <v>0.2295</v>
+        <v>0.3661</v>
       </c>
       <c r="F58" t="n">
-        <v>0.2309</v>
+        <v>0.3683</v>
       </c>
       <c r="G58" t="n">
-        <v>159.0684</v>
-      </c>
-      <c r="H58" t="inlineStr"/>
+        <v>99.72539999999999</v>
+      </c>
+      <c r="H58" t="n">
+        <v>4.6</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>avg_g_window</t>
+          <t>baseline_dynstock2</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>60</v>
       </c>
       <c r="C59" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D59" t="n">
-        <v>0.2283</v>
+        <v>0.2488</v>
       </c>
       <c r="E59" t="n">
-        <v>0.2276</v>
+        <v>0.2481</v>
       </c>
       <c r="F59" t="n">
-        <v>0.2291</v>
+        <v>0.2496</v>
       </c>
       <c r="G59" t="n">
-        <v>160.3908</v>
+        <v>147.1485</v>
       </c>
       <c r="H59" t="n">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>peak_g</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -2089,49 +2091,51 @@
         <v>2</v>
       </c>
       <c r="D60" t="n">
-        <v>0.2258</v>
+        <v>0.2302</v>
       </c>
       <c r="E60" t="n">
-        <v>0.2252</v>
+        <v>0.2295</v>
       </c>
       <c r="F60" t="n">
-        <v>0.2263</v>
+        <v>0.2309</v>
       </c>
       <c r="G60" t="n">
-        <v>162.2099</v>
+        <v>159.0684</v>
       </c>
       <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>peak_g_norpm</t>
+          <t>avg_g_window</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>60</v>
       </c>
       <c r="C61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D61" t="n">
-        <v>0.2245</v>
+        <v>0.2283</v>
       </c>
       <c r="E61" t="n">
-        <v>0.2238</v>
+        <v>0.2276</v>
       </c>
       <c r="F61" t="n">
-        <v>0.2252</v>
+        <v>0.2291</v>
       </c>
       <c r="G61" t="n">
-        <v>163.1152</v>
-      </c>
-      <c r="H61" t="inlineStr"/>
+        <v>160.3908</v>
+      </c>
+      <c r="H61" t="n">
+        <v>3.2</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>baseline_dynstock</t>
+          <t>yaw_intent</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -2141,25 +2145,23 @@
         <v>2</v>
       </c>
       <c r="D62" t="n">
-        <v>0.2241</v>
+        <v>0.2258</v>
       </c>
       <c r="E62" t="n">
-        <v>0.2235</v>
+        <v>0.2252</v>
       </c>
       <c r="F62" t="n">
-        <v>0.2247</v>
+        <v>0.2263</v>
       </c>
       <c r="G62" t="n">
-        <v>163.3969</v>
-      </c>
-      <c r="H62" t="n">
-        <v>3.05</v>
-      </c>
+        <v>162.2099</v>
+      </c>
+      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs</t>
+          <t>peak_g_norpm</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -2169,79 +2171,79 @@
         <v>2</v>
       </c>
       <c r="D63" t="n">
-        <v>0.1982</v>
+        <v>0.2245</v>
       </c>
       <c r="E63" t="n">
-        <v>0.198</v>
+        <v>0.2238</v>
       </c>
       <c r="F63" t="n">
-        <v>0.1985</v>
+        <v>0.2252</v>
       </c>
       <c r="G63" t="n">
-        <v>184.7105</v>
-      </c>
-      <c r="H63" t="n">
-        <v>3.75</v>
-      </c>
+        <v>163.1152</v>
+      </c>
+      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>avg_g_window_hg</t>
+          <t>baseline_dynstock</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D64" t="n">
-        <v>1.0148</v>
+        <v>0.2241</v>
       </c>
       <c r="E64" t="n">
-        <v>1.0148</v>
+        <v>0.2235</v>
       </c>
       <c r="F64" t="n">
-        <v>1.0148</v>
+        <v>0.2247</v>
       </c>
       <c r="G64" t="n">
-        <v>64.18680000000001</v>
+        <v>163.3969</v>
       </c>
       <c r="H64" t="n">
-        <v>3.8</v>
+        <v>3.05</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>baseline_dynstocknoabs</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C65" t="n">
         <v>2</v>
       </c>
       <c r="D65" t="n">
-        <v>1.011</v>
+        <v>0.1982</v>
       </c>
       <c r="E65" t="n">
-        <v>1.0062</v>
+        <v>0.198</v>
       </c>
       <c r="F65" t="n">
-        <v>1.0158</v>
+        <v>0.1985</v>
       </c>
       <c r="G65" t="n">
-        <v>50.3918</v>
-      </c>
-      <c r="H65" t="inlineStr"/>
+        <v>184.7105</v>
+      </c>
+      <c r="H65" t="n">
+        <v>3.75</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>avg_g_window_hg</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -2251,101 +2253,103 @@
         <v>1</v>
       </c>
       <c r="D66" t="n">
-        <v>0.9869</v>
+        <v>1.0148</v>
       </c>
       <c r="E66" t="n">
-        <v>0.9869</v>
+        <v>1.0148</v>
       </c>
       <c r="F66" t="n">
-        <v>0.9869</v>
+        <v>1.0148</v>
       </c>
       <c r="G66" t="n">
-        <v>66.0052</v>
-      </c>
-      <c r="H66" t="inlineStr"/>
+        <v>64.18680000000001</v>
+      </c>
+      <c r="H66" t="n">
+        <v>3.8</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>combined</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>80</v>
       </c>
       <c r="C67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D67" t="n">
-        <v>0.2276</v>
+        <v>1.011</v>
       </c>
       <c r="E67" t="n">
-        <v>0.2276</v>
+        <v>1.0062</v>
       </c>
       <c r="F67" t="n">
-        <v>0.2276</v>
+        <v>1.0158</v>
       </c>
       <c r="G67" t="n">
-        <v>160.9226</v>
+        <v>50.3918</v>
       </c>
       <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>80</v>
       </c>
       <c r="C68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D68" t="n">
-        <v>0.2159</v>
+        <v>0.9869</v>
       </c>
       <c r="E68" t="n">
-        <v>0.2156</v>
+        <v>0.9869</v>
       </c>
       <c r="F68" t="n">
-        <v>0.2162</v>
+        <v>0.9869</v>
       </c>
       <c r="G68" t="n">
-        <v>301.7328</v>
+        <v>66.0052</v>
       </c>
       <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>combined</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>80</v>
       </c>
       <c r="C69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D69" t="n">
-        <v>0.1782</v>
+        <v>0.2276</v>
       </c>
       <c r="E69" t="n">
-        <v>0.1779</v>
+        <v>0.2276</v>
       </c>
       <c r="F69" t="n">
-        <v>0.1784</v>
+        <v>0.2276</v>
       </c>
       <c r="G69" t="n">
-        <v>365.637</v>
+        <v>160.9226</v>
       </c>
       <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>avg_g_window</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -2355,23 +2359,23 @@
         <v>2</v>
       </c>
       <c r="D70" t="n">
-        <v>0.1778</v>
+        <v>0.2159</v>
       </c>
       <c r="E70" t="n">
-        <v>0.1776</v>
+        <v>0.2156</v>
       </c>
       <c r="F70" t="n">
-        <v>0.178</v>
+        <v>0.2162</v>
       </c>
       <c r="G70" t="n">
-        <v>366.3356</v>
+        <v>301.7328</v>
       </c>
       <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>peak_g</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -2381,18 +2385,70 @@
         <v>2</v>
       </c>
       <c r="D71" t="n">
+        <v>0.1782</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0.1779</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0.1784</v>
+      </c>
+      <c r="G71" t="n">
+        <v>365.637</v>
+      </c>
+      <c r="H71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>avg_g_window</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>80</v>
+      </c>
+      <c r="C72" t="n">
+        <v>2</v>
+      </c>
+      <c r="D72" t="n">
+        <v>0.1778</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0.1776</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="G72" t="n">
+        <v>366.3356</v>
+      </c>
+      <c r="H72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>yaw_intent</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>80</v>
+      </c>
+      <c r="C73" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" t="n">
         <v>0.1766</v>
       </c>
-      <c r="E71" t="n">
+      <c r="E73" t="n">
         <v>0.1766</v>
       </c>
-      <c r="F71" t="n">
+      <c r="F73" t="n">
         <v>0.1766</v>
       </c>
-      <c r="G71" t="n">
+      <c r="G73" t="n">
         <v>368.9042</v>
       </c>
-      <c r="H71" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2405,7 +2461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J159"/>
+  <dimension ref="A1:J162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7937,235 +7993,241 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>restructure</t>
+          <t>epg3</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
+          <t>baseline_all_epg3_s0</t>
         </is>
       </c>
       <c r="D149" t="n">
         <v>60</v>
       </c>
       <c r="E149" t="n">
-        <v>1.1085</v>
+        <v>1.1522</v>
       </c>
       <c r="F149" t="n">
-        <v>33.0351</v>
+        <v>31.7822</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>1788399311-0002</t>
+          <t>1788496288-0001</t>
         </is>
       </c>
       <c r="H149" t="n">
-        <v>33.04</v>
+        <v>31.78</v>
       </c>
       <c r="I149" t="n">
-        <v>4.8</v>
+        <v>2.1</v>
       </c>
       <c r="J149" t="n">
-        <v>2.4</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>lockweight</t>
+          <t>epg3</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>baseline_dyn_lock</t>
+          <t>baseline_all_epg3_s0</t>
         </is>
       </c>
       <c r="D150" t="n">
         <v>60</v>
       </c>
       <c r="E150" t="n">
-        <v>1.0756</v>
+        <v>1.0915</v>
       </c>
       <c r="F150" t="n">
-        <v>34.0434</v>
+        <v>33.5493</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>1788409205-0003</t>
+          <t>1788496321-0002</t>
         </is>
       </c>
       <c r="H150" t="n">
-        <v>34.04</v>
+        <v>33.55</v>
       </c>
       <c r="I150" t="n">
-        <v>4.5</v>
+        <v>3.7</v>
       </c>
       <c r="J150" t="n">
-        <v>2.45</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>lockweight</t>
+          <t>epg3</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>baseline_dyn_lock</t>
+          <t>baseline_all_epg3_s1</t>
         </is>
       </c>
       <c r="D151" t="n">
         <v>60</v>
       </c>
       <c r="E151" t="n">
-        <v>1.0817</v>
+        <v>1.0741</v>
       </c>
       <c r="F151" t="n">
-        <v>33.8519</v>
+        <v>34.0906</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>1788409238-0004</t>
+          <t>1788496358-0003</t>
         </is>
       </c>
       <c r="H151" t="n">
-        <v>33.85</v>
+        <v>34.09</v>
       </c>
       <c r="I151" t="n">
-        <v>4.3</v>
+        <v>3.4</v>
       </c>
       <c r="J151" t="n">
-        <v>2.43</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>epg</t>
+          <t>restructure</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>baseline_mix_epg_s0</t>
+          <t>baseline_dyn</t>
         </is>
       </c>
       <c r="D152" t="n">
         <v>60</v>
       </c>
       <c r="E152" t="n">
-        <v>1.1411</v>
+        <v>1.1085</v>
       </c>
       <c r="F152" t="n">
-        <v>32.0898</v>
+        <v>33.0351</v>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>1788494508-0001</t>
-        </is>
-      </c>
-      <c r="H152" t="inlineStr"/>
-      <c r="I152" t="inlineStr"/>
-      <c r="J152" t="inlineStr"/>
+          <t>1788399311-0002</t>
+        </is>
+      </c>
+      <c r="H152" t="n">
+        <v>33.04</v>
+      </c>
+      <c r="I152" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="J152" t="n">
+        <v>2.4</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>epg</t>
+          <t>lockweight</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>baseline_mix_epg_s0</t>
+          <t>baseline_dyn_lock</t>
         </is>
       </c>
       <c r="D153" t="n">
         <v>60</v>
       </c>
       <c r="E153" t="n">
-        <v>1.1429</v>
+        <v>1.0756</v>
       </c>
       <c r="F153" t="n">
-        <v>32.0399</v>
+        <v>34.0434</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>1788494541-0002</t>
+          <t>1788409205-0003</t>
         </is>
       </c>
       <c r="H153" t="n">
-        <v>32.04</v>
+        <v>34.04</v>
       </c>
       <c r="I153" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="J153" t="n">
-        <v>2.33</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>epg</t>
+          <t>lockweight</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>baseline_mix_epg_s1</t>
+          <t>baseline_dyn_lock</t>
         </is>
       </c>
       <c r="D154" t="n">
         <v>60</v>
       </c>
       <c r="E154" t="n">
-        <v>1.0512</v>
+        <v>1.0817</v>
       </c>
       <c r="F154" t="n">
-        <v>34.8362</v>
+        <v>33.8519</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>1788494578-0003</t>
+          <t>1788409238-0004</t>
         </is>
       </c>
       <c r="H154" t="n">
-        <v>34.84</v>
+        <v>33.85</v>
       </c>
       <c r="I154" t="n">
-        <v>2.8</v>
+        <v>4.3</v>
       </c>
       <c r="J154" t="n">
-        <v>2.48</v>
+        <v>2.43</v>
       </c>
     </row>
     <row r="155">
@@ -8181,32 +8243,26 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>baseline_mix_epg_s1</t>
+          <t>baseline_mix_epg_s0</t>
         </is>
       </c>
       <c r="D155" t="n">
         <v>60</v>
       </c>
       <c r="E155" t="n">
-        <v>1.0525</v>
+        <v>1.1411</v>
       </c>
       <c r="F155" t="n">
-        <v>34.7916</v>
+        <v>32.0898</v>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>1788494611-0004</t>
-        </is>
-      </c>
-      <c r="H155" t="n">
-        <v>34.79</v>
-      </c>
-      <c r="I155" t="n">
-        <v>3</v>
-      </c>
-      <c r="J155" t="n">
-        <v>2.46</v>
-      </c>
+          <t>1788494508-0001</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -8221,31 +8277,31 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>baseline_mix_epg_s2</t>
+          <t>baseline_mix_epg_s0</t>
         </is>
       </c>
       <c r="D156" t="n">
         <v>60</v>
       </c>
       <c r="E156" t="n">
-        <v>1.1439</v>
+        <v>1.1429</v>
       </c>
       <c r="F156" t="n">
-        <v>32.0107</v>
+        <v>32.0399</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>1788494647-0005</t>
+          <t>1788494541-0002</t>
         </is>
       </c>
       <c r="H156" t="n">
-        <v>32.01</v>
+        <v>32.04</v>
       </c>
       <c r="I156" t="n">
-        <v>1.9</v>
+        <v>1</v>
       </c>
       <c r="J156" t="n">
-        <v>2.34</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="157">
@@ -8261,110 +8317,230 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>baseline_mix_epg_s2</t>
+          <t>baseline_mix_epg_s1</t>
         </is>
       </c>
       <c r="D157" t="n">
         <v>60</v>
       </c>
       <c r="E157" t="n">
-        <v>1.1472</v>
+        <v>1.0512</v>
       </c>
       <c r="F157" t="n">
-        <v>31.9194</v>
+        <v>34.8362</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>1788494680-0006</t>
+          <t>1788494578-0003</t>
         </is>
       </c>
       <c r="H157" t="n">
-        <v>31.92</v>
+        <v>34.84</v>
       </c>
       <c r="I157" t="n">
-        <v>1.2</v>
+        <v>2.8</v>
       </c>
       <c r="J157" t="n">
-        <v>2.33</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>ensemble</t>
+          <t>epg</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>ens_band_g_mix5</t>
+          <t>baseline_mix_epg_s1</t>
         </is>
       </c>
       <c r="D158" t="n">
         <v>60</v>
       </c>
       <c r="E158" t="n">
-        <v>1.0736</v>
+        <v>1.0525</v>
       </c>
       <c r="F158" t="n">
-        <v>34.1079</v>
+        <v>34.7916</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>1788400929-0001</t>
+          <t>1788494611-0004</t>
         </is>
       </c>
       <c r="H158" t="n">
-        <v>34.11</v>
+        <v>34.79</v>
       </c>
       <c r="I158" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="J158" t="n">
-        <v>2.44</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>epg</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>baseline_mix_epg_s2</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>60</v>
+      </c>
+      <c r="E159" t="n">
+        <v>1.1439</v>
+      </c>
+      <c r="F159" t="n">
+        <v>32.0107</v>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>1788494647-0005</t>
+        </is>
+      </c>
+      <c r="H159" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="I159" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J159" t="n">
+        <v>2.34</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>epg</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>baseline_mix_epg_s2</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>60</v>
+      </c>
+      <c r="E160" t="n">
+        <v>1.1472</v>
+      </c>
+      <c r="F160" t="n">
+        <v>31.9194</v>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>1788494680-0006</t>
+        </is>
+      </c>
+      <c r="H160" t="n">
+        <v>31.92</v>
+      </c>
+      <c r="I160" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J160" t="n">
+        <v>2.33</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr">
+      <c r="B161" t="inlineStr">
         <is>
           <t>ensemble</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr">
+      <c r="C161" t="inlineStr">
         <is>
           <t>ens_band_g_mix5</t>
         </is>
       </c>
-      <c r="D159" t="n">
-        <v>60</v>
-      </c>
-      <c r="E159" t="n">
+      <c r="D161" t="n">
+        <v>60</v>
+      </c>
+      <c r="E161" t="n">
+        <v>1.0736</v>
+      </c>
+      <c r="F161" t="n">
+        <v>34.1079</v>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>1788400929-0001</t>
+        </is>
+      </c>
+      <c r="H161" t="n">
+        <v>34.11</v>
+      </c>
+      <c r="I161" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J161" t="n">
+        <v>2.44</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>ensemble</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>ens_band_g_mix5</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>60</v>
+      </c>
+      <c r="E162" t="n">
         <v>1.0538</v>
       </c>
-      <c r="F159" t="n">
+      <c r="F162" t="n">
         <v>34.7482</v>
       </c>
-      <c r="G159" t="inlineStr">
+      <c r="G162" t="inlineStr">
         <is>
           <t>1788400962-0002</t>
         </is>
       </c>
-      <c r="H159" t="n">
+      <c r="H162" t="n">
         <v>34.75</v>
       </c>
-      <c r="I159" t="n">
+      <c r="I162" t="n">
         <v>2</v>
       </c>
-      <c r="J159" t="n">
+      <c r="J162" t="n">
         <v>2.48</v>
       </c>
     </row>
@@ -8379,7 +8555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:N67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -10513,31 +10689,63 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
+          <t>baseline_all_epg3_s0</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2026-09-03T21:28:27</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>5</v>
+      </c>
+      <c r="K43" t="n">
+        <v>1</v>
+      </c>
+      <c r="L43" t="n">
+        <v>2386</v>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>[0.14934, 0.15368, 0.16516, 0.16712]</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>baseline_dyn_lock</t>
+          <t>baseline_all_epg3_s1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -10547,12 +10755,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-09-02T21:17:44</t>
+          <t>2026-09-03T21:30:07</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>dyn_abs</t>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
@@ -10562,7 +10770,7 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -10581,11 +10789,11 @@
         <v>1</v>
       </c>
       <c r="L44" t="n">
-        <v>1129</v>
+        <v>2386</v>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>[0.13261, 0.15194, 0.08818, 0.08624]</t>
+          <t>[0.14639, 0.15277, 0.16447, 0.16807]</t>
         </is>
       </c>
       <c r="N44" t="inlineStr"/>
@@ -10593,7 +10801,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>baseline_dynnoimu</t>
+          <t>baseline_dyn</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
@@ -10617,31 +10825,63 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>baseline_dynstock2</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
+          <t>baseline_dyn_lock</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2026-09-02T21:17:44</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>dyn_abs</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>5</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1</v>
+      </c>
+      <c r="L46" t="n">
+        <v>1129</v>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>[0.13261, 0.15194, 0.08818, 0.08624]</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>baseline_dynstock</t>
+          <t>baseline_dynnoimu</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -10665,7 +10905,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs2</t>
+          <t>baseline_dynstock2</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -10689,7 +10929,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs</t>
+          <t>baseline_dynstock</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -10713,7 +10953,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>baseline_hg</t>
+          <t>baseline_dynstocknoabs2</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -10737,119 +10977,55 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>baseline_mix_epg_s0</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>baseline</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>2026-09-03T20:55:00</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
-        </is>
-      </c>
+          <t>baseline_dynstocknoabs</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>etk800</t>
-        </is>
-      </c>
-      <c r="G51" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>sensor_z,roll_angle,pitch_angle,gear</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>gy2</t>
-        </is>
-      </c>
-      <c r="J51" t="n">
-        <v>5</v>
-      </c>
-      <c r="K51" t="n">
-        <v>1</v>
-      </c>
-      <c r="L51" t="n">
-        <v>2289</v>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>[0.14917, 0.15195, 0.17024, 0.17111]</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>baseline_mix_epg_s1</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>baseline</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>2026-09-03T20:56:49</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
-        </is>
-      </c>
+          <t>baseline_hg</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>etk800</t>
-        </is>
-      </c>
-      <c r="G52" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>sensor_z,roll_angle,pitch_angle,gear</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>gy2</t>
-        </is>
-      </c>
-      <c r="J52" t="n">
-        <v>5</v>
-      </c>
-      <c r="K52" t="n">
-        <v>1</v>
-      </c>
-      <c r="L52" t="n">
-        <v>2289</v>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>[0.15347, 0.15532, 0.17054, 0.1711]</t>
-        </is>
-      </c>
-      <c r="N52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>baseline_mix_epg_s2</t>
+          <t>baseline_mix_epg_s0</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -10859,7 +11035,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-09-03T20:58:34</t>
+          <t>2026-09-03T20:55:00</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -10897,7 +11073,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>[0.1528, 0.15348, 0.16971, 0.17046]</t>
+          <t>[0.14917, 0.15195, 0.17024, 0.17111]</t>
         </is>
       </c>
       <c r="N53" t="inlineStr"/>
@@ -10905,55 +11081,119 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>baseline_norpm</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
+          <t>baseline_mix_epg_s1</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2026-09-03T20:56:49</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J54" t="n">
+        <v>5</v>
+      </c>
+      <c r="K54" t="n">
+        <v>1</v>
+      </c>
+      <c r="L54" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>[0.15347, 0.15532, 0.17054, 0.1711]</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>baseline_stock16</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
+          <t>baseline_mix_epg_s2</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2026-09-03T20:58:34</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>5</v>
+      </c>
+      <c r="K55" t="n">
+        <v>1</v>
+      </c>
+      <c r="L55" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>[0.1528, 0.15348, 0.16971, 0.17046]</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>baseline_norpm</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
@@ -10977,7 +11217,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>baseline_stock</t>
+          <t>baseline_stock16</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
@@ -11001,7 +11241,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>baseline_stocknorpm</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
@@ -11025,7 +11265,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>combined</t>
+          <t>baseline_stock</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
@@ -11049,7 +11289,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>baseline_stocknorpm</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
@@ -11073,7 +11313,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>curation_hg</t>
+          <t>combined</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
@@ -11097,7 +11337,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ens_band_g_mix5</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
@@ -11112,12 +11352,16 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>curation_hg</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
@@ -11141,7 +11385,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>peak_g_norpm</t>
+          <t>ens_band_g_mix5</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
@@ -11156,16 +11400,12 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="N64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>peak_g</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
@@ -11186,6 +11426,54 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>peak_g_norpm</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>yaw_intent</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Reporting: exclude non-OK runs (a DAMAGED collision was being counted as a 1.53g stop)
</commit_message>
<xml_diff>
--- a/results/LSTM_ABS_RESULTS.xlsx
+++ b/results/LSTM_ABS_RESULTS.xlsx
@@ -8555,13 +8555,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N67"/>
+  <dimension ref="A1:N69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -10801,31 +10801,63 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>baseline_dyn</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
+          <t>baseline_ctrl_epg_s0</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2026-09-03T22:23:45</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>dyn_abs,dyn_ctrl,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>5</v>
+      </c>
+      <c r="K45" t="n">
+        <v>1</v>
+      </c>
+      <c r="L45" t="n">
+        <v>2409</v>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>[0.14959, 0.15359, 0.17507, 0.17397]</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>baseline_dyn_lock</t>
+          <t>baseline_ctrl_epg_s2</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -10835,12 +10867,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-09-02T21:17:44</t>
+          <t>2026-09-03T22:25:55</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>dyn_abs</t>
+          <t>dyn_abs,dyn_ctrl,stock_tel,no_abs,no_safety</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -10869,11 +10901,11 @@
         <v>1</v>
       </c>
       <c r="L46" t="n">
-        <v>1129</v>
+        <v>2409</v>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>[0.13261, 0.15194, 0.08818, 0.08624]</t>
+          <t>[0.14948, 0.152, 0.17421, 0.1732]</t>
         </is>
       </c>
       <c r="N46" t="inlineStr"/>
@@ -10881,7 +10913,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>baseline_dynnoimu</t>
+          <t>baseline_dyn</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -10905,31 +10937,63 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>baseline_dynstock2</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
+          <t>baseline_dyn_lock</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2026-09-02T21:17:44</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>dyn_abs</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>5</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1</v>
+      </c>
+      <c r="L48" t="n">
+        <v>1129</v>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>[0.13261, 0.15194, 0.08818, 0.08624]</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>baseline_dynstock</t>
+          <t>baseline_dynnoimu</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -10953,7 +11017,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs2</t>
+          <t>baseline_dynstock2</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -10977,7 +11041,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>baseline_dynstocknoabs</t>
+          <t>baseline_dynstock</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
@@ -11001,7 +11065,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>baseline_hg</t>
+          <t>baseline_dynstocknoabs2</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -11025,119 +11089,55 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>baseline_mix_epg_s0</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>baseline</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>2026-09-03T20:55:00</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
-        </is>
-      </c>
+          <t>baseline_dynstocknoabs</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>etk800</t>
-        </is>
-      </c>
-      <c r="G53" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>sensor_z,roll_angle,pitch_angle,gear</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>gy2</t>
-        </is>
-      </c>
-      <c r="J53" t="n">
-        <v>5</v>
-      </c>
-      <c r="K53" t="n">
-        <v>1</v>
-      </c>
-      <c r="L53" t="n">
-        <v>2289</v>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>[0.14917, 0.15195, 0.17024, 0.17111]</t>
-        </is>
-      </c>
-      <c r="N53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>baseline_mix_epg_s1</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>baseline</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>2026-09-03T20:56:49</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
-        </is>
-      </c>
+          <t>baseline_hg</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>etk800</t>
-        </is>
-      </c>
-      <c r="G54" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>sensor_z,roll_angle,pitch_angle,gear</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>gy2</t>
-        </is>
-      </c>
-      <c r="J54" t="n">
-        <v>5</v>
-      </c>
-      <c r="K54" t="n">
-        <v>1</v>
-      </c>
-      <c r="L54" t="n">
-        <v>2289</v>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>[0.15347, 0.15532, 0.17054, 0.1711]</t>
-        </is>
-      </c>
-      <c r="N54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>baseline_mix_epg_s2</t>
+          <t>baseline_mix_epg_s0</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -11147,7 +11147,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-09-03T20:58:34</t>
+          <t>2026-09-03T20:55:00</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -11185,7 +11185,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>[0.1528, 0.15348, 0.16971, 0.17046]</t>
+          <t>[0.14917, 0.15195, 0.17024, 0.17111]</t>
         </is>
       </c>
       <c r="N55" t="inlineStr"/>
@@ -11193,55 +11193,119 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>baseline_norpm</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
+          <t>baseline_mix_epg_s1</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2026-09-03T20:56:49</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>5</v>
+      </c>
+      <c r="K56" t="n">
+        <v>1</v>
+      </c>
+      <c r="L56" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>[0.15347, 0.15532, 0.17054, 0.1711]</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>baseline_stock16</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
+          <t>baseline_mix_epg_s2</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2026-09-03T20:58:34</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>dyn_abs,stock_tel,no_abs,no_safety</t>
+        </is>
+      </c>
       <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>etk800</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>sensor_z,roll_angle,pitch_angle,gear</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>gy2</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>5</v>
+      </c>
+      <c r="K57" t="n">
+        <v>1</v>
+      </c>
+      <c r="L57" t="n">
+        <v>2289</v>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>[0.1528, 0.15348, 0.16971, 0.17046]</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>baseline_stock800</t>
+          <t>baseline_norpm</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
@@ -11265,7 +11329,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>baseline_stock</t>
+          <t>baseline_stock16</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
@@ -11289,7 +11353,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>baseline_stocknorpm</t>
+          <t>baseline_stock800</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
@@ -11313,7 +11377,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>combined</t>
+          <t>baseline_stock</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
@@ -11337,7 +11401,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>curation</t>
+          <t>baseline_stocknorpm</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
@@ -11361,7 +11425,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>curation_hg</t>
+          <t>combined</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
@@ -11385,7 +11449,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ens_band_g_mix5</t>
+          <t>curation</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
@@ -11400,12 +11464,16 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>peak_g</t>
+          <t>curation_hg</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
@@ -11429,7 +11497,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>peak_g_norpm</t>
+          <t>ens_band_g_mix5</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
@@ -11444,16 +11512,12 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr">
-        <is>
-          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
-        </is>
-      </c>
+      <c r="N66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>yaw_intent</t>
+          <t>peak_g</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
@@ -11474,6 +11538,54 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>peak_g_norpm</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>yaw_intent</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>training args not recorded for migrated runs; see results/raw_2026-09-02 logs and docs/INVESTIGATION.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>